<commit_message>
Add ranking data for 2026-07-27
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -64,6 +64,7 @@
     <sheet name="2026-07-06" sheetId="56" state="visible" r:id="rId56"/>
     <sheet name="2026-07-13" sheetId="57" state="visible" r:id="rId57"/>
     <sheet name="2026-07-20" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet name="2026-07-27" sheetId="59" state="visible" r:id="rId59"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -54416,22 +54417,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>異種族レビュアーズ</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>天原(原作) masha(作画)</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第94話</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第81話 前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第40話：親友だから②</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第156話	触覚フィードバックを主因とした外部非依存型報酬回路活性化メカニズムの予備的考察</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第７９話『呉越停止』②</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第８３話　ラッキースケベの戦いが始まった（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第12話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第88話その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>帰ってください！ 阿久津さん</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>長岡太一(著者)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第209話</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第138話　ひさびさに本気出してみるⅢ（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第11話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第17話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>まんきつしたい常連さん</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>しんみりん(著者)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第57話後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第24話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第40話</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第149話　復活！</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第83話➁</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>ぽんドロイド！ はまさん</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>はれやまはれぞう(著者)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第23話</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>アザミヤコを好きになる</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第17話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>コミックス2巻発売告知記事</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第６２話　単独調査する器用貧乏（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第40話 独身貴族は友人を実家に連れていく（3）</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>俺の担当は怪物</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>ぴざし(著者)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第3話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第３０食　シルバーホーンのステーキ、パクパクですわ！（その２）（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>転生貴族の異世界冒険録 ～自重を知らない神々の使徒～</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>夜州 nini 藻</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第76話（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第11話後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第53話 友の兄とお茶会を④</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>拷問192</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>寿司ガキ</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>ichika(著者)</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>【マンガ総選挙出馬中】清き一票をお願いします！</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>【マンガ総選挙出馬中】清き一票をお願いします！</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第16話-2：落ちていく少女</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第157話 よくわからないけれど清算してもらうみたいです（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第４９話　ガイアスと剣神、激戦を繰り広げる。勇者は、オカモトさんに不吉な占いをされてしまう（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>聖者無双</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第100話　将来の夢と目標②</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第11話-2：仲良くしましょう！</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>小林さんちのメイドラゴン</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>クール教信者</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第170話</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>幼女戦記</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第百十八章-2：邂逅Ⅲ</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第65話　復讐からは、何も生まれない</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第99話</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第11話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>ギャルの自転車を直したら懐かれた</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>タケチケイ（漫画） 生姜寧也（原作）</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第3話　ギャルと約束した（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>魔法少女リリカルなのは EXCEEDS</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>都築真紀 川上修一</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第１４話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>俺は星間国家の悪徳領主！</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第49話　最高に無駄だろう!?</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第90話 竜牙、漆黒を駆ける!!</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>六志麻あさ 業務用餅 kisui</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第９０話</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>セレビィ量産型(著者)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第28.5話</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第24話④</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>EP.28①</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第8話(1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>ライブダンジョン！</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第98話前半</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>異種族レビュアーズ</t>
+          <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>天原(原作) masha(作画)</t>
+          <t>丈(著者)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第94話</t>
+          <t>第139話</t>
         </is>
       </c>
     </row>
@@ -54441,17 +55478,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+          <t>異世界おじさん</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+          <t>殆ど死んでいる(著者)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第81話 前編</t>
+          <t>第79話</t>
         </is>
       </c>
     </row>
@@ -54461,17 +55498,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+          <t>ワンパンマン</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>zunta(作画) はらわたさいぞう(原作)</t>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第40話：親友だから②</t>
+          <t>232撃目</t>
         </is>
       </c>
     </row>
@@ -54481,17 +55518,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>むちまろ</t>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第156話	触覚フィードバックを主因とした外部非依存型報酬回路活性化メカニズムの予備的考察</t>
+          <t>第40話：親友だから③</t>
         </is>
       </c>
     </row>
@@ -54501,17 +55538,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第７９話『呉越停止』②</t>
+          <t>第25話-1「女神教の狙い」</t>
         </is>
       </c>
     </row>
@@ -54521,17 +55558,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第８３話　ラッキースケベの戦いが始まった（１）</t>
+          <t>第７９話『呉越停止』③</t>
         </is>
       </c>
     </row>
@@ -54541,17 +55578,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第12話後半</t>
+          <t>第８３話　ラッキースケベの戦いが始まった（２）</t>
         </is>
       </c>
     </row>
@@ -54561,17 +55598,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第88話その2</t>
+          <t>第8話後編：アトリ</t>
         </is>
       </c>
     </row>
@@ -54581,17 +55618,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>帰ってください！ 阿久津さん</t>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>長岡太一(著者)</t>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第209話</t>
+          <t>第43話①</t>
         </is>
       </c>
     </row>
@@ -54601,17 +55638,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第138話　ひさびさに本気出してみるⅢ（後編）</t>
+          <t>第11話 前編</t>
         </is>
       </c>
     </row>
@@ -54621,17 +55658,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>三部べべ(漫画) ねうしとら(原作)</t>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第11話-2</t>
+          <t>第21話-2</t>
         </is>
       </c>
     </row>
@@ -54641,17 +55678,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+          <t>いとこのこ</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+          <t>いぬちく(著者)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第17話-2</t>
+          <t>休載イラスト</t>
         </is>
       </c>
     </row>
@@ -54661,17 +55698,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>まんきつしたい常連さん</t>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>しんみりん(著者)</t>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第57話後編</t>
+          <t>第100話　禁じ手</t>
         </is>
       </c>
     </row>
@@ -54681,17 +55718,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>クセ強彼女は床にいざなう</t>
+          <t>美人女上司滝沢さん</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>須河篤志(著者)</t>
+          <t>やんBARU(著者)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第24話前半</t>
+          <t>コミックス告知</t>
         </is>
       </c>
     </row>
@@ -54701,17 +55738,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第40話</t>
+          <t>第150話　支配する者</t>
         </is>
       </c>
     </row>
@@ -54721,17 +55758,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第149話　復活！</t>
+          <t>第83話③</t>
         </is>
       </c>
     </row>
@@ -54741,17 +55778,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第83話➁</t>
+          <t>第40話 独身貴族は友人を実家に連れていく（4）</t>
         </is>
       </c>
     </row>
@@ -54761,17 +55798,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ぽんドロイド！ はまさん</t>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>はれやまはれぞう(著者)</t>
+          <t>モリタ Ｕ４ nima</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第23話</t>
+          <t>第17話（２）　クリスティーナお姉さまの結婚（２）</t>
         </is>
       </c>
     </row>
@@ -54781,17 +55818,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>アザミヤコを好きになる</t>
+          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第17話前編</t>
+          <t>第47話-2</t>
         </is>
       </c>
     </row>
@@ -54801,17 +55838,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+          <t>描けないのでヤってみた</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+          <t>逢上おかき(著者)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>コミックス2巻発売告知記事</t>
+          <t>第4話</t>
         </is>
       </c>
     </row>
@@ -54831,7 +55868,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第６２話　単独調査する器用貧乏（１）</t>
+          <t>第６２話　単独調査する器用貧乏（２）</t>
         </is>
       </c>
     </row>
@@ -54841,17 +55878,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第40話 独身貴族は友人を実家に連れていく（3）</t>
+          <t>第5話④</t>
         </is>
       </c>
     </row>
@@ -54861,17 +55898,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>俺の担当は怪物</t>
+          <t>「お相手は一般の方です」</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ぴざし(著者)</t>
+          <t>嵯峨祐介(著者)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第3話前半</t>
+          <t>第1話</t>
         </is>
       </c>
     </row>
@@ -54881,17 +55918,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+          <t>お前がヤったんだろ！</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>島知宏 音速炒飯 有都あらゆる</t>
+          <t>クシザキ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第３０食　シルバーホーンのステーキ、パクパクですわ！（その２）（３）</t>
+          <t>第15話	君に入らせたい部活があるんだ</t>
         </is>
       </c>
     </row>
@@ -54901,17 +55938,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>転生貴族の異世界冒険録 ～自重を知らない神々の使徒～</t>
+          <t>リアデイルの大地にて</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>夜州 nini 藻</t>
+          <t>月見だしお(著者) Ceez(原作) てんまそ(キャラクター原案) 涼風涼(構成)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第76話（前編）</t>
+          <t>第43章</t>
         </is>
       </c>
     </row>
@@ -54921,17 +55958,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+          <t>板垣恵介 林たかあき</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第11話後編</t>
+          <t>第74話 止まらぬ思考</t>
         </is>
       </c>
     </row>
@@ -54941,17 +55978,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第53話 友の兄とお茶会を④</t>
+          <t>第49話　奴の罪（後編）</t>
         </is>
       </c>
     </row>
@@ -54961,17 +55998,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>ヨウハ(著者)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>拷問192</t>
+          <t>第3話-2</t>
         </is>
       </c>
     </row>
@@ -54981,17 +56018,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>寿司ガキ</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ichika(著者)</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>【マンガ総選挙出馬中】清き一票をお願いします！</t>
+          <t>第69話②　あにめを見てみた</t>
         </is>
       </c>
     </row>
@@ -55001,17 +56038,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>【マンガ総選挙出馬中】清き一票をお願いします！</t>
+          <t>第158話 よくわからないけれど新たな問題が発生したみたいです（１）</t>
         </is>
       </c>
     </row>
@@ -55021,17 +56058,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第16話-2：落ちていく少女</t>
+          <t>拷問193</t>
         </is>
       </c>
     </row>
@@ -55041,17 +56078,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第157話 よくわからないけれど清算してもらうみたいです（２）</t>
+          <t>コミックス発売告知</t>
         </is>
       </c>
     </row>
@@ -55071,7 +56108,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第４９話　ガイアスと剣神、激戦を繰り広げる。勇者は、オカモトさんに不吉な占いをされてしまう（２）</t>
+          <t>第４９話　ガイアスと剣神、激戦を繰り広げる。勇者は、オカモトさんに不吉な占いをされてしまう（３）</t>
         </is>
       </c>
     </row>
@@ -55081,17 +56118,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>聖者無双</t>
+          <t>追放僧侶の賢者タイム</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+          <t>原作・野原のはて 作画・鈴木シオン</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第100話　将来の夢と目標②</t>
+          <t>第8話　ワンオンワン</t>
         </is>
       </c>
     </row>
@@ -55101,17 +56138,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+          <t>はぐはぐ(著者)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第11話-2：仲良くしましょう！</t>
+          <t>第101話後編</t>
         </is>
       </c>
     </row>
@@ -55121,17 +56158,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>小林さんちのメイドラゴン</t>
+          <t>物語の黒幕に転生して</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>クール教信者</t>
+          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第170話</t>
+          <t>第42話</t>
         </is>
       </c>
     </row>
@@ -55141,17 +56178,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>幼女戦記</t>
+          <t>このヒーラー、めんどくさい</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
+          <t>丹念に発酵(著者)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第百十八章-2：邂逅Ⅲ</t>
+          <t>【コメント募集企画】もしもカーラが現代日本でバイトするならどんなお仕事!?【コミックス発売記念】</t>
         </is>
       </c>
     </row>
@@ -55161,17 +56198,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
+          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
+          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第65話　復讐からは、何も生まれない</t>
+          <t>第10話-２</t>
         </is>
       </c>
     </row>
@@ -55181,17 +56218,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>くらいあの子としたいこと</t>
+          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>碇マナツ(著者)</t>
+          <t>FUNA 東西 モトエ恵介</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第99話</t>
+          <t>第132話 第2回異世界懇談会［その③］</t>
         </is>
       </c>
     </row>
@@ -55201,17 +56238,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第11話-1</t>
+          <t>第3話-2</t>
         </is>
       </c>
     </row>
@@ -55221,17 +56258,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ギャルの自転車を直したら懐かれた</t>
+          <t>幼女戦記</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>タケチケイ（漫画） 生姜寧也（原作）</t>
+          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第3話　ギャルと約束した（前編）</t>
+          <t>第百十九章：邂逅Ⅳ</t>
         </is>
       </c>
     </row>
@@ -55241,17 +56278,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS</t>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>都築真紀 川上修一</t>
+          <t>KAKERU</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第１４話①</t>
+          <t>第78話「ケンタウロス」（後半）</t>
         </is>
       </c>
     </row>
@@ -55261,17 +56298,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>俺は星間国家の悪徳領主！</t>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
+          <t>空野進 sorani ファルまろ</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第49話　最高に無駄だろう!?</t>
+          <t>第22話　最弱貴族、伯爵を撃退する(４)</t>
         </is>
       </c>
     </row>
@@ -55281,17 +56318,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>北斗の拳 世紀末ドラマ撮影伝</t>
+          <t>雨森潤奈は湿度が高い</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
+          <t>水城水城(原作) 稲鳴四季(作画) 潮崎しの(キャラクター原案)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第90話 竜牙、漆黒を駆ける!!</t>
+          <t>第3話</t>
         </is>
       </c>
     </row>
@@ -55301,17 +56338,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は 気ままなセカンドライフを謳歌する。</t>
+          <t>塔の管理をしてみよう</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>六志麻あさ 業務用餅 kisui</t>
+          <t>盧恩＆雪笠(Friendly Land)(著者) 早秋(原作) 雨神(キャラクター原案)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第９０話</t>
+          <t>第103話前編</t>
         </is>
       </c>
     </row>
@@ -55321,17 +56358,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>三枝さんはメガネ先輩と恋を描く</t>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>セレビィ量産型(著者)</t>
+          <t>漫画/すたひろ 原作/Y.A</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第28.5話</t>
+          <t>chapter90【47話①】</t>
         </is>
       </c>
     </row>
@@ -55341,17 +56378,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+          <t>おせっかい女子、恋をする</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+          <t>音竹 ひかる(著者)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第24話④</t>
+          <t>第26話</t>
         </is>
       </c>
     </row>
@@ -55361,17 +56398,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+          <t>黄金の経験値</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+          <t>原純(原作) 霜月汐(作画) fixro2n(キャラクター原案)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>EP.28①</t>
+          <t>第27話</t>
         </is>
       </c>
     </row>
@@ -55381,17 +56418,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+          <t>解雇された暗黒兵士(30代)のスローなセカンドライフ</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+          <t>岡沢六十四 るれくちぇ sage・ジョー</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第8話(1)</t>
+          <t>第83話(前編) 修羅と地獄</t>
         </is>
       </c>
     </row>
@@ -55401,17 +56438,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ライブダンジョン！</t>
+          <t>魔王になったので、ダンジョン造って人外娘とほのぼのする</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+          <t>遠野ノオト(作画) 流優(原作) だぶ竜(キャラクター原案)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第98話前半</t>
+          <t>第91話後半</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-08-03
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -65,6 +65,7 @@
     <sheet name="2026-07-13" sheetId="57" state="visible" r:id="rId57"/>
     <sheet name="2026-07-20" sheetId="58" state="visible" r:id="rId58"/>
     <sheet name="2026-07-27" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet name="2026-08-03" sheetId="60" state="visible" r:id="rId60"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -55453,1000 +55454,1000 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="0" t="inlineStr">
         <is>
           <t>丈(著者)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>第139話</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>異世界おじさん</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>殆ど死んでいる(著者)</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
         <is>
           <t>第79話</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>ワンパンマン</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>232撃目</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
         <is>
           <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>zunta(作画) はらわたさいぞう(原作)</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>第40話：親友だから③</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="0" t="inlineStr">
         <is>
           <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>第25話-1「女神教の狙い」</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="0" t="inlineStr">
         <is>
           <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>光永康則</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>第７９話『呉越停止』③</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="0" t="inlineStr">
         <is>
           <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>マツモトケンゴ</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>第８３話　ラッキースケベの戦いが始まった（２）</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
         <is>
           <t>第8話後編：アトリ</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="0" t="inlineStr">
         <is>
           <t>クラスで２番目に可愛い女の子と友だちになった</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
         <is>
           <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr">
         <is>
           <t>第43話①</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="0" t="inlineStr">
         <is>
           <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
         <is>
           <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="0" t="inlineStr">
         <is>
           <t>第11話 前編</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="0" t="inlineStr">
         <is>
           <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>第21話-2</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t>いとこのこ</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>いぬちく(著者)</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>休載イラスト</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="0" t="n">
         <v>13</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>板垣恵介 猪原賽 陸井栄史</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>第100話　禁じ手</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="0" t="inlineStr">
         <is>
           <t>美人女上司滝沢さん</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>やんBARU(著者)</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>コミックス告知</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
         <is>
           <t>実は俺、最強でした？</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="0" t="inlineStr">
         <is>
           <t>第150話　支配する者</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="0" t="inlineStr">
         <is>
           <t>リビルドワールド</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t>第83話③</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" s="0" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="0" t="inlineStr">
         <is>
           <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="0" t="inlineStr">
         <is>
           <t>第40話 独身貴族は友人を実家に連れていく（4）</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="0" t="inlineStr">
         <is>
           <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="0" t="inlineStr">
         <is>
           <t>モリタ Ｕ４ nima</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="0" t="inlineStr">
         <is>
           <t>第17話（２）　クリスティーナお姉さまの結婚（２）</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="0" t="inlineStr">
         <is>
           <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="0" t="inlineStr">
         <is>
           <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="0" t="inlineStr">
         <is>
           <t>第47話-2</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="0" t="inlineStr">
         <is>
           <t>描けないのでヤってみた</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="0" t="inlineStr">
         <is>
           <t>逢上おかき(著者)</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>第4話</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="0" t="inlineStr">
         <is>
           <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr">
         <is>
           <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>第６２話　単独調査する器用貧乏（２）</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="A23" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="0" t="inlineStr">
         <is>
           <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
         <is>
           <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>第5話④</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="n">
+      <c r="A24" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="0" t="inlineStr">
         <is>
           <t>「お相手は一般の方です」</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>嵯峨祐介(著者)</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>第1話</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
+      <c r="A25" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="0" t="inlineStr">
         <is>
           <t>お前がヤったんだろ！</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr">
         <is>
           <t>クシザキ</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="0" t="inlineStr">
         <is>
           <t>第15話	君に入らせたい部活があるんだ</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="n">
+      <c r="A26" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="0" t="inlineStr">
         <is>
           <t>リアデイルの大地にて</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>月見だしお(著者) Ceez(原作) てんまそ(キャラクター原案) 涼風涼(構成)</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="0" t="inlineStr">
         <is>
           <t>第43章</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="n">
+      <c r="A27" s="0" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="0" t="inlineStr">
         <is>
           <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="0" t="inlineStr">
         <is>
           <t>板垣恵介 林たかあき</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="0" t="inlineStr">
         <is>
           <t>第74話 止まらぬ思考</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="n">
+      <c r="A28" s="0" t="n">
         <v>27</v>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="0" t="inlineStr">
         <is>
           <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="0" t="inlineStr">
         <is>
           <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="0" t="inlineStr">
         <is>
           <t>第49話　奴の罪（後編）</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="n">
+      <c r="A29" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="0" t="inlineStr">
         <is>
           <t>イケメンお姉さんはそーゆー目で見られたい</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="0" t="inlineStr">
         <is>
           <t>ヨウハ(著者)</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="0" t="inlineStr">
         <is>
           <t>第3話-2</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="n">
+      <c r="A30" s="0" t="n">
         <v>29</v>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="0" t="inlineStr">
         <is>
           <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="0" t="inlineStr">
         <is>
           <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="0" t="inlineStr">
         <is>
           <t>第69話②　あにめを見てみた</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="n">
+      <c r="A31" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="0" t="inlineStr">
         <is>
           <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="0" t="inlineStr">
         <is>
           <t>内々けやき あし カオミン</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="0" t="inlineStr">
         <is>
           <t>第158話 よくわからないけれど新たな問題が発生したみたいです（１）</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="n">
+      <c r="A32" s="0" t="n">
         <v>31</v>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="0" t="inlineStr">
         <is>
           <t>姫様“拷問”の時間です</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr">
         <is>
           <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="0" t="inlineStr">
         <is>
           <t>拷問193</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="n">
+      <c r="A33" s="0" t="n">
         <v>32</v>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="0" t="inlineStr">
         <is>
           <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="0" t="inlineStr">
         <is>
           <t>コミックス発売告知</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="n">
+      <c r="A34" s="0" t="n">
         <v>33</v>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="0" t="inlineStr">
         <is>
           <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="0" t="inlineStr">
         <is>
           <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="0" t="inlineStr">
         <is>
           <t>第４９話　ガイアスと剣神、激戦を繰り広げる。勇者は、オカモトさんに不吉な占いをされてしまう（３）</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="n">
+      <c r="A35" s="0" t="n">
         <v>34</v>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="0" t="inlineStr">
         <is>
           <t>追放僧侶の賢者タイム</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="0" t="inlineStr">
         <is>
           <t>原作・野原のはて 作画・鈴木シオン</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="0" t="inlineStr">
         <is>
           <t>第8話　ワンオンワン</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="n">
+      <c r="A36" s="0" t="n">
         <v>35</v>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="0" t="inlineStr">
         <is>
           <t>サーシャちゃんとクラスメイトオタクくん</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="0" t="inlineStr">
         <is>
           <t>はぐはぐ(著者)</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="0" t="inlineStr">
         <is>
           <t>第101話後編</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="n">
+      <c r="A37" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="0" t="inlineStr">
         <is>
           <t>物語の黒幕に転生して</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="0" t="inlineStr">
         <is>
           <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="0" t="inlineStr">
         <is>
           <t>第42話</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="n">
+      <c r="A38" s="0" t="n">
         <v>37</v>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="0" t="inlineStr">
         <is>
           <t>このヒーラー、めんどくさい</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="0" t="inlineStr">
         <is>
           <t>丹念に発酵(著者)</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="0" t="inlineStr">
         <is>
           <t>【コメント募集企画】もしもカーラが現代日本でバイトするならどんなお仕事!?【コミックス発売記念】</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="n">
+      <c r="A39" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="0" t="inlineStr">
         <is>
           <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="0" t="inlineStr">
         <is>
           <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="0" t="inlineStr">
         <is>
           <t>第10話-２</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="n">
+      <c r="A40" s="0" t="n">
         <v>39</v>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="0" t="inlineStr">
         <is>
           <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="0" t="inlineStr">
         <is>
           <t>FUNA 東西 モトエ恵介</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="0" t="inlineStr">
         <is>
           <t>第132話 第2回異世界懇談会［その③］</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="n">
+      <c r="A41" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="0" t="inlineStr">
         <is>
           <t>俺の幼馴染がデッッッッかくなりすぎた</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="0" t="inlineStr">
         <is>
           <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="0" t="inlineStr">
         <is>
           <t>第3話-2</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="n">
+      <c r="A42" s="0" t="n">
         <v>41</v>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="0" t="inlineStr">
         <is>
           <t>幼女戦記</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="0" t="inlineStr">
         <is>
           <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="0" t="inlineStr">
         <is>
           <t>第百十九章：邂逅Ⅳ</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="n">
+      <c r="A43" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="0" t="inlineStr">
         <is>
           <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="0" t="inlineStr">
         <is>
           <t>KAKERU</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="0" t="inlineStr">
         <is>
           <t>第78話「ケンタウロス」（後半）</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="n">
+      <c r="A44" s="0" t="n">
         <v>43</v>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="0" t="inlineStr">
         <is>
           <t>最弱貴族に転生したので悪役たちを集めてみた</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="0" t="inlineStr">
         <is>
           <t>空野進 sorani ファルまろ</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="0" t="inlineStr">
         <is>
           <t>第22話　最弱貴族、伯爵を撃退する(４)</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="n">
+      <c r="A45" s="0" t="n">
         <v>44</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="0" t="inlineStr">
         <is>
           <t>雨森潤奈は湿度が高い</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="0" t="inlineStr">
         <is>
           <t>水城水城(原作) 稲鳴四季(作画) 潮崎しの(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="0" t="inlineStr">
         <is>
           <t>第3話</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="n">
+      <c r="A46" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="0" t="inlineStr">
         <is>
           <t>塔の管理をしてみよう</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="0" t="inlineStr">
         <is>
           <t>盧恩＆雪笠(Friendly Land)(著者) 早秋(原作) 雨神(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="0" t="inlineStr">
         <is>
           <t>第103話前編</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="n">
+      <c r="A47" s="0" t="n">
         <v>46</v>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="0" t="inlineStr">
         <is>
           <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="0" t="inlineStr">
         <is>
           <t>漫画/すたひろ 原作/Y.A</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="0" t="inlineStr">
         <is>
           <t>chapter90【47話①】</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="n">
+      <c r="A48" s="0" t="n">
         <v>47</v>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="0" t="inlineStr">
         <is>
           <t>おせっかい女子、恋をする</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="0" t="inlineStr">
         <is>
           <t>音竹 ひかる(著者)</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="0" t="inlineStr">
         <is>
           <t>第26話</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="n">
+      <c r="A49" s="0" t="n">
         <v>48</v>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="0" t="inlineStr">
         <is>
           <t>黄金の経験値</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="0" t="inlineStr">
         <is>
           <t>原純(原作) 霜月汐(作画) fixro2n(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="0" t="inlineStr">
         <is>
           <t>第27話</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="n">
+      <c r="A50" s="0" t="n">
         <v>49</v>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="0" t="inlineStr">
         <is>
           <t>解雇された暗黒兵士(30代)のスローなセカンドライフ</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="0" t="inlineStr">
         <is>
           <t>岡沢六十四 るれくちぇ sage・ジョー</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="0" t="inlineStr">
         <is>
           <t>第83話(前編) 修羅と地獄</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="n">
+      <c r="A51" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="0" t="inlineStr">
         <is>
           <t>魔王になったので、ダンジョン造って人外娘とほのぼのする</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="0" t="inlineStr">
         <is>
           <t>遠野ノオト(作画) 流優(原作) だぶ竜(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="0" t="inlineStr">
         <is>
           <t>第91話後半</t>
         </is>
@@ -57493,6 +57494,1042 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>魔術師クノンは見えている</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>第50話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>第81話 後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>第157話	文珠たんたん</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>異世界居酒屋「のぶ」</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>第133話</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>第７９話『呉越停止』④</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>第８４話　告白の戦いが始まった（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>いとこのこ</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>いぬちく(著者)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>『いとこのこ』コミックス６巻 速報!!!</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>淫獄団地</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>最終話</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>おまけ75</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>第12話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>第329話</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>第24話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ダークサモナーとデキている</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>車王(著者)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>第95話</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>「おかえり、パパ」</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>蝉丸</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>第37話　内緒話</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>剥かせて！竜ケ崎さん</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>一智和智</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>大学生編 第23話</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>第83話④</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>第5話⑤</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>第６２話　単独調査する器用貧乏（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>第12話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>第54話 次期侯爵と二次会を①</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>姫ヶ崎櫻子は今日も不憫可愛い</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>安田剛助(著者)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>第58話</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>異世界食堂　洋食のねこや</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>第48話➁</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>おとなりのダウナーさんは無理させない</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>瑠璃いろ(著者)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>第17話</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>第90話その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>田舎で恋は難しい!?</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ねこうめ(著者)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>1巻告知</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>第17話-1：二番弟子</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>第４９話　ガイアスと剣神、激戦を繰り広げる。勇者は、オカモトさんに不吉な占いをされてしまう（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>拷問194</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>第11話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>第158話 よくわからないけれど新たな問題が発生したみたいです（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>不純な彼女達は懺悔しない</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ポロロッカ(著者)</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>コミックス告知</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>第32話</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>セレビィ量産型(著者)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>第29話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>インフィニット・デンドログラム</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>第80話</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>回復術士のやり直し</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>月夜涙(原作) 羽賀ソウケン(漫画) しおこんぶ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>第79話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>【目つき悪いシリーズ】ミタメトウラハラ</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ウラベスナヒト</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>#14印象</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>第100話</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ギャル神官はリザレがダルい</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>秋★枝</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>第9話</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ギャルの自転車を直したら懐かれた</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>タケチケイ（漫画） 生姜寧也（原作）</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>第3話　ギャルと約束した（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ライブダンジョン！</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>第98話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>第25話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>宇崎ちゃんは遊びたい！</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>丈(著者)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>第139話</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>EP.28②</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>最果てのパラディン</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>奥橋睦（漫画） 柳野かなた（原作） 輪くすさが（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>第72章　無敵の巨人Ⅴ</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>「お相手は一般の方です」</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>嵯峨祐介(著者)</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>第2話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>おせっかい女子、恋をする</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>音竹 ひかる(著者)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>第27話</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>役目を果たした日陰の勇者は、辺境で自由に生きていきます</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>船野真帆(作画) 丘野優(原作) 布施龍太(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>第17話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>女子高生の無駄づかい</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ビーノ(著者)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>第147話　じっけん</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>オタクに優しいギャルはいない!?</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>のりしろちゃん 魚住さかな</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>【#202】瀬尾卓也へ捧ぐ</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>無職の英雄　別にスキルなんか要らなかったんだが</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>原作：九頭七尾・上田夢人 漫画：名苗秋緒</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>第56話</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add ranking data for 2026-08-10
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -66,6 +66,7 @@
     <sheet name="2026-07-20" sheetId="58" state="visible" r:id="rId58"/>
     <sheet name="2026-07-27" sheetId="59" state="visible" r:id="rId59"/>
     <sheet name="2026-08-03" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet name="2026-08-10" sheetId="61" state="visible" r:id="rId61"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -57526,22 +57527,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>魔術師クノンは見えている</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第50話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第81話 後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第157話	文珠たんたん</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>異世界居酒屋「のぶ」</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第133話</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第７９話『呉越停止』④</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第８４話　告白の戦いが始まった（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>いとこのこ</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>いぬちく(著者)</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>『いとこのこ』コミックス６巻 速報!!!</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>淫獄団地</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>最終話</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>おまけ75</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第12話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第329話</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第24話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>ダークサモナーとデキている</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>車王(著者)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第95話</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>「おかえり、パパ」</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>蝉丸</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第37話　内緒話</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>剥かせて！竜ケ崎さん</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>一智和智</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>大学生編 第23話</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第83話④</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第5話⑤</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第６２話　単独調査する器用貧乏（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第12話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第54話 次期侯爵と二次会を①</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>姫ヶ崎櫻子は今日も不憫可愛い</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>安田剛助(著者)</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第58話</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>異世界食堂　洋食のねこや</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第48話➁</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>おとなりのダウナーさんは無理させない</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>瑠璃いろ(著者)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第17話</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第90話その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>田舎で恋は難しい!?</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>ねこうめ(著者)</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>1巻告知</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第17話-1：二番弟子</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第４９話　ガイアスと剣神、激戦を繰り広げる。勇者は、オカモトさんに不吉な占いをされてしまう（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>拷問194</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第11話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第158話 よくわからないけれど新たな問題が発生したみたいです（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>不純な彼女達は懺悔しない</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>ポロロッカ(著者)</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>コミックス告知</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第32話</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>セレビィ量産型(著者)</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第29話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>インフィニット・デンドログラム</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第80話</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>回復術士のやり直し</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>月夜涙(原作) 羽賀ソウケン(漫画) しおこんぶ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第79話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>【目つき悪いシリーズ】ミタメトウラハラ</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>ウラベスナヒト</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>#14印象</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第100話</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>ギャル神官はリザレがダルい</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>秋★枝</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第9話</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>ギャルの自転車を直したら懐かれた</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>タケチケイ（漫画） 生姜寧也（原作）</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第3話　ギャルと約束した（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>ライブダンジョン！</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第98話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第25話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>宇崎ちゃんは遊びたい！</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>丈(著者)</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第139話</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>EP.28②</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>最果てのパラディン</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>奥橋睦（漫画） 柳野かなた（原作） 輪くすさが（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第72章　無敵の巨人Ⅴ</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>「お相手は一般の方です」</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>嵯峨祐介(著者)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第2話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>おせっかい女子、恋をする</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>音竹 ひかる(著者)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第27話</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>役目を果たした日陰の勇者は、辺境で自由に生きていきます</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>船野真帆(作画) 丘野優(原作) 布施龍太(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第17話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>女子高生の無駄づかい</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>ビーノ(著者)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第147話　じっけん</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>オタクに優しいギャルはいない!?</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>のりしろちゃん 魚住さかな</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>【#202】瀬尾卓也へ捧ぐ</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>無職の英雄　別にスキルなんか要らなかったんだが</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>原作：九頭七尾・上田夢人 漫画：名苗秋緒</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第56話</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>魔術師クノンは見えている</t>
+          <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+          <t>丈(著者)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第50話①</t>
+          <t>第140話</t>
         </is>
       </c>
     </row>
@@ -57551,17 +58588,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+          <t>ワンパンマン</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第81話 後編</t>
+          <t>233撃目</t>
         </is>
       </c>
     </row>
@@ -57571,17 +58608,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>むちまろ</t>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第157話	文珠たんたん</t>
+          <t>第41話：「女の先輩」として①</t>
         </is>
       </c>
     </row>
@@ -57591,17 +58628,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>異世界居酒屋「のぶ」</t>
+          <t>魔王の俺が奴隷エルフを嫁にしたんだが、どう愛でればいい？</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
+          <t>原作／手島史詞 キャラクター原案／COMTA 漫画／板垣ハコ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第133話</t>
+          <t>第81話</t>
         </is>
       </c>
     </row>
@@ -57611,17 +58648,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第７９話『呉越停止』④</t>
+          <t>第89話その1</t>
         </is>
       </c>
     </row>
@@ -57631,17 +58668,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第８４話　告白の戦いが始まった（１）</t>
+          <t>第８０話『異教停止』①</t>
         </is>
       </c>
     </row>
@@ -57651,17 +58688,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>いとこのこ</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>いぬちく(著者)</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>『いとこのこ』コミックス６巻 速報!!!</t>
+          <t>第８４話　告白の戦いが始まった（２）</t>
         </is>
       </c>
     </row>
@@ -57671,17 +58708,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>淫獄団地</t>
+          <t>王子様の友達</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>搾精研究所(原作) 丈山雄為(漫画)</t>
+          <t>すけろく(著者)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>最終話</t>
+          <t>第39話</t>
         </is>
       </c>
     </row>
@@ -57691,17 +58728,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>いとこのこ</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>いぬちく(著者)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>おまけ75</t>
+          <t>しばらく休載と尊のお怒りイラスト</t>
         </is>
       </c>
     </row>
@@ -57711,17 +58748,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>三部べべ(漫画) ねうしとら(原作)</t>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第12話-1</t>
+          <t>第25話</t>
         </is>
       </c>
     </row>
@@ -57731,17 +58768,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>異世界のんびり農家</t>
+          <t>帰ってください！ 阿久津さん</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+          <t>長岡太一(著者)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第329話</t>
+          <t>第210話</t>
         </is>
       </c>
     </row>
@@ -57751,17 +58788,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>クセ強彼女は床にいざなう</t>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>須河篤志(著者)</t>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第24話後半</t>
+          <t>特別イラスト</t>
         </is>
       </c>
     </row>
@@ -57771,17 +58808,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ダークサモナーとデキている</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>車王(著者)</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第95話</t>
+          <t>第139話　ひさびさに本気出してみるⅣ（前編）</t>
         </is>
       </c>
     </row>
@@ -57791,17 +58828,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>「おかえり、パパ」</t>
+          <t>このヒーラー、めんどくさい</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>蝉丸</t>
+          <t>丹念に発酵(著者)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第37話　内緒話</t>
+          <t>第100話：見つめていたい</t>
         </is>
       </c>
     </row>
@@ -57811,17 +58848,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>剥かせて！竜ケ崎さん</t>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>一智和智</t>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>大学生編 第23話</t>
+          <t>第101話　己の意を通す力</t>
         </is>
       </c>
     </row>
@@ -57831,17 +58868,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>まんきつしたい常連さん</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>しんみりん(著者)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第83話④</t>
+          <t>第58話前編</t>
         </is>
       </c>
     </row>
@@ -57851,17 +58888,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第5話⑤</t>
+          <t>第151話　テレジアの秘密</t>
         </is>
       </c>
     </row>
@@ -57871,17 +58908,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第６２話　単独調査する器用貧乏（３）</t>
+          <t>第84話①</t>
         </is>
       </c>
     </row>
@@ -57891,17 +58928,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+          <t>田舎で恋は難しい!?</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+          <t>ねこうめ(著者)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第12話前編</t>
+          <t>第9話</t>
         </is>
       </c>
     </row>
@@ -57911,17 +58948,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+          <t>望まぬ不死の冒険者</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+          <t>中曽根ハイジ（漫画） 丘野 優（原作） じゃいあん（キャラクター原案）</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第54話 次期侯爵と二次会を①</t>
+          <t>第66話　因縁の敵（前編）</t>
         </is>
       </c>
     </row>
@@ -57931,17 +58968,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>姫ヶ崎櫻子は今日も不憫可愛い</t>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>安田剛助(著者)</t>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第58話</t>
+          <t>第３１食　氷結果実、パクパクですわ！（２）</t>
         </is>
       </c>
     </row>
@@ -57951,17 +58988,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>異世界食堂　洋食のねこや</t>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
+          <t>モリタ Ｕ４ nima</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第48話➁</t>
+          <t>第17話（３）　クリスティーナお姉さまの結婚（３）</t>
         </is>
       </c>
     </row>
@@ -57971,17 +59008,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>おとなりのダウナーさんは無理させない</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>瑠璃いろ(著者)</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第17話</t>
+          <t>第6話①</t>
         </is>
       </c>
     </row>
@@ -57991,17 +59028,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>お前がヤったんだろ！</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>クシザキ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第90話その1</t>
+          <t>第16話	川原ナデシコの動揺</t>
         </is>
       </c>
     </row>
@@ -58011,17 +59048,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>田舎で恋は難しい!?</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ねこうめ(著者)</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>1巻告知</t>
+          <t>第６２話　単独調査する器用貧乏（４）</t>
         </is>
       </c>
     </row>
@@ -58031,17 +59068,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第17話-1：二番弟子</t>
+          <t>第70話①　あにめを作ってみた</t>
         </is>
       </c>
     </row>
@@ -58051,17 +59088,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>美人女上司滝沢さん</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>やんBARU(著者)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第４９話　ガイアスと剣神、激戦を繰り広げる。勇者は、オカモトさんに不吉な占いをされてしまう（４）</t>
+          <t>第222.5話</t>
         </is>
       </c>
     </row>
@@ -58071,17 +59108,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>オタくんにだけ優しすぎるアヤメさん</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>藤田丞(原作) 御影夏(作画)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>拷問194</t>
+          <t>第1話　おつきあい</t>
         </is>
       </c>
     </row>
@@ -58091,17 +59128,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+          <t>板垣恵介 林たかあき</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第11話-2</t>
+          <t>第75話 忍耐力</t>
         </is>
       </c>
     </row>
@@ -58111,17 +59148,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第158話 よくわからないけれど新たな問題が発生したみたいです（２）</t>
+          <t>第90話その2</t>
         </is>
       </c>
     </row>
@@ -58131,17 +59168,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>不純な彼女達は懺悔しない</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ポロロッカ(著者)</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>コミックス告知</t>
+          <t>拷問195</t>
         </is>
       </c>
     </row>
@@ -58151,17 +59188,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
+          <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
+          <t>クール教信者</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第32話</t>
+          <t>第171話</t>
         </is>
       </c>
     </row>
@@ -58171,17 +59208,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>三枝さんはメガネ先輩と恋を描く</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>セレビィ量産型(著者)</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第29話前半</t>
+          <t>第４９話　ガイアスと剣神、激戦を繰り広げる。勇者は、オカモトさんに不吉な占いをされてしまう（５）</t>
         </is>
       </c>
     </row>
@@ -58191,17 +59228,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>インフィニット・デンドログラム</t>
+          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
+          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第80話</t>
+          <t>第48話-2</t>
         </is>
       </c>
     </row>
@@ -58211,17 +59248,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>回復術士のやり直し</t>
+          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>月夜涙(原作) 羽賀ソウケン(漫画) しおこんぶ(キャラクター原案)</t>
+          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第79話-2</t>
+          <t>第6話</t>
         </is>
       </c>
     </row>
@@ -58231,17 +59268,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>【目つき悪いシリーズ】ミタメトウラハラ</t>
+          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ウラベスナヒト</t>
+          <t>六志麻あさ 業務用餅 kisui</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>#14印象</t>
+          <t>第９１話</t>
         </is>
       </c>
     </row>
@@ -58251,17 +59288,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>くらいあの子としたいこと</t>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>碇マナツ(著者)</t>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第100話</t>
+          <t>特別イラスト２</t>
         </is>
       </c>
     </row>
@@ -58271,17 +59308,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ギャル神官はリザレがダルい</t>
+          <t>理想のヒモ生活</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>秋★枝</t>
+          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第9話</t>
+          <t>第109話　その2</t>
         </is>
       </c>
     </row>
@@ -58291,17 +59328,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ギャルの自転車を直したら懐かれた</t>
+          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>タケチケイ（漫画） 生姜寧也（原作）</t>
+          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第3話　ギャルと約束した（後編）</t>
+          <t>第66話　扉の先へ</t>
         </is>
       </c>
     </row>
@@ -58311,17 +59348,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ライブダンジョン！</t>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+          <t>原作:剃り残し 漫画:大窪太一</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第98話後半</t>
+          <t>第10話(後編)</t>
         </is>
       </c>
     </row>
@@ -58331,17 +59368,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+          <t>KAKERU</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第25話①</t>
+          <t>第79話「ケンタウロス2」（前半）</t>
         </is>
       </c>
     </row>
@@ -58351,17 +59388,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>宇崎ちゃんは遊びたい！</t>
+          <t>美容スキルでクラスの女の子を可愛くしたい</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>丈(著者)</t>
+          <t>藤白ぺるか(原作) 紺野あずれ(漫画) 水野早桜(キャラクター原案)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第139話</t>
+          <t>第9話</t>
         </is>
       </c>
     </row>
@@ -58371,17 +59408,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+          <t>魔法少女リリカルなのは EXCEEDS</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+          <t>都築真紀 川上修一</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>EP.28②</t>
+          <t>第１４話②</t>
         </is>
       </c>
     </row>
@@ -58391,17 +59428,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>最果てのパラディン</t>
+          <t>世界最強の後衛 ～迷宮国の新人探索者～</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>奥橋睦（漫画） 柳野かなた（原作） 輪くすさが（キャラクター原案）</t>
+          <t>力蔵(著者) とーわ(原作) 風花風花(キャラクター原案)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第72章　無敵の巨人Ⅴ</t>
+          <t>第44話-2</t>
         </is>
       </c>
     </row>
@@ -58411,17 +59448,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>「お相手は一般の方です」</t>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>嵯峨祐介(著者)</t>
+          <t>はぐはぐ(著者)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第2話前半</t>
+          <t>第102話</t>
         </is>
       </c>
     </row>
@@ -58431,17 +59468,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>おせっかい女子、恋をする</t>
+          <t>遊遊じてき。</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>音竹 ひかる(著者)</t>
+          <t>カンケー</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第27話</t>
+          <t>第12話</t>
         </is>
       </c>
     </row>
@@ -58451,17 +59488,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>役目を果たした日陰の勇者は、辺境で自由に生きていきます</t>
+          <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>船野真帆(作画) 丘野優(原作) 布施龍太(キャラクター原案)</t>
+          <t>昼行燈（原作） しいたけ元帥（漫画）</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第17話後半</t>
+          <t>第50話</t>
         </is>
       </c>
     </row>
@@ -58471,17 +59508,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>女子高生の無駄づかい</t>
+          <t>おせっかい女子、恋をする</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ビーノ(著者)</t>
+          <t>音竹 ひかる(著者)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第147話　じっけん</t>
+          <t>第28話</t>
         </is>
       </c>
     </row>
@@ -58491,17 +59528,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>オタクに優しいギャルはいない!?</t>
+          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>のりしろちゃん 魚住さかな</t>
+          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>【#202】瀬尾卓也へ捧ぐ</t>
+          <t>第11話①「かなわないな」</t>
         </is>
       </c>
     </row>
@@ -58511,17 +59548,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>無職の英雄　別にスキルなんか要らなかったんだが</t>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>原作：九頭七尾・上田夢人 漫画：名苗秋緒</t>
+          <t>空野進 sorani ファルまろ</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第56話</t>
+          <t>第23話 最弱貴族、エルフの里へ向かう（１）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-08-17
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -67,6 +67,7 @@
     <sheet name="2026-07-27" sheetId="59" state="visible" r:id="rId59"/>
     <sheet name="2026-08-03" sheetId="60" state="visible" r:id="rId60"/>
     <sheet name="2026-08-10" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet name="2026-08-17" sheetId="62" state="visible" r:id="rId62"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -58563,22 +58564,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>宇崎ちゃんは遊びたい！</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>丈(著者)</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第140話</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>ワンパンマン</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>233撃目</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第41話：「女の先輩」として①</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>魔王の俺が奴隷エルフを嫁にしたんだが、どう愛でればいい？</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>原作／手島史詞 キャラクター原案／COMTA 漫画／板垣ハコ</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第81話</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第89話その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第８０話『異教停止』①</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第８４話　告白の戦いが始まった（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>王子様の友達</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>すけろく(著者)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第39話</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>いとこのこ</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>いぬちく(著者)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>しばらく休載と尊のお怒りイラスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第25話</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>帰ってください！ 阿久津さん</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>長岡太一(著者)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第210話</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>特別イラスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第139話　ひさびさに本気出してみるⅣ（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>このヒーラー、めんどくさい</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>丹念に発酵(著者)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第100話：見つめていたい</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第101話　己の意を通す力</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>まんきつしたい常連さん</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>しんみりん(著者)</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第58話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第151話　テレジアの秘密</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第84話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>田舎で恋は難しい!?</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>ねこうめ(著者)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第9話</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>望まぬ不死の冒険者</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>中曽根ハイジ（漫画） 丘野 優（原作） じゃいあん（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第66話　因縁の敵（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第３１食　氷結果実、パクパクですわ！（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>モリタ Ｕ４ nima</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第17話（３）　クリスティーナお姉さまの結婚（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第6話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>クシザキ</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第16話	川原ナデシコの動揺</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第６２話　単独調査する器用貧乏（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第70話①　あにめを作ってみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>美人女上司滝沢さん</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>やんBARU(著者)</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第222.5話</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>オタくんにだけ優しすぎるアヤメさん</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>藤田丞(原作) 御影夏(作画)</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第1話　おつきあい</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 林たかあき</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第75話 忍耐力</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第90話その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>拷問195</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>小林さんちのメイドラゴン</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>クール教信者</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第171話</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第４９話　ガイアスと剣神、激戦を繰り広げる。勇者は、オカモトさんに不吉な占いをされてしまう（５）</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第48話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第6話</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>六志麻あさ 業務用餅 kisui</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第９１話</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>特別イラスト２</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>理想のヒモ生活</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第109話　その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第66話　扉の先へ</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>原作:剃り残し 漫画:大窪太一</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第10話(後編)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>KAKERU</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第79話「ケンタウロス2」（前半）</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>美容スキルでクラスの女の子を可愛くしたい</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>藤白ぺるか(原作) 紺野あずれ(漫画) 水野早桜(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第9話</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>魔法少女リリカルなのは EXCEEDS</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>都築真紀 川上修一</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第１４話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の後衛 ～迷宮国の新人探索者～</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>力蔵(著者) とーわ(原作) 風花風花(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第44話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>はぐはぐ(著者)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第102話</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>遊遊じてき。</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>カンケー</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第12話</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>昼行燈（原作） しいたけ元帥（漫画）</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第50話</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>おせっかい女子、恋をする</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>音竹 ひかる(著者)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第28話</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第11話①「かなわないな」</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>空野進 sorani ファルまろ</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第23話 最弱貴族、エルフの里へ向かう（１）</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>宇崎ちゃんは遊びたい！</t>
+          <t>不徳のギルド</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>丈(著者)</t>
+          <t>河添太一</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第140話</t>
+          <t>第１０９話：五合目</t>
         </is>
       </c>
     </row>
@@ -58588,17 +59625,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ワンパンマン</t>
+          <t>魔術師クノンは見えている</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>原作/ＯＮＥ 作画/村田雄介</t>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>233撃目</t>
+          <t>第50話②</t>
         </is>
       </c>
     </row>
@@ -58618,7 +59655,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第41話：「女の先輩」として①</t>
+          <t>第41話：「女の先輩」として②</t>
         </is>
       </c>
     </row>
@@ -58628,17 +59665,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>魔王の俺が奴隷エルフを嫁にしたんだが、どう愛でればいい？</t>
+          <t>蜘蛛ですが、なにか？</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>原作／手島史詞 キャラクター原案／COMTA 漫画／板垣ハコ</t>
+          <t>かかし朝浩(著者) 馬場翁(原作) 輝竜司(キャラクター原案)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第81話</t>
+          <t>第80話その1</t>
         </is>
       </c>
     </row>
@@ -58648,17 +59685,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第89話その1</t>
+          <t>第25話-2「女神教の狙い」</t>
         </is>
       </c>
     </row>
@@ -58678,7 +59715,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第８０話『異教停止』①</t>
+          <t>第８０話『異教停止』②</t>
         </is>
       </c>
     </row>
@@ -58688,17 +59725,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第８４話　告白の戦いが始まった（２）</t>
+          <t>第9話前編：出立の朝</t>
         </is>
       </c>
     </row>
@@ -58708,17 +59745,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>王子様の友達</t>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>すけろく(著者)</t>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第39話</t>
+          <t>第43話②</t>
         </is>
       </c>
     </row>
@@ -58728,17 +59765,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>いとこのこ</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>いぬちく(著者)</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>しばらく休載と尊のお怒りイラスト</t>
+          <t>第８５話　プールサイドの戦いが始まった</t>
         </is>
       </c>
     </row>
@@ -58748,17 +59785,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+          <t>ダンジョンの幼なじみ</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+          <t>久真やすひさ(著者)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第25話</t>
+          <t>第67話</t>
         </is>
       </c>
     </row>
@@ -58768,17 +59805,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>帰ってください！ 阿久津さん</t>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>長岡太一(著者)</t>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第210話</t>
+          <t>第22話-1</t>
         </is>
       </c>
     </row>
@@ -58788,17 +59825,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+          <t>久遠まこと(著者) 石のやっさん(原作)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>特別イラスト</t>
+          <t>第39話</t>
         </is>
       </c>
     </row>
@@ -58808,17 +59845,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>ダークサモナーとデキている</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>車王(著者)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第139話　ひさびさに本気出してみるⅣ（前編）</t>
+          <t>第96話</t>
         </is>
       </c>
     </row>
@@ -58828,17 +59865,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>このヒーラー、めんどくさい</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>丹念に発酵(著者)</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第100話：見つめていたい</t>
+          <t>第139話　ひさびさに本気出してみるⅣ（中編）</t>
         </is>
       </c>
     </row>
@@ -58848,17 +59885,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>板垣恵介 猪原賽 陸井栄史</t>
+          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第101話　己の意を通す力</t>
+          <t>第41話</t>
         </is>
       </c>
     </row>
@@ -58868,17 +59905,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>まんきつしたい常連さん</t>
+          <t>クールな同級生の10年後</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>しんみりん(著者)</t>
+          <t>狛野まこ(著者) 球体X(原作・キャラクター原案) 雨音恵(ノベル原作)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第58話前編</t>
+          <t>第1話</t>
         </is>
       </c>
     </row>
@@ -58888,17 +59925,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第151話　テレジアの秘密</t>
+          <t>第12話-2</t>
         </is>
       </c>
     </row>
@@ -58908,17 +59945,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第84話①</t>
+          <t>第152話　三主神</t>
         </is>
       </c>
     </row>
@@ -58928,17 +59965,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>田舎で恋は難しい!?</t>
+          <t>魔のものたちは企てる</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ねこうめ(著者)</t>
+          <t>加藤拓弐(原作) ガしガし(作画)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第9話</t>
+          <t>第38話</t>
         </is>
       </c>
     </row>
@@ -58948,17 +59985,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>望まぬ不死の冒険者</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>中曽根ハイジ（漫画） 丘野 優（原作） じゃいあん（キャラクター原案）</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第66話　因縁の敵（前編）</t>
+          <t>第84話➁</t>
         </is>
       </c>
     </row>
@@ -58968,17 +60005,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+          <t>クセ強彼女は床にいざなう</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>島知宏 音速炒飯 有都あらゆる</t>
+          <t>須河篤志(著者)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第３１食　氷結果実、パクパクですわ！（２）</t>
+          <t>休載イラスト</t>
         </is>
       </c>
     </row>
@@ -58988,17 +60025,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>モリタ Ｕ４ nima</t>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第17話（３）　クリスティーナお姉さまの結婚（３）</t>
+          <t>第10話 フェア</t>
         </is>
       </c>
     </row>
@@ -59018,7 +60055,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第6話①</t>
+          <t>第6話②</t>
         </is>
       </c>
     </row>
@@ -59028,17 +60065,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>お前がヤったんだろ！</t>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>クシザキ</t>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第16話	川原ナデシコの動揺</t>
+          <t>休載イラスト</t>
         </is>
       </c>
     </row>
@@ -59048,17 +60085,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>転生貴族の異世界冒険録 ～自重を知らない神々の使徒～</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>夜州 nini 藻</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第６２話　単独調査する器用貧乏（４）</t>
+          <t>第76話（後編）</t>
         </is>
       </c>
     </row>
@@ -59068,17 +60105,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第70話①　あにめを作ってみた</t>
+          <t>第54話 次期侯爵と二次会を②</t>
         </is>
       </c>
     </row>
@@ -59088,17 +60125,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>美人女上司滝沢さん</t>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>やんBARU(著者)</t>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第222.5話</t>
+          <t>第３１食　氷結果実、パクパクですわ！（３）</t>
         </is>
       </c>
     </row>
@@ -59108,17 +60145,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>オタくんにだけ優しすぎるアヤメさん</t>
+          <t>まったく最近の探偵ときたら</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>藤田丞(原作) 御影夏(作画)</t>
+          <t>五十嵐正邦(著者)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第1話　おつきあい</t>
+          <t>第118話①</t>
         </is>
       </c>
     </row>
@@ -59128,17 +60165,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+          <t>お前がヤったんだろ！</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>板垣恵介 林たかあき</t>
+          <t>クシザキ</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第75話 忍耐力</t>
+          <t>第17話	佐倉モモカの幸運</t>
         </is>
       </c>
     </row>
@@ -59148,17 +60185,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>ヨウハ(著者)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第90話その2</t>
+          <t>第4話-1</t>
         </is>
       </c>
     </row>
@@ -59178,7 +60215,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>拷問195</t>
+          <t>拷問196</t>
         </is>
       </c>
     </row>
@@ -59188,17 +60225,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>小林さんちのメイドラゴン</t>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>クール教信者</t>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第171話</t>
+          <t>第17話-2：二番弟子</t>
         </is>
       </c>
     </row>
@@ -59208,17 +60245,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第４９話　ガイアスと剣神、激戦を繰り広げる。勇者は、オカモトさんに不吉な占いをされてしまう（５）</t>
+          <t>第50話　奴は土下座する（前編）</t>
         </is>
       </c>
     </row>
@@ -59228,17 +60265,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第48話-2</t>
+          <t>第６３話　妖精と出会った器用貧乏（１）</t>
         </is>
       </c>
     </row>
@@ -59248,17 +60285,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
+          <t>望まぬ不死の冒険者</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
+          <t>中曽根ハイジ（漫画） 丘野 優（原作） じゃいあん（キャラクター原案）</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第6話</t>
+          <t>第66話　因縁の敵（後編）</t>
         </is>
       </c>
     </row>
@@ -59268,17 +60305,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>六志麻あさ 業務用餅 kisui</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第９１話</t>
+          <t>第70話②　あにめを作ってみた</t>
         </is>
       </c>
     </row>
@@ -59288,17 +60325,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>女友達は頼めば意外とヤらせてくれる</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ろくろ(漫画) 鏡遊(原作)</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>特別イラスト２</t>
+          <t>第90話その3</t>
         </is>
       </c>
     </row>
@@ -59308,17 +60345,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>理想のヒモ生活</t>
+          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
+          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第109話　その2</t>
+          <t>第4話-②</t>
         </is>
       </c>
     </row>
@@ -59328,17 +60365,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
+          <t>セレビィ量産型(著者)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第66話　扉の先へ</t>
+          <t>第29話後半</t>
         </is>
       </c>
     </row>
@@ -59348,17 +60385,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>原作:剃り残し 漫画:大窪太一</t>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第10話(後編)</t>
+          <t>第4話-1</t>
         </is>
       </c>
     </row>
@@ -59368,17 +60405,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>KAKERU</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第79話「ケンタウロス2」（前半）</t>
+          <t>第５０話　勇者、神々に封印される・・・いや、マジで！（１）</t>
         </is>
       </c>
     </row>
@@ -59388,17 +60425,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>美容スキルでクラスの女の子を可愛くしたい</t>
+          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>藤白ぺるか(原作) 紺野あずれ(漫画) 水野早桜(キャラクター原案)</t>
+          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第9話</t>
+          <t>第１話　冒険者パーティと開拓します！（２）</t>
         </is>
       </c>
     </row>
@@ -59408,17 +60445,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS</t>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>都築真紀 川上修一</t>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第１４話②</t>
+          <t>第12話-1</t>
         </is>
       </c>
     </row>
@@ -59428,17 +60465,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>世界最強の後衛 ～迷宮国の新人探索者～</t>
+          <t>俺は星間国家の悪徳領主！</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>力蔵(著者) とーわ(原作) 風花風花(キャラクター原案)</t>
+          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第44話-2</t>
+          <t>第50話　復讐心の正体</t>
         </is>
       </c>
     </row>
@@ -59448,17 +60485,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>サーシャちゃんとクラスメイトオタクくん</t>
+          <t>くらいあの子としたいこと</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>はぐはぐ(著者)</t>
+          <t>碇マナツ(著者)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第102話</t>
+          <t>第101話</t>
         </is>
       </c>
     </row>
@@ -59468,17 +60505,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>遊遊じてき。</t>
+          <t>異世界転生ダンジョンマスター　温泉ダンジョンを作る</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>カンケー</t>
+          <t>天原(原作) アルデヒド(作画) じゅん(キャラクター原案)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第12話</t>
+          <t>第5話</t>
         </is>
       </c>
     </row>
@@ -59488,17 +60525,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
+          <t>バーサス</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>昼行燈（原作） しいたけ元帥（漫画）</t>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第50話</t>
+          <t>第35話　ギンバックVS.大魔班（1）</t>
         </is>
       </c>
     </row>
@@ -59508,17 +60545,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>おせっかい女子、恋をする</t>
+          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>音竹 ひかる(著者)</t>
+          <t>FUNA 東西 モトエ恵介</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第28話</t>
+          <t>第133話 第2回異世界懇談会［その④］</t>
         </is>
       </c>
     </row>
@@ -59528,17 +60565,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
+          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
+          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第11話①「かなわないな」</t>
+          <t>EP.29①</t>
         </is>
       </c>
     </row>
@@ -59548,17 +60585,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+          <t>めっちゃ召喚された件 THE COMIC</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>空野進 sorani ファルまろ</t>
+          <t>漫画：六甲島カモメ 原作：さいとうさ キャラクター原案：ツグトク</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第23話 最弱貴族、エルフの里へ向かう（１）</t>
+          <t>第57話②</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-08-24
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -68,6 +68,7 @@
     <sheet name="2026-08-03" sheetId="60" state="visible" r:id="rId60"/>
     <sheet name="2026-08-10" sheetId="61" state="visible" r:id="rId61"/>
     <sheet name="2026-08-17" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet name="2026-08-24" sheetId="63" state="visible" r:id="rId63"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -59600,22 +59601,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>不徳のギルド</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>河添太一</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第１０９話：五合目</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>魔術師クノンは見えている</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第50話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第41話：「女の先輩」として②</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>蜘蛛ですが、なにか？</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>かかし朝浩(著者) 馬場翁(原作) 輝竜司(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第80話その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第25話-2「女神教の狙い」</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第８０話『異教停止』②</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第9話前編：出立の朝</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第43話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第８５話　プールサイドの戦いが始まった</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>ダンジョンの幼なじみ</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>久真やすひさ(著者)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第67話</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第22話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>久遠まこと(著者) 石のやっさん(原作)</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第39話</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>ダークサモナーとデキている</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>車王(著者)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第96話</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第139話　ひさびさに本気出してみるⅣ（中編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第41話</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>クールな同級生の10年後</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>狛野まこ(著者) 球体X(原作・キャラクター原案) 雨音恵(ノベル原作)</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第12話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第152話　三主神</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>魔のものたちは企てる</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>加藤拓弐(原作) ガしガし(作画)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第38話</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第84話➁</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>休載イラスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第10話 フェア</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第6話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>休載イラスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>転生貴族の異世界冒険録 ～自重を知らない神々の使徒～</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>夜州 nini 藻</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第76話（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第54話 次期侯爵と二次会を②</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第３１食　氷結果実、パクパクですわ！（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>まったく最近の探偵ときたら</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>五十嵐正邦(著者)</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第118話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>クシザキ</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第17話	佐倉モモカの幸運</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>ヨウハ(著者)</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第4話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>拷問196</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第17話-2：二番弟子</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第50話　奴は土下座する（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第６３話　妖精と出会った器用貧乏（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>望まぬ不死の冒険者</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>中曽根ハイジ（漫画） 丘野 優（原作） じゃいあん（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第66話　因縁の敵（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第70話②　あにめを作ってみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第90話その3</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第4話-②</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>セレビィ量産型(著者)</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第29話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第4話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第５０話　勇者、神々に封印される・・・いや、マジで！（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第１話　冒険者パーティと開拓します！（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第12話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>俺は星間国家の悪徳領主！</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第50話　復讐心の正体</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第101話</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>異世界転生ダンジョンマスター　温泉ダンジョンを作る</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>天原(原作) アルデヒド(作画) じゅん(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第5話</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>バーサス</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第35話　ギンバックVS.大魔班（1）</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>FUNA 東西 モトエ恵介</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第133話 第2回異世界懇談会［その④］</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>EP.29①</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>めっちゃ召喚された件 THE COMIC</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>漫画：六甲島カモメ 原作：さいとうさ キャラクター原案：ツグトク</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第57話②</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>不徳のギルド</t>
+          <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>河添太一</t>
+          <t>丈(著者)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第１０９話：五合目</t>
+          <t>第141話</t>
         </is>
       </c>
     </row>
@@ -59625,17 +60662,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>魔術師クノンは見えている</t>
+          <t>ワンパンマン</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第50話②</t>
+          <t>234撃目</t>
         </is>
       </c>
     </row>
@@ -59655,7 +60692,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第41話：「女の先輩」として②</t>
+          <t>第41話：「女の先輩」として③</t>
         </is>
       </c>
     </row>
@@ -59665,17 +60702,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>蜘蛛ですが、なにか？</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>かかし朝浩(著者) 馬場翁(原作) 輝竜司(キャラクター原案)</t>
+          <t>むちまろ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第80話その1</t>
+          <t>第158話	我が子の成長！</t>
         </is>
       </c>
     </row>
@@ -59685,17 +60722,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第25話-2「女神教の狙い」</t>
+          <t>第８０話『異教停止』③</t>
         </is>
       </c>
     </row>
@@ -59705,17 +60742,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第８０話『異教停止』②</t>
+          <t>第89話その2</t>
         </is>
       </c>
     </row>
@@ -59725,17 +60762,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第9話前編：出立の朝</t>
+          <t>第13話前半</t>
         </is>
       </c>
     </row>
@@ -59745,17 +60782,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+          <t>まんきつしたい常連さん</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+          <t>しんみりん(著者)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第43話②</t>
+          <t>第58話後編</t>
         </is>
       </c>
     </row>
@@ -59765,17 +60802,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第８５話　プールサイドの戦いが始まった</t>
+          <t>第102話　帰還</t>
         </is>
       </c>
     </row>
@@ -59785,17 +60822,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ダンジョンの幼なじみ</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>久真やすひさ(著者)</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第67話</t>
+          <t>第139話　ひさびさに本気出してみるⅣ（後編）</t>
         </is>
       </c>
     </row>
@@ -59805,17 +60842,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第22話-1</t>
+          <t>第153話　ヴィーイ VS. ユリヤ＆テレジア</t>
         </is>
       </c>
     </row>
@@ -59825,17 +60862,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>久遠まこと(著者) 石のやっさん(原作)</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第39話</t>
+          <t>第84話③</t>
         </is>
       </c>
     </row>
@@ -59845,17 +60882,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ダークサモナーとデキている</t>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>車王(著者)</t>
+          <t>モリタ Ｕ４ nima</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第96話</t>
+          <t>第17話（４）　クリスティーナお姉さまの結婚（４）</t>
         </is>
       </c>
     </row>
@@ -59865,17 +60902,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第139話　ひさびさに本気出してみるⅣ（中編）</t>
+          <t>第12話後編</t>
         </is>
       </c>
     </row>
@@ -59885,17 +60922,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+          <t>お前がヤったんだろ！</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+          <t>クシザキ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第41話</t>
+          <t>第18話	たとえあなたが虫になっても</t>
         </is>
       </c>
     </row>
@@ -59905,17 +60942,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>クールな同級生の10年後</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>狛野まこ(著者) 球体X(原作・キャラクター原案) 雨音恵(ノベル原作)</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第1話</t>
+          <t>第6話③</t>
         </is>
       </c>
     </row>
@@ -59925,17 +60962,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>三部べべ(漫画) ねうしとら(原作)</t>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第12話-2</t>
+          <t>第３１食　氷結果実、パクパクですわ！（３）</t>
         </is>
       </c>
     </row>
@@ -59945,17 +60982,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>骸骨騎士様、只今異世界へお出掛け中</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>サワノアキラ（漫画） 秤猿鬼（原作） KeG（キャラクター原案）</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第152話　三主神</t>
+          <t>第69章　連合</t>
         </is>
       </c>
     </row>
@@ -59965,17 +61002,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>魔のものたちは企てる</t>
+          <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>加藤拓弐(原作) ガしガし(作画)</t>
+          <t>クール教信者</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第38話</t>
+          <t>第172話</t>
         </is>
       </c>
     </row>
@@ -59985,17 +61022,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第84話➁</t>
+          <t>第６３話　妖精と出会った器用貧乏（２）</t>
         </is>
       </c>
     </row>
@@ -60005,17 +61042,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>クセ強彼女は床にいざなう</t>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>須河篤志(著者)</t>
+          <t>板垣恵介 林たかあき</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>休載イラスト</t>
+          <t>第76話 不良街道</t>
         </is>
       </c>
     </row>
@@ -60025,17 +61062,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+          <t>転生剣豪ズバババァーン！！</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+          <t>富士田けやき(原作) 坂崎ふれでぃ(作画)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第10話 フェア</t>
+          <t>第4話</t>
         </is>
       </c>
     </row>
@@ -60045,17 +61082,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第6話②</t>
+          <t>第71話①　契約をしてみた</t>
         </is>
       </c>
     </row>
@@ -60065,17 +61102,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+          <t>衛宮さんちの今日のごはん</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+          <t>TAa(漫画) 只野まこと(料理監修) ＴＹＰＥ－ＭＯＯＮ(原作)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>休載イラスト</t>
+          <t>第80話</t>
         </is>
       </c>
     </row>
@@ -60085,17 +61122,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>転生貴族の異世界冒険録 ～自重を知らない神々の使徒～</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>夜州 nini 藻</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第76話（後編）</t>
+          <t>第90話その4</t>
         </is>
       </c>
     </row>
@@ -60105,17 +61142,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第54話 次期侯爵と二次会を②</t>
+          <t>第34話①</t>
         </is>
       </c>
     </row>
@@ -60125,17 +61162,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>島知宏 音速炒飯 有都あらゆる</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第３１食　氷結果実、パクパクですわ！（３）</t>
+          <t>第159話 よくわからないけれど幽霊船に出くわしたみたいです（１）</t>
         </is>
       </c>
     </row>
@@ -60145,17 +61182,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>まったく最近の探偵ときたら</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>五十嵐正邦(著者)</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第118話①</t>
+          <t>第５０話　勇者、神々に封印される・・・いや、マジで！（２）</t>
         </is>
       </c>
     </row>
@@ -60165,17 +61202,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>お前がヤったんだろ！</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>クシザキ</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第17話	佐倉モモカの幸運</t>
+          <t>拷問197</t>
         </is>
       </c>
     </row>
@@ -60185,17 +61222,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ヨウハ(著者)</t>
+          <t>KAKERU</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第4話-1</t>
+          <t>第79話「ケンタウロス2」（後半）</t>
         </is>
       </c>
     </row>
@@ -60205,17 +61242,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>きのした魔法工務店　異世界工法で最強の家づくりを（コミック）</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>漫画／©梃子山ジャンボ 原作／長野文三郎 キャラクター原案／かぼちゃ</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>拷問196</t>
+          <t>第20話(1)</t>
         </is>
       </c>
     </row>
@@ -60225,17 +61262,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+          <t>ライブダンジョン！</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第17話-2：二番弟子</t>
+          <t>第99話前半</t>
         </is>
       </c>
     </row>
@@ -60245,17 +61282,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+          <t>女子高生の無駄づかい</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+          <t>ビーノ(著者)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第50話　奴は土下座する（前編）</t>
+          <t>第148話　けつろん</t>
         </is>
       </c>
     </row>
@@ -60265,17 +61302,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>如意自在(著者)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第６３話　妖精と出会った器用貧乏（１）</t>
+          <t>第4話後半</t>
         </is>
       </c>
     </row>
@@ -60285,17 +61322,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>望まぬ不死の冒険者</t>
+          <t>僕だけの甘くてこわいマネージャーさんたち</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>中曽根ハイジ（漫画） 丘野 優（原作） じゃいあん（キャラクター原案）</t>
+          <t>生瓶鵜義(著者)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第66話　因縁の敵（後編）</t>
+          <t>第１話</t>
         </is>
       </c>
     </row>
@@ -60305,17 +61342,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>異世界ではじめる二拠点生活 ～空間魔法で王都と田舎をいったりきたり～</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>丸山りん(漫画) 錬金王(原作) あんべよしろう(キャラクター原案)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第70話②　あにめを作ってみた</t>
+          <t>第37話</t>
         </is>
       </c>
     </row>
@@ -60325,17 +61362,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>最弱と呼ばれた剣闘士のゲーム知識無双　ー女尊男卑世界のコロシアムで成り上がるー</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>ワタナベタカシ(著者) ケンノジ(原作)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第90話その3</t>
+          <t>第3話</t>
         </is>
       </c>
     </row>
@@ -60345,17 +61382,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
+          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
+          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第4話-②</t>
+          <t>第11話②「かなわないな」</t>
         </is>
       </c>
     </row>
@@ -60365,17 +61402,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>三枝さんはメガネ先輩と恋を描く</t>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>セレビィ量産型(著者)</t>
+          <t>漫画/すたひろ 原作/Y.A</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第29話後半</t>
+          <t>chapter92【48話①】</t>
         </is>
       </c>
     </row>
@@ -60385,17 +61422,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+          <t>空野進 sorani ファルまろ</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第4話-1</t>
+          <t>第23話　最弱貴族、エルフの里へ向かう（３）</t>
         </is>
       </c>
     </row>
@@ -60405,17 +61442,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>黄金の経験値</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>原純(原作) 霜月汐(作画) fixro2n(キャラクター原案)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第５０話　勇者、神々に封印される・・・いや、マジで！（１）</t>
+          <t>第28話</t>
         </is>
       </c>
     </row>
@@ -60435,7 +61472,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第１話　冒険者パーティと開拓します！（２）</t>
+          <t>第２話　レッドドラゴンを倒して開拓します！（１）</t>
         </is>
       </c>
     </row>
@@ -60445,17 +61482,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+          <t>天獄で悪魔がボクを魅惑する</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+          <t>銀河味めてお(著者)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第12話-1</t>
+          <t>第43話</t>
         </is>
       </c>
     </row>
@@ -60465,17 +61502,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>俺は星間国家の悪徳領主！</t>
+          <t>オトナを知りたい女友達</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
+          <t>望公太(原作) ぷよちゃ(作画)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第50話　復讐心の正体</t>
+          <t>第17話 前半</t>
         </is>
       </c>
     </row>
@@ -60485,17 +61522,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>くらいあの子としたいこと</t>
+          <t>オタクに優しいギャルはいない!?</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>碇マナツ(著者)</t>
+          <t>のりしろちゃん 魚住さかな</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第101話</t>
+          <t>【#205】伊地知のバレンタインデー</t>
         </is>
       </c>
     </row>
@@ -60505,17 +61542,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>異世界転生ダンジョンマスター　温泉ダンジョンを作る</t>
+          <t>地味子な三葉さんが僕を誘惑する</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>天原(原作) アルデヒド(作画) じゅん(キャラクター原案)</t>
+          <t>はぶらえる(著者)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第5話</t>
+          <t>第17.5話</t>
         </is>
       </c>
     </row>
@@ -60525,17 +61562,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>バーサス</t>
+          <t>塔の管理をしてみよう</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+          <t>盧恩＆雪笠(Friendly Land)(著者) 早秋(原作) 雨神(キャラクター原案)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第35話　ギンバックVS.大魔班（1）</t>
+          <t>第104話前編</t>
         </is>
       </c>
     </row>
@@ -60545,17 +61582,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
+          <t>世界最高の暗殺者、異世界貴族に転生する</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>FUNA 東西 モトエ恵介</t>
+          <t>月夜涙(原作) 皇ハマオ(漫画) れい亜(キャラクター原案)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第133話 第2回異世界懇談会［その④］</t>
+          <t>第44話-2</t>
         </is>
       </c>
     </row>
@@ -60565,17 +61602,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+          <t>魔法少女リリカルなのは EXCEEDS</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+          <t>都築真紀 川上修一</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>EP.29①</t>
+          <t>番外編③</t>
         </is>
       </c>
     </row>
@@ -60585,17 +61622,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>めっちゃ召喚された件 THE COMIC</t>
+          <t>虚無ねーちゃんはかまってほしい</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>漫画：六甲島カモメ 原作：さいとうさ キャラクター原案：ツグトク</t>
+          <t>観音リツ(著者)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第57話②</t>
+          <t>第6話後半</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-08-31
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -69,6 +69,7 @@
     <sheet name="2026-08-10" sheetId="61" state="visible" r:id="rId61"/>
     <sheet name="2026-08-17" sheetId="62" state="visible" r:id="rId62"/>
     <sheet name="2026-08-24" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet name="2026-08-31" sheetId="64" state="visible" r:id="rId64"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -60637,22 +60638,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>宇崎ちゃんは遊びたい！</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>丈(著者)</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第141話</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>ワンパンマン</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>234撃目</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第41話：「女の先輩」として③</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第158話	我が子の成長！</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第８０話『異教停止』③</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第89話その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第13話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>まんきつしたい常連さん</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>しんみりん(著者)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第58話後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第102話　帰還</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第139話　ひさびさに本気出してみるⅣ（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第153話　ヴィーイ VS. ユリヤ＆テレジア</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第84話③</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>モリタ Ｕ４ nima</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第17話（４）　クリスティーナお姉さまの結婚（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第12話後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>クシザキ</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第18話	たとえあなたが虫になっても</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第6話③</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第３１食　氷結果実、パクパクですわ！（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>骸骨騎士様、只今異世界へお出掛け中</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>サワノアキラ（漫画） 秤猿鬼（原作） KeG（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第69章　連合</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>小林さんちのメイドラゴン</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>クール教信者</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第172話</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第６３話　妖精と出会った器用貧乏（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 林たかあき</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第76話 不良街道</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>転生剣豪ズバババァーン！！</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>富士田けやき(原作) 坂崎ふれでぃ(作画)</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第4話</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第71話①　契約をしてみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>衛宮さんちの今日のごはん</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>TAa(漫画) 只野まこと(料理監修) ＴＹＰＥ－ＭＯＯＮ(原作)</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第80話</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第90話その4</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第34話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第159話 よくわからないけれど幽霊船に出くわしたみたいです（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第５０話　勇者、神々に封印される・・・いや、マジで！（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>拷問197</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>KAKERU</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第79話「ケンタウロス2」（後半）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>きのした魔法工務店　異世界工法で最強の家づくりを（コミック）</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>漫画／©梃子山ジャンボ 原作／長野文三郎 キャラクター原案／かぼちゃ</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第20話(1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>ライブダンジョン！</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第99話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>女子高生の無駄づかい</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>ビーノ(著者)</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第148話　けつろん</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>如意自在(著者)</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第4話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>僕だけの甘くてこわいマネージャーさんたち</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>生瓶鵜義(著者)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第１話</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>異世界ではじめる二拠点生活 ～空間魔法で王都と田舎をいったりきたり～</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>丸山りん(漫画) 錬金王(原作) あんべよしろう(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第37話</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>最弱と呼ばれた剣闘士のゲーム知識無双　ー女尊男卑世界のコロシアムで成り上がるー</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>ワタナベタカシ(著者) ケンノジ(原作)</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第3話</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第11話②「かなわないな」</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>漫画/すたひろ 原作/Y.A</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>chapter92【48話①】</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>空野進 sorani ファルまろ</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第23話　最弱貴族、エルフの里へ向かう（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>黄金の経験値</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>原純(原作) 霜月汐(作画) fixro2n(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第28話</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第２話　レッドドラゴンを倒して開拓します！（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>天獄で悪魔がボクを魅惑する</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>銀河味めてお(著者)</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第43話</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>オトナを知りたい女友達</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>望公太(原作) ぷよちゃ(作画)</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第17話 前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>オタクに優しいギャルはいない!?</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>のりしろちゃん 魚住さかな</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>【#205】伊地知のバレンタインデー</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>地味子な三葉さんが僕を誘惑する</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>はぶらえる(著者)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第17.5話</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>塔の管理をしてみよう</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>盧恩＆雪笠(Friendly Land)(著者) 早秋(原作) 雨神(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第104話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>世界最高の暗殺者、異世界貴族に転生する</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>月夜涙(原作) 皇ハマオ(漫画) れい亜(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第44話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>魔法少女リリカルなのは EXCEEDS</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>都築真紀 川上修一</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>番外編③</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>虚無ねーちゃんはかまってほしい</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>観音リツ(著者)</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第6話後半</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>宇崎ちゃんは遊びたい！</t>
+          <t>異世界おじさん</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>丈(著者)</t>
+          <t>殆ど死んでいる(著者)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第141話</t>
+          <t>第80話</t>
         </is>
       </c>
     </row>
@@ -60662,17 +61699,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ワンパンマン</t>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>原作/ＯＮＥ 作画/村田雄介</t>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>234撃目</t>
+          <t>第82話 前編</t>
         </is>
       </c>
     </row>
@@ -60682,17 +61719,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>zunta(作画) はらわたさいぞう(原作)</t>
+          <t>むちまろ</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第41話：「女の先輩」として③</t>
+          <t>第159話	真幸の敗北！</t>
         </is>
       </c>
     </row>
@@ -60702,17 +61739,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>むちまろ</t>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第158話	我が子の成長！</t>
+          <t>第26話-1「家族を守るために」</t>
         </is>
       </c>
     </row>
@@ -60732,7 +61769,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第８０話『異教停止』③</t>
+          <t>第８０話『異教停止』④</t>
         </is>
       </c>
     </row>
@@ -60742,17 +61779,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+          <t>異世界居酒屋「のぶ」</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第89話その2</t>
+          <t>第134話</t>
         </is>
       </c>
     </row>
@@ -60762,17 +61799,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第13話前半</t>
+          <t>第44話①</t>
         </is>
       </c>
     </row>
@@ -60782,17 +61819,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>まんきつしたい常連さん</t>
+          <t>帰ってください！ 阿久津さん</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>しんみりん(著者)</t>
+          <t>長岡太一(著者)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第58話後編</t>
+          <t>第211話</t>
         </is>
       </c>
     </row>
@@ -60802,17 +61839,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>板垣恵介 猪原賽 陸井栄史</t>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第102話　帰還</t>
+          <t>第9話後編：出立の朝</t>
         </is>
       </c>
     </row>
@@ -60822,17 +61859,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第139話　ひさびさに本気出してみるⅣ（後編）</t>
+          <t>第22話-2</t>
         </is>
       </c>
     </row>
@@ -60842,17 +61879,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>金属スライムを倒しまくった俺が【黒鋼の王】と呼ばれるまで</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>藤屋いずこ(著者) 温泉カピバラ(原作) 山椒魚(キャラクター原案)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第153話　ヴィーイ VS. ユリヤ＆テレジア</t>
+          <t>第21章-2</t>
         </is>
       </c>
     </row>
@@ -60862,17 +61899,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>異世界のんびり農家</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第84話③</t>
+          <t>第330話</t>
         </is>
       </c>
     </row>
@@ -60882,17 +61919,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+          <t>ツンな彼女の太もも事情</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>モリタ Ｕ４ nima</t>
+          <t>新島なるい(著者)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第17話（４）　クリスティーナお姉さまの結婚（４）</t>
+          <t>第1話</t>
         </is>
       </c>
     </row>
@@ -60902,17 +61939,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+          <t>クセ強彼女は床にいざなう</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+          <t>須河篤志(著者)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第12話後編</t>
+          <t>第25話前半</t>
         </is>
       </c>
     </row>
@@ -60922,17 +61959,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>お前がヤったんだろ！</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>クシザキ</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第18話	たとえあなたが虫になっても</t>
+          <t>おまけ76</t>
         </is>
       </c>
     </row>
@@ -60942,17 +61979,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>「おかえり、パパ」</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>蝉丸</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第6話③</t>
+          <t>第38話　プレゼント</t>
         </is>
       </c>
     </row>
@@ -60962,17 +61999,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+          <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>島知宏 音速炒飯 有都あらゆる</t>
+          <t>丈(著者)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第３１食　氷結果実、パクパクですわ！（３）</t>
+          <t>第141話</t>
         </is>
       </c>
     </row>
@@ -60982,17 +62019,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>骸骨騎士様、只今異世界へお出掛け中</t>
+          <t>このヒーラー、めんどくさい</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>サワノアキラ（漫画） 秤猿鬼（原作） KeG（キャラクター原案）</t>
+          <t>丹念に発酵(著者)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第69章　連合</t>
+          <t>「コミックス１０巻発売記念♪　もしもカーラが現代日本でバイトするならどんなお仕事!?」結果発表マンガ</t>
         </is>
       </c>
     </row>
@@ -61002,17 +62039,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>小林さんちのメイドラゴン</t>
+          <t>物語の黒幕に転生して</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>クール教信者</t>
+          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第172話</t>
+          <t>第43話</t>
         </is>
       </c>
     </row>
@@ -61022,17 +62059,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第６３話　妖精と出会った器用貧乏（２）</t>
+          <t>第11話 生きて</t>
         </is>
       </c>
     </row>
@@ -61042,17 +62079,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+          <t>姫ヶ崎櫻子は今日も不憫可愛い</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>板垣恵介 林たかあき</t>
+          <t>安田剛助(著者)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第76話 不良街道</t>
+          <t>第59話</t>
         </is>
       </c>
     </row>
@@ -61062,17 +62099,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>転生剣豪ズバババァーン！！</t>
+          <t>美人女上司滝沢さん</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>富士田けやき(原作) 坂崎ふれでぃ(作画)</t>
+          <t>やんBARU(著者)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第4話</t>
+          <t>第223話</t>
         </is>
       </c>
     </row>
@@ -61082,17 +62119,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>アザミヤコを好きになる</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第71話①　契約をしてみた</t>
+          <t>第17話後編</t>
         </is>
       </c>
     </row>
@@ -61102,17 +62139,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>衛宮さんちの今日のごはん</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>TAa(漫画) 只野まこと(料理監修) ＴＹＰＥ－ＭＯＯＮ(原作)</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第80話</t>
+          <t>第6話④</t>
         </is>
       </c>
     </row>
@@ -61122,17 +62159,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>ぽんドロイド！ はまさん</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>はれやまはれぞう(著者)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第90話その4</t>
+          <t>第24話</t>
         </is>
       </c>
     </row>
@@ -61142,17 +62179,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>女友達は頼めば意外とヤらせてくれる</t>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ろくろ(漫画) 鏡遊(原作)</t>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第34話①</t>
+          <t>第55話 破壊の魔剣①</t>
         </is>
       </c>
     </row>
@@ -61162,17 +62199,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>ヨウハ(著者)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第159話 よくわからないけれど幽霊船に出くわしたみたいです（１）</t>
+          <t>第4話-2</t>
         </is>
       </c>
     </row>
@@ -61182,17 +62219,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第５０話　勇者、神々に封印される・・・いや、マジで！（２）</t>
+          <t>休載イラスト</t>
         </is>
       </c>
     </row>
@@ -61202,17 +62239,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>貞操逆転世界の童貞辺境領主騎士</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>柳瀬こたつ（漫画） 道造（原作） めろん２２（キャラクター原案）</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>拷問197</t>
+          <t>第12話後半　神の館</t>
         </is>
       </c>
     </row>
@@ -61222,17 +62259,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>KAKERU</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第79話「ケンタウロス2」（後半）</t>
+          <t>第６３話　妖精と出会った器用貧乏（３）</t>
         </is>
       </c>
     </row>
@@ -61242,17 +62279,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>きのした魔法工務店　異世界工法で最強の家づくりを（コミック）</t>
+          <t>幼女戦記</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>漫画／©梃子山ジャンボ 原作／長野文三郎 キャラクター原案／かぼちゃ</t>
+          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第20話(1)</t>
+          <t>第百二十章：ドアノッカー作戦Ⅰ</t>
         </is>
       </c>
     </row>
@@ -61262,17 +62299,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ライブダンジョン！</t>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第99話前半</t>
+          <t>第50話　奴は土下座する（後編）</t>
         </is>
       </c>
     </row>
@@ -61282,17 +62319,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>女子高生の無駄づかい</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ビーノ(著者)</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第148話　けつろん</t>
+          <t>第71話②　契約をしてみた</t>
         </is>
       </c>
     </row>
@@ -61312,7 +62349,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第4話後半</t>
+          <t>第5話前半</t>
         </is>
       </c>
     </row>
@@ -61322,17 +62359,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>僕だけの甘くてこわいマネージャーさんたち</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>生瓶鵜義(著者)</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第１話</t>
+          <t>第91話その1</t>
         </is>
       </c>
     </row>
@@ -61342,17 +62379,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>異世界ではじめる二拠点生活 ～空間魔法で王都と田舎をいったりきたり～</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>丸山りん(漫画) 錬金王(原作) あんべよしろう(キャラクター原案)</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第37話</t>
+          <t>第５０話　勇者、神々に封印される・・・いや、マジで！（３）</t>
         </is>
       </c>
     </row>
@@ -61362,17 +62399,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>最弱と呼ばれた剣闘士のゲーム知識無双　ー女尊男卑世界のコロシアムで成り上がるー</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ワタナベタカシ(著者) ケンノジ(原作)</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第3話</t>
+          <t>第159話 よくわからないけれど幽霊船に出くわしたみたいです（２）</t>
         </is>
       </c>
     </row>
@@ -61382,17 +62419,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
+          <t>くらいあの子としたいこと</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
+          <t>碇マナツ(著者)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第11話②「かなわないな」</t>
+          <t>第102話</t>
         </is>
       </c>
     </row>
@@ -61402,17 +62439,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>漫画/すたひろ 原作/Y.A</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>chapter92【48話①】</t>
+          <t>拷問198</t>
         </is>
       </c>
     </row>
@@ -61422,17 +62459,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>空野進 sorani ファルまろ</t>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第23話　最弱貴族、エルフの里へ向かう（３）</t>
+          <t>第12話-2</t>
         </is>
       </c>
     </row>
@@ -61442,17 +62479,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>黄金の経験値</t>
+          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>原純(原作) 霜月汐(作画) fixro2n(キャラクター原案)</t>
+          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第28話</t>
+          <t>第33話</t>
         </is>
       </c>
     </row>
@@ -61462,17 +62499,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
+          <t>バーサス</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第２話　レッドドラゴンを倒して開拓します！（１）</t>
+          <t>第35話　ギンバックVS.大魔班（2）</t>
         </is>
       </c>
     </row>
@@ -61482,17 +62519,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>天獄で悪魔がボクを魅惑する</t>
+          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>銀河味めてお(著者)</t>
+          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第43話</t>
+          <t>第11話-1</t>
         </is>
       </c>
     </row>
@@ -61502,17 +62539,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>オトナを知りたい女友達</t>
+          <t>最弱と呼ばれた剣闘士のゲーム知識無双　ー女尊男卑世界のコロシアムで成り上がるー</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>望公太(原作) ぷよちゃ(作画)</t>
+          <t>ワタナベタカシ(著者) ケンノジ(原作)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第17話 前半</t>
+          <t>第4話</t>
         </is>
       </c>
     </row>
@@ -61522,17 +62559,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>オタクに優しいギャルはいない!?</t>
+          <t>隣の席の聖女様は俺にこっそりスカートの中を教えてくれる</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>のりしろちゃん 魚住さかな</t>
+          <t>しろみね(漫画) 桜木桜（GA文庫）(原作) ただのゆきこ(原作イラスト)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>【#205】伊地知のバレンタインデー</t>
+          <t>第1話</t>
         </is>
       </c>
     </row>
@@ -61542,17 +62579,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>地味子な三葉さんが僕を誘惑する</t>
+          <t>ギャルの自転車を直したら懐かれた</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>はぶらえる(著者)</t>
+          <t>タケチケイ（漫画） 生姜寧也（原作）</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第17.5話</t>
+          <t>第4話　ギャルとのデートが始まった（後編）</t>
         </is>
       </c>
     </row>
@@ -61562,17 +62599,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>塔の管理をしてみよう</t>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>盧恩＆雪笠(Friendly Land)(著者) 早秋(原作) 雨神(キャラクター原案)</t>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第104話前編</t>
+          <t>第4話-2</t>
         </is>
       </c>
     </row>
@@ -61582,17 +62619,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>世界最高の暗殺者、異世界貴族に転生する</t>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>月夜涙(原作) 皇ハマオ(漫画) れい亜(キャラクター原案)</t>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第44話-2</t>
+          <t>第25話②</t>
         </is>
       </c>
     </row>
@@ -61602,17 +62639,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS</t>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>都築真紀 川上修一</t>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>番外編③</t>
+          <t>第8話(2)</t>
         </is>
       </c>
     </row>
@@ -61622,17 +62659,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>虚無ねーちゃんはかまってほしい</t>
+          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>観音リツ(著者)</t>
+          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第6話後半</t>
+          <t>EP.29②</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-09-07
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -70,6 +70,7 @@
     <sheet name="2026-08-17" sheetId="62" state="visible" r:id="rId62"/>
     <sheet name="2026-08-24" sheetId="63" state="visible" r:id="rId63"/>
     <sheet name="2026-08-31" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet name="2026-09-07" sheetId="65" state="visible" r:id="rId65"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -61674,22 +61675,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>異世界おじさん</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>殆ど死んでいる(著者)</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第80話</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第82話 前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第159話	真幸の敗北！</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第26話-1「家族を守るために」</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第８０話『異教停止』④</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>異世界居酒屋「のぶ」</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第134話</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第44話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>帰ってください！ 阿久津さん</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>長岡太一(著者)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第211話</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第9話後編：出立の朝</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第22話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>金属スライムを倒しまくった俺が【黒鋼の王】と呼ばれるまで</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>藤屋いずこ(著者) 温泉カピバラ(原作) 山椒魚(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第21章-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第330話</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>ツンな彼女の太もも事情</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>新島なるい(著者)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第25話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>おまけ76</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>「おかえり、パパ」</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>蝉丸</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第38話　プレゼント</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>宇崎ちゃんは遊びたい！</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>丈(著者)</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第141話</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>このヒーラー、めんどくさい</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>丹念に発酵(著者)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>「コミックス１０巻発売記念♪　もしもカーラが現代日本でバイトするならどんなお仕事!?」結果発表マンガ</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>物語の黒幕に転生して</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第43話</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第11話 生きて</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>姫ヶ崎櫻子は今日も不憫可愛い</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>安田剛助(著者)</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第59話</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>美人女上司滝沢さん</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>やんBARU(著者)</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第223話</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>アザミヤコを好きになる</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第17話後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第6話④</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>ぽんドロイド！ はまさん</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>はれやまはれぞう(著者)</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第24話</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第55話 破壊の魔剣①</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>ヨウハ(著者)</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第4話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>休載イラスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>貞操逆転世界の童貞辺境領主騎士</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>柳瀬こたつ（漫画） 道造（原作） めろん２２（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第12話後半　神の館</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第６３話　妖精と出会った器用貧乏（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>幼女戦記</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第百二十章：ドアノッカー作戦Ⅰ</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第50話　奴は土下座する（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第71話②　契約をしてみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>如意自在(著者)</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第5話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第91話その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第５０話　勇者、神々に封印される・・・いや、マジで！（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第159話 よくわからないけれど幽霊船に出くわしたみたいです（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第102話</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>拷問198</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第12話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第33話</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>バーサス</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第35話　ギンバックVS.大魔班（2）</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第11話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>最弱と呼ばれた剣闘士のゲーム知識無双　ー女尊男卑世界のコロシアムで成り上がるー</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>ワタナベタカシ(著者) ケンノジ(原作)</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第4話</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>隣の席の聖女様は俺にこっそりスカートの中を教えてくれる</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>しろみね(漫画) 桜木桜（GA文庫）(原作) ただのゆきこ(原作イラスト)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>ギャルの自転車を直したら懐かれた</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>タケチケイ（漫画） 生姜寧也（原作）</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第4話　ギャルとのデートが始まった（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第4話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第25話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第8話(2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>EP.29②</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>異世界おじさん</t>
+          <t>ワンパンマン</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>殆ど死んでいる(著者)</t>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第80話</t>
+          <t>235撃目</t>
         </is>
       </c>
     </row>
@@ -61699,17 +62736,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第82話 前編</t>
+          <t>第８１話『炎神停止』①</t>
         </is>
       </c>
     </row>
@@ -61719,17 +62756,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>むちまろ</t>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第159話	真幸の敗北！</t>
+          <t>第26話</t>
         </is>
       </c>
     </row>
@@ -61739,17 +62776,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第26話-1「家族を守るために」</t>
+          <t>第８６話　除霊の戦いが始まった（１）</t>
         </is>
       </c>
     </row>
@@ -61759,17 +62796,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第８０話『異教停止』④</t>
+          <t>第11話 中編</t>
         </is>
       </c>
     </row>
@@ -61779,17 +62816,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>異世界居酒屋「のぶ」</t>
+          <t>王子様の友達</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
+          <t>すけろく(著者)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第134話</t>
+          <t>第40話</t>
         </is>
       </c>
     </row>
@@ -61799,17 +62836,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第44話①</t>
+          <t>第90話その1</t>
         </is>
       </c>
     </row>
@@ -61819,17 +62856,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>帰ってください！ 阿久津さん</t>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>長岡太一(著者)</t>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第211話</t>
+          <t>特別編２</t>
         </is>
       </c>
     </row>
@@ -61839,17 +62876,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+          <t>寿司ガキ</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+          <t>ichika(著者)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第9話後編：出立の朝</t>
+          <t>第12話</t>
         </is>
       </c>
     </row>
@@ -61859,17 +62896,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第22話-2</t>
+          <t>第140話　エリーナ・ルフォリア（前編）</t>
         </is>
       </c>
     </row>
@@ -61879,17 +62916,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>金属スライムを倒しまくった俺が【黒鋼の王】と呼ばれるまで</t>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>藤屋いずこ(著者) 温泉カピバラ(原作) 山椒魚(キャラクター原案)</t>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第21章-2</t>
+          <t>第103話　龍の道(ドラゴン・ロード)</t>
         </is>
       </c>
     </row>
@@ -61899,17 +62936,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>異世界のんびり農家</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第330話</t>
+          <t>第154話　テレジアの真の姿</t>
         </is>
       </c>
     </row>
@@ -61919,17 +62956,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ツンな彼女の太もも事情</t>
+          <t>まんきつしたい常連さん</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>新島なるい(著者)</t>
+          <t>しんみりん(著者)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第1話</t>
+          <t>第59話前編</t>
         </is>
       </c>
     </row>
@@ -61939,17 +62976,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>クセ強彼女は床にいざなう</t>
+          <t>このヒーラー、めんどくさい</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>須河篤志(著者)</t>
+          <t>丹念に発酵(著者)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第25話前半</t>
+          <t>第101話：相性占い</t>
         </is>
       </c>
     </row>
@@ -61959,17 +62996,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>異世界のんびり農家</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>おまけ76</t>
+          <t>第331話</t>
         </is>
       </c>
     </row>
@@ -61979,17 +63016,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>「おかえり、パパ」</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>蝉丸</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第38話　プレゼント</t>
+          <t>第84話④</t>
         </is>
       </c>
     </row>
@@ -61999,17 +63036,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>宇崎ちゃんは遊びたい！</t>
+          <t>田舎で恋は難しい!?</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>丈(著者)</t>
+          <t>ねこうめ(著者)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第141話</t>
+          <t>第10話</t>
         </is>
       </c>
     </row>
@@ -62019,17 +63056,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>このヒーラー、めんどくさい</t>
+          <t>異世界食堂　洋食のねこや</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>丹念に発酵(著者)</t>
+          <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>「コミックス１０巻発売記念♪　もしもカーラが現代日本でバイトするならどんなお仕事!?」結果発表マンガ</t>
+          <t>第49話➁</t>
         </is>
       </c>
     </row>
@@ -62039,17 +63076,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>物語の黒幕に転生して</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第43話</t>
+          <t>第6話⑤</t>
         </is>
       </c>
     </row>
@@ -62059,17 +63096,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第11話 生きて</t>
+          <t>第18話-1：すれ違い</t>
         </is>
       </c>
     </row>
@@ -62079,17 +63116,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>姫ヶ崎櫻子は今日も不憫可愛い</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>安田剛助(著者)</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第59話</t>
+          <t>第６３話　妖精と出会った器用貧乏（４）</t>
         </is>
       </c>
     </row>
@@ -62099,17 +63136,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>美人女上司滝沢さん</t>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>やんBARU(著者)</t>
+          <t>板垣恵介 林たかあき</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第223話</t>
+          <t>第77話 諸刃の剣</t>
         </is>
       </c>
     </row>
@@ -62119,17 +63156,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>アザミヤコを好きになる</t>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第17話後編</t>
+          <t>第34話②</t>
         </is>
       </c>
     </row>
@@ -62139,17 +63176,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>まったく最近の探偵ときたら</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>五十嵐正邦(著者)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第6話④</t>
+          <t>第118話➁</t>
         </is>
       </c>
     </row>
@@ -62159,17 +63196,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ぽんドロイド！ はまさん</t>
+          <t>聖者無双</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>はれやまはれぞう(著者)</t>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第24話</t>
+          <t>おまけ　番外編　十五夜その①</t>
         </is>
       </c>
     </row>
@@ -62179,17 +63216,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第55話 破壊の魔剣①</t>
+          <t>第91話その2</t>
         </is>
       </c>
     </row>
@@ -62199,17 +63236,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+          <t>おとなりのダウナーさんは無理させない</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ヨウハ(著者)</t>
+          <t>瑠璃いろ(著者)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第4話-2</t>
+          <t>第18話</t>
         </is>
       </c>
     </row>
@@ -62219,17 +63256,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>三部べべ(漫画) ねうしとら(原作)</t>
+          <t>原作:剃り残し 漫画:大窪太一</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>休載イラスト</t>
+          <t>第11話(後編)</t>
         </is>
       </c>
     </row>
@@ -62239,17 +63276,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>貞操逆転世界の童貞辺境領主騎士</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>柳瀬こたつ（漫画） 道造（原作） めろん２２（キャラクター原案）</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第12話後半　神の館</t>
+          <t>第５０話　勇者、神々に封印される・・・いや、マジで！（４）</t>
         </is>
       </c>
     </row>
@@ -62259,17 +63296,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第６３話　妖精と出会った器用貧乏（３）</t>
+          <t>第160話 よくわからないけれどスニークインするみたいです（１）</t>
         </is>
       </c>
     </row>
@@ -62279,17 +63316,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>幼女戦記</t>
+          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
+          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第百二十章：ドアノッカー作戦Ⅰ</t>
+          <t>第49話-2</t>
         </is>
       </c>
     </row>
@@ -62299,17 +63336,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第50話　奴は土下座する（後編）</t>
+          <t>拷問199</t>
         </is>
       </c>
     </row>
@@ -62319,17 +63356,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>クール教信者</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第71話②　契約をしてみた</t>
+          <t>第173話</t>
         </is>
       </c>
     </row>
@@ -62339,17 +63376,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
+          <t>インフィニット・デンドログラム</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>如意自在(著者)</t>
+          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第5話前半</t>
+          <t>第81話</t>
         </is>
       </c>
     </row>
@@ -62359,17 +63396,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第91話その1</t>
+          <t>第12話-1：新しい魔法？</t>
         </is>
       </c>
     </row>
@@ -62379,17 +63416,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>如意自在(著者)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第５０話　勇者、神々に封印される・・・いや、マジで！（３）</t>
+          <t>第5話後半</t>
         </is>
       </c>
     </row>
@@ -62399,17 +63436,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第159話 よくわからないけれど幽霊船に出くわしたみたいです（２）</t>
+          <t>第67話　骸の王</t>
         </is>
       </c>
     </row>
@@ -62419,17 +63456,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>くらいあの子としたいこと</t>
+          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>碇マナツ(著者)</t>
+          <t>六志麻あさ 業務用餅 kisui</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第102話</t>
+          <t>第９２話</t>
         </is>
       </c>
     </row>
@@ -62439,17 +63476,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>おせっかい女子、恋をする</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>音竹 ひかる(著者)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>拷問198</t>
+          <t>第31話</t>
         </is>
       </c>
     </row>
@@ -62459,17 +63496,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+          <t>セレビィ量産型(著者)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第12話-2</t>
+          <t>第29.5話</t>
         </is>
       </c>
     </row>
@@ -62479,17 +63516,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
+          <t>雨森潤奈は湿度が高い</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
+          <t>水城水城(原作) 稲鳴四季(作画) 潮崎しの(キャラクター原案)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第33話</t>
+          <t>第4話</t>
         </is>
       </c>
     </row>
@@ -62499,17 +63536,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>バーサス</t>
+          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第35話　ギンバックVS.大魔班（2）</t>
+          <t>第２話　レッドドラゴンを倒して開拓します！（３）</t>
         </is>
       </c>
     </row>
@@ -62519,17 +63556,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>路地裏で拾った女の子がバッドエンド後の乙女ゲームのヒロインだった件</t>
+          <t>回復術士のやり直し</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>カボチャマスク(原作) 樋乃えなが(作画) へいろー(キャラクター原案)</t>
+          <t>月夜涙(原作) 羽賀ソウケン(漫画) しおこんぶ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第11話-1</t>
+          <t>第80話-1</t>
         </is>
       </c>
     </row>
@@ -62539,17 +63576,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>最弱と呼ばれた剣闘士のゲーム知識無双　ー女尊男卑世界のコロシアムで成り上がるー</t>
+          <t>魔法少女リリカルなのは EXCEEDS</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ワタナベタカシ(著者) ケンノジ(原作)</t>
+          <t>都築真紀 川上修一</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第4話</t>
+          <t>第１５話①</t>
         </is>
       </c>
     </row>
@@ -62559,17 +63596,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>隣の席の聖女様は俺にこっそりスカートの中を教えてくれる</t>
+          <t>異世界おじさん</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>しろみね(漫画) 桜木桜（GA文庫）(原作) ただのゆきこ(原作イラスト)</t>
+          <t>殆ど死んでいる(著者)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第1話</t>
+          <t>第80話</t>
         </is>
       </c>
     </row>
@@ -62579,17 +63616,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ギャルの自転車を直したら懐かれた</t>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>タケチケイ（漫画） 生姜寧也（原作）</t>
+          <t>漫画/すたひろ 原作/Y.A</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第4話　ギャルとのデートが始まった（後編）</t>
+          <t>chapter93【48話②】</t>
         </is>
       </c>
     </row>
@@ -62599,17 +63636,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+          <t>空野進 sorani ファルまろ</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第4話-2</t>
+          <t>第24話　最弱貴族、エルフの里の長に謁見する(１)</t>
         </is>
       </c>
     </row>
@@ -62619,17 +63656,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+          <t>オタクに優しいギャルはいない!?</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+          <t>のりしろちゃん 魚住さかな</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第25話②</t>
+          <t>【#207】天音、ふり絞る</t>
         </is>
       </c>
     </row>
@@ -62639,17 +63676,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+          <t>オタくんにだけ優しすぎるアヤメさん</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+          <t>藤田丞(原作) 御影夏(作画)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第8話(2)</t>
+          <t>第2話-1　恋人の実感</t>
         </is>
       </c>
     </row>
@@ -62659,17 +63696,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
+          <t>才女のお世話 高嶺の花だらけな名門校で、学院一のお嬢様（生活能力皆無）を陰ながらお世話することになりました</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
+          <t>漫画：水島空彦 原作：坂石遊作 キャラクター原案：みわべさくら</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>EP.29②</t>
+          <t>第41話</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-09-14
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -71,6 +71,7 @@
     <sheet name="2026-08-24" sheetId="63" state="visible" r:id="rId63"/>
     <sheet name="2026-08-31" sheetId="64" state="visible" r:id="rId64"/>
     <sheet name="2026-09-07" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="2026-09-14" sheetId="66" state="visible" r:id="rId66"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -62711,22 +62712,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>ワンパンマン</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>235撃目</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第８１話『炎神停止』①</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第26話</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第８６話　除霊の戦いが始まった（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第11話 中編</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>王子様の友達</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>すけろく(著者)</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第40話</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第90話その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>特別編２</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>寿司ガキ</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>ichika(著者)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第12話</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第140話　エリーナ・ルフォリア（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第103話　龍の道(ドラゴン・ロード)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第154話　テレジアの真の姿</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>まんきつしたい常連さん</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>しんみりん(著者)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第59話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>このヒーラー、めんどくさい</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>丹念に発酵(著者)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第101話：相性占い</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第331話</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第84話④</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>田舎で恋は難しい!?</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>ねこうめ(著者)</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第10話</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>異世界食堂　洋食のねこや</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第49話➁</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第6話⑤</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第18話-1：すれ違い</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第６３話　妖精と出会った器用貧乏（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 林たかあき</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第77話 諸刃の剣</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第34話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>まったく最近の探偵ときたら</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>五十嵐正邦(著者)</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第118話➁</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>聖者無双</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>おまけ　番外編　十五夜その①</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第91話その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>おとなりのダウナーさんは無理させない</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>瑠璃いろ(著者)</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第18話</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>原作:剃り残し 漫画:大窪太一</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第11話(後編)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第５０話　勇者、神々に封印される・・・いや、マジで！（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第160話 よくわからないけれどスニークインするみたいです（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第49話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>拷問199</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>小林さんちのメイドラゴン</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>クール教信者</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第173話</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>インフィニット・デンドログラム</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第81話</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第12話-1：新しい魔法？</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>如意自在(著者)</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第5話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第67話　骸の王</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>六志麻あさ 業務用餅 kisui</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第９２話</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>おせっかい女子、恋をする</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>音竹 ひかる(著者)</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第31話</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>セレビィ量産型(著者)</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第29.5話</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>雨森潤奈は湿度が高い</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>水城水城(原作) 稲鳴四季(作画) 潮崎しの(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第4話</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第２話　レッドドラゴンを倒して開拓します！（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>回復術士のやり直し</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>月夜涙(原作) 羽賀ソウケン(漫画) しおこんぶ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第80話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>魔法少女リリカルなのは EXCEEDS</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>都築真紀 川上修一</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第１５話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>異世界おじさん</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>殆ど死んでいる(著者)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第80話</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>漫画/すたひろ 原作/Y.A</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>chapter93【48話②】</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>空野進 sorani ファルまろ</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第24話　最弱貴族、エルフの里の長に謁見する(１)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>オタクに優しいギャルはいない!?</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>のりしろちゃん 魚住さかな</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>【#207】天音、ふり絞る</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>オタくんにだけ優しすぎるアヤメさん</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>藤田丞(原作) 御影夏(作画)</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第2話-1　恋人の実感</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>才女のお世話 高嶺の花だらけな名門校で、学院一のお嬢様（生活能力皆無）を陰ながらお世話することになりました</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>漫画：水島空彦 原作：坂石遊作 キャラクター原案：みわべさくら</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第41話</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ワンパンマン</t>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>原作/ＯＮＥ 作画/村田雄介</t>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>235撃目</t>
+          <t>第82話 後編</t>
         </is>
       </c>
     </row>
@@ -62736,17 +63773,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第８１話『炎神停止』①</t>
+          <t>第26話-2「家族を守るために」</t>
         </is>
       </c>
     </row>
@@ -62756,17 +63793,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第26話</t>
+          <t>第８１話『炎神停止』②</t>
         </is>
       </c>
     </row>
@@ -62776,17 +63813,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>不徳のギルド</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>河添太一</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第８６話　除霊の戦いが始まった（１）</t>
+          <t>第１１０話：偉大なる理想</t>
         </is>
       </c>
     </row>
@@ -62796,17 +63833,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+          <t>魔王の俺が奴隷エルフを嫁にしたんだが、どう愛でればいい？</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+          <t>原作／手島史詞 キャラクター原案／COMTA 漫画／板垣ハコ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第11話 中編</t>
+          <t>第82話</t>
         </is>
       </c>
     </row>
@@ -62816,17 +63853,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>王子様の友達</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>すけろく(著者)</t>
+          <t>むちまろ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第40話</t>
+          <t>第160話	照井有栖は遊びたい！</t>
         </is>
       </c>
     </row>
@@ -62836,17 +63873,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第90話その1</t>
+          <t>第８６話　除霊の戦いが始まった（２）</t>
         </is>
       </c>
     </row>
@@ -62856,17 +63893,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+          <t>いとこのこ</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+          <t>いぬちく(著者)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>特別編２</t>
+          <t>コミックス告知</t>
         </is>
       </c>
     </row>
@@ -62876,17 +63913,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>寿司ガキ</t>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ichika(著者)</t>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第12話</t>
+          <t>第10話前編：人間の悪意</t>
         </is>
       </c>
     </row>
@@ -62896,17 +63933,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第140話　エリーナ・ルフォリア（前編）</t>
+          <t>第44話②</t>
         </is>
       </c>
     </row>
@@ -62916,17 +63953,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+          <t>ダンジョンの幼なじみ</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>板垣恵介 猪原賽 陸井栄史</t>
+          <t>久真やすひさ(著者)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第103話　龍の道(ドラゴン・ロード)</t>
+          <t>第68話</t>
         </is>
       </c>
     </row>
@@ -62936,17 +63973,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第154話　テレジアの真の姿</t>
+          <t>第23話-1</t>
         </is>
       </c>
     </row>
@@ -62956,17 +63993,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>まんきつしたい常連さん</t>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>しんみりん(著者)</t>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第59話前編</t>
+          <t>コミックス告知</t>
         </is>
       </c>
     </row>
@@ -62976,17 +64013,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>このヒーラー、めんどくさい</t>
+          <t>異世界のんびり農家</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>丹念に発酵(著者)</t>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第101話：相性占い</t>
+          <t>第332話</t>
         </is>
       </c>
     </row>
@@ -62996,17 +64033,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>異世界のんびり農家</t>
+          <t>クセ強彼女は床にいざなう</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+          <t>須河篤志(著者)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第331話</t>
+          <t>第25話後半</t>
         </is>
       </c>
     </row>
@@ -63016,17 +64053,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第84話④</t>
+          <t>第140話　エリーナ・ルフォリア（中編）</t>
         </is>
       </c>
     </row>
@@ -63036,17 +64073,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>田舎で恋は難しい!?</t>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ねこうめ(著者)</t>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第10話</t>
+          <t>第18話-2</t>
         </is>
       </c>
     </row>
@@ -63056,17 +64093,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>異世界食堂　洋食のねこや</t>
+          <t>魔のものたちは企てる</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
+          <t>加藤拓弐(原作) ガしガし(作画)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第49話➁</t>
+          <t>第39話</t>
         </is>
       </c>
     </row>
@@ -63076,17 +64113,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第6話⑤</t>
+          <t>第85話①</t>
         </is>
       </c>
     </row>
@@ -63096,17 +64133,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第18話-1：すれ違い</t>
+          <t>第155話　帝国との勝敗</t>
         </is>
       </c>
     </row>
@@ -63116,17 +64153,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第６３話　妖精と出会った器用貧乏（４）</t>
+          <t>第12話 セレン</t>
         </is>
       </c>
     </row>
@@ -63136,17 +64173,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>板垣恵介 林たかあき</t>
+          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第77話 諸刃の剣</t>
+          <t>第42話前半</t>
         </is>
       </c>
     </row>
@@ -63156,17 +64193,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>女友達は頼めば意外とヤらせてくれる</t>
+          <t>お前がヤったんだろ！</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ろくろ(漫画) 鏡遊(原作)</t>
+          <t>クシザキ</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第34話②</t>
+          <t>第19話	イニシエーション・ポカ</t>
         </is>
       </c>
     </row>
@@ -63176,17 +64213,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>まったく最近の探偵ときたら</t>
+          <t>美人女上司滝沢さん</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>五十嵐正邦(著者)</t>
+          <t>やんBARU(著者)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第118話➁</t>
+          <t>第224話</t>
         </is>
       </c>
     </row>
@@ -63196,17 +64233,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>聖者無双</t>
+          <t>ぽんドロイド！ はまさん</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+          <t>はれやまはれぞう(著者)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>おまけ　番外編　十五夜その①</t>
+          <t>第25話</t>
         </is>
       </c>
     </row>
@@ -63216,17 +64253,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第91話その2</t>
+          <t>第7話①</t>
         </is>
       </c>
     </row>
@@ -63236,17 +64273,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>おとなりのダウナーさんは無理させない</t>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>瑠璃いろ(著者)</t>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第18話</t>
+          <t>第13話前編</t>
         </is>
       </c>
     </row>
@@ -63256,17 +64293,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>原作:剃り残し 漫画:大窪太一</t>
+          <t>モリタ Ｕ４ nima</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第11話(後編)</t>
+          <t>第17話（５）　クリスティーナお姉さまの結婚（５）</t>
         </is>
       </c>
     </row>
@@ -63276,17 +64313,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>ヨウハ(著者)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第５０話　勇者、神々に封印される・・・いや、マジで！（４）</t>
+          <t>第5話-1</t>
         </is>
       </c>
     </row>
@@ -63296,17 +64333,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第160話 よくわからないけれどスニークインするみたいです（１）</t>
+          <t>第３話　「暁の剣」を雇って開拓します！（１）</t>
         </is>
       </c>
     </row>
@@ -63316,17 +64353,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
+          <t>くらいあの子としたいこと</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
+          <t>碇マナツ(著者)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第49話-2</t>
+          <t>第103話</t>
         </is>
       </c>
     </row>
@@ -63336,17 +64373,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>拷問199</t>
+          <t>第7話</t>
         </is>
       </c>
     </row>
@@ -63356,17 +64393,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>小林さんちのメイドラゴン</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>クール教信者</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第173話</t>
+          <t>第６４話　迷宮の秘密に気付く器用貧乏（１）</t>
         </is>
       </c>
     </row>
@@ -63376,17 +64413,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>インフィニット・デンドログラム</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第81話</t>
+          <t>第91話その3</t>
         </is>
       </c>
     </row>
@@ -63396,17 +64433,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第12話-1：新しい魔法？</t>
+          <t>第5話</t>
         </is>
       </c>
     </row>
@@ -63416,17 +64453,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>如意自在(著者)</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第5話後半</t>
+          <t>第72話①　あにめを公開してみた</t>
         </is>
       </c>
     </row>
@@ -63436,17 +64473,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ハズレ枠の【状態異常スキル】で最強になった俺がすべてを蹂躙するまで</t>
+          <t>異世界黙示録マイノグーラ ～破滅の文明で始める世界征服～</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>鵜吉しょう（作画） 内々けやき（構成） 篠崎 芳（原作） KWKM（キャラクター原案）</t>
+          <t>緑華野菜子(著者) 鹿角フェフ(原作) じゅん(キャラクター原案)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第67話　骸の王</t>
+          <t>第33話　乙女覚醒①</t>
         </is>
       </c>
     </row>
@@ -63456,17 +64493,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
+          <t>理想のヒモ生活</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>六志麻あさ 業務用餅 kisui</t>
+          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第９２話</t>
+          <t>第110話　その2</t>
         </is>
       </c>
     </row>
@@ -63476,17 +64513,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>おせっかい女子、恋をする</t>
+          <t>アザミヤコを好きになる</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>音竹 ひかる(著者)</t>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第31話</t>
+          <t>番外1P漫画②</t>
         </is>
       </c>
     </row>
@@ -63496,17 +64533,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>三枝さんはメガネ先輩と恋を描く</t>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>セレビィ量産型(著者)</t>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第29.5話</t>
+          <t>第51話　奴は合コンに行く（前編）</t>
         </is>
       </c>
     </row>
@@ -63516,17 +64553,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>雨森潤奈は湿度が高い</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>水城水城(原作) 稲鳴四季(作画) 潮崎しの(キャラクター原案)</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第4話</t>
+          <t>第160話 よくわからないけれどスニークインするみたいです（２）</t>
         </is>
       </c>
     </row>
@@ -63536,17 +64573,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第２話　レッドドラゴンを倒して開拓します！（３）</t>
+          <t>第５０話　勇者、神々に封印される・・・いや、マジで！（５）</t>
         </is>
       </c>
     </row>
@@ -63556,17 +64593,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>回復術士のやり直し</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>月夜涙(原作) 羽賀ソウケン(漫画) しおこんぶ(キャラクター原案)</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第80話-1</t>
+          <t>拷問200</t>
         </is>
       </c>
     </row>
@@ -63576,17 +64613,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>魔法少女リリカルなのは EXCEEDS</t>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>都築真紀 川上修一</t>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第１５話①</t>
+          <t>第13話-1</t>
         </is>
       </c>
     </row>
@@ -63596,17 +64633,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>異世界おじさん</t>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>殆ど死んでいる(著者)</t>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第80話</t>
+          <t>コミックス２巻発売！</t>
         </is>
       </c>
     </row>
@@ -63616,17 +64653,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+          <t>「お相手は一般の方です」</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>漫画/すたひろ 原作/Y.A</t>
+          <t>嵯峨祐介(著者)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>chapter93【48話②】</t>
+          <t>第3話後半</t>
         </is>
       </c>
     </row>
@@ -63636,17 +64673,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+          <t>バーサス</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>空野進 sorani ファルまろ</t>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第24話　最弱貴族、エルフの里の長に謁見する(１)</t>
+          <t>第36話　巨影（１）</t>
         </is>
       </c>
     </row>
@@ -63656,17 +64693,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>オタクに優しいギャルはいない!?</t>
+          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>のりしろちゃん 魚住さかな</t>
+          <t>FUNA 東西 モトエ恵介</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>【#207】天音、ふり絞る</t>
+          <t>第134話 攻撃反射作戦［その①］</t>
         </is>
       </c>
     </row>
@@ -63676,17 +64713,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>オタくんにだけ優しすぎるアヤメさん</t>
+          <t>異世界転生ダンジョンマスター　温泉ダンジョンを作る</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>藤田丞(原作) 御影夏(作画)</t>
+          <t>天原(原作) アルデヒド(作画) じゅん(キャラクター原案)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第2話-1　恋人の実感</t>
+          <t>第6話</t>
         </is>
       </c>
     </row>
@@ -63696,17 +64733,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>才女のお世話 高嶺の花だらけな名門校で、学院一のお嬢様（生活能力皆無）を陰ながらお世話することになりました</t>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>漫画：水島空彦 原作：坂石遊作 キャラクター原案：みわべさくら</t>
+          <t>如意自在(著者)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第41話</t>
+          <t>第6話前半</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-09-21
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -72,6 +72,7 @@
     <sheet name="2026-08-31" sheetId="64" state="visible" r:id="rId64"/>
     <sheet name="2026-09-07" sheetId="65" state="visible" r:id="rId65"/>
     <sheet name="2026-09-14" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet name="2026-09-21" sheetId="67" state="visible" r:id="rId67"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -63748,22 +63749,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第82話 後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第26話-2「家族を守るために」</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第８１話『炎神停止』②</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>不徳のギルド</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>河添太一</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第１１０話：偉大なる理想</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>魔王の俺が奴隷エルフを嫁にしたんだが、どう愛でればいい？</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>原作／手島史詞 キャラクター原案／COMTA 漫画／板垣ハコ</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第82話</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第160話	照井有栖は遊びたい！</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第８６話　除霊の戦いが始まった（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>いとこのこ</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>いぬちく(著者)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>コミックス告知</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第10話前編：人間の悪意</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第44話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>ダンジョンの幼なじみ</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>久真やすひさ(著者)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第68話</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第23話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>コミックス告知</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第332話</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第25話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第140話　エリーナ・ルフォリア（中編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第18話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>魔のものたちは企てる</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>加藤拓弐(原作) ガしガし(作画)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第39話</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第85話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第155話　帝国との勝敗</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第12話 セレン</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第42話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>クシザキ</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第19話	イニシエーション・ポカ</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>美人女上司滝沢さん</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>やんBARU(著者)</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第224話</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>ぽんドロイド！ はまさん</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>はれやまはれぞう(著者)</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第25話</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第7話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第13話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>モリタ Ｕ４ nima</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第17話（５）　クリスティーナお姉さまの結婚（５）</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>ヨウハ(著者)</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第5話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第３話　「暁の剣」を雇って開拓します！（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第103話</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第7話</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第６４話　迷宮の秘密に気付く器用貧乏（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第91話その3</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第5話</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第72話①　あにめを公開してみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>異世界黙示録マイノグーラ ～破滅の文明で始める世界征服～</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>緑華野菜子(著者) 鹿角フェフ(原作) じゅん(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第33話　乙女覚醒①</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>理想のヒモ生活</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第110話　その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>アザミヤコを好きになる</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>番外1P漫画②</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第51話　奴は合コンに行く（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第160話 よくわからないけれどスニークインするみたいです（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第５０話　勇者、神々に封印される・・・いや、マジで！（５）</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>拷問200</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第13話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>コミックス２巻発売！</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>「お相手は一般の方です」</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>嵯峨祐介(著者)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第3話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>バーサス</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第36話　巨影（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>FUNA 東西 モトエ恵介</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第134話 攻撃反射作戦［その①］</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>異世界転生ダンジョンマスター　温泉ダンジョンを作る</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>天原(原作) アルデヒド(作画) じゅん(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第6話</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>如意自在(著者)</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第6話前半</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+          <t>ワンパンマン</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第82話 後編</t>
+          <t>236撃目</t>
         </is>
       </c>
     </row>
@@ -63773,17 +64810,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第26話-2「家族を守るために」</t>
+          <t>第８１話『炎神停止』③</t>
         </is>
       </c>
     </row>
@@ -63793,17 +64830,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第８１話『炎神停止』②</t>
+          <t>第90話その2</t>
         </is>
       </c>
     </row>
@@ -63813,17 +64850,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>不徳のギルド</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>河添太一</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第１１０話：偉大なる理想</t>
+          <t>第８７話　ビーチバレーの戦いが始まった（１）</t>
         </is>
       </c>
     </row>
@@ -63833,17 +64870,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>魔王の俺が奴隷エルフを嫁にしたんだが、どう愛でればいい？</t>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>原作／手島史詞 キャラクター原案／COMTA 漫画／板垣ハコ</t>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第82話</t>
+          <t>第13話後半</t>
         </is>
       </c>
     </row>
@@ -63853,17 +64890,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>氷結令嬢さまをフォローしたら、メチャメチャ溺愛されてしまった件@comic</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>むちまろ</t>
+          <t>漫画：ハレノチアメ 原作：愛坂タカト キャラクター原案：Bcoca</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第160話	照井有栖は遊びたい！</t>
+          <t>アリシア様セクシーショット集2（担当編集厳選）</t>
         </is>
       </c>
     </row>
@@ -63873,17 +64910,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第８６話　除霊の戦いが始まった（２）</t>
+          <t>第140話　エリーナ・ルフォリア（後編）</t>
         </is>
       </c>
     </row>
@@ -63893,17 +64930,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>いとこのこ</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>いぬちく(著者)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>コミックス告知</t>
+          <t>第156話　戴冠式・前編</t>
         </is>
       </c>
     </row>
@@ -63913,17 +64950,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+          <t>まんきつしたい常連さん</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+          <t>しんみりん(著者)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第10話前編：人間の悪意</t>
+          <t>第59話後編</t>
         </is>
       </c>
     </row>
@@ -63933,17 +64970,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第44話②</t>
+          <t>第104話　番人</t>
         </is>
       </c>
     </row>
@@ -63953,17 +64990,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ダンジョンの幼なじみ</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>久真やすひさ(著者)</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第68話</t>
+          <t>第85話➁</t>
         </is>
       </c>
     </row>
@@ -63973,17 +65010,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+          <t>ダークサモナーとデキている</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+          <t>車王(著者)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第23話-1</t>
+          <t>第97話</t>
         </is>
       </c>
     </row>
@@ -63993,17 +65030,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>zunta(作画) はらわたさいぞう(原作)</t>
+          <t>久遠まこと(著者) 石のやっさん(原作)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>コミックス告知</t>
+          <t>第40話</t>
         </is>
       </c>
     </row>
@@ -64023,7 +65060,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第332話</t>
+          <t>第333話</t>
         </is>
       </c>
     </row>
@@ -64033,17 +65070,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>クセ強彼女は床にいざなう</t>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>須河篤志(著者)</t>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第25話後半</t>
+          <t>第３２食　エリクサー、ゴクゴクですわ！（前編）（２）</t>
         </is>
       </c>
     </row>
@@ -64053,17 +65090,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第140話　エリーナ・ルフォリア（中編）</t>
+          <t>第48話-2</t>
         </is>
       </c>
     </row>
@@ -64073,17 +65110,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第18話-2</t>
+          <t>第7話②</t>
         </is>
       </c>
     </row>
@@ -64093,17 +65130,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>魔のものたちは企てる</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>加藤拓弐(原作) ガしガし(作画)</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第39話</t>
+          <t>第６４話　迷宮の秘密に気付く器用貧乏（２）</t>
         </is>
       </c>
     </row>
@@ -64113,17 +65150,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第85話①</t>
+          <t>第55話 破壊の魔剣②</t>
         </is>
       </c>
     </row>
@@ -64133,17 +65170,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>板垣恵介 林たかあき</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第155話　帝国との勝敗</t>
+          <t>第78話 箸使い</t>
         </is>
       </c>
     </row>
@@ -64153,17 +65190,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+          <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+          <t>クール教信者</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第12話 セレン</t>
+          <t>第174話</t>
         </is>
       </c>
     </row>
@@ -64173,17 +65210,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第42話前半</t>
+          <t>第18話-2：すれ違い</t>
         </is>
       </c>
     </row>
@@ -64193,17 +65230,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>お前がヤったんだろ！</t>
+          <t>まったく最近の探偵ときたら</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>クシザキ</t>
+          <t>五十嵐正邦(著者)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第19話	イニシエーション・ポカ</t>
+          <t>第119話</t>
         </is>
       </c>
     </row>
@@ -64213,17 +65250,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>美人女上司滝沢さん</t>
+          <t>オタくんにだけ優しすぎるアヤメさん</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>やんBARU(著者)</t>
+          <t>藤田丞(原作) 御影夏(作画)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第224話</t>
+          <t>第2話-2　恋人の実感</t>
         </is>
       </c>
     </row>
@@ -64233,17 +65270,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ぽんドロイド！ はまさん</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>はれやまはれぞう(著者)</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第25話</t>
+          <t>第72話②　あにめを公開してみた</t>
         </is>
       </c>
     </row>
@@ -64253,17 +65290,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第7話①</t>
+          <t>第161話 よくわからないけれどマウンティングされたみたいです（１）</t>
         </is>
       </c>
     </row>
@@ -64273,17 +65310,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第13話前編</t>
+          <t>第３話　「暁の剣」を雇って開拓します！（２）</t>
         </is>
       </c>
     </row>
@@ -64293,17 +65330,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+          <t>聖者無双</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>モリタ Ｕ４ nima</t>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第17話（５）　クリスティーナお姉さまの結婚（５）</t>
+          <t>おまけ　番外編　十五夜その②</t>
         </is>
       </c>
     </row>
@@ -64313,17 +65350,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ヨウハ(著者)</t>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第5話-1</t>
+          <t>第35話①</t>
         </is>
       </c>
     </row>
@@ -64333,17 +65370,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
+          <t>俺は星間国家の悪徳領主！</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
+          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第３話　「暁の剣」を雇って開拓します！（１）</t>
+          <t>第51話　懐かしの故郷</t>
         </is>
       </c>
     </row>
@@ -64353,17 +65390,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>くらいあの子としたいこと</t>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>碇マナツ(著者)</t>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第103話</t>
+          <t>第12話-2：新しい魔法？</t>
         </is>
       </c>
     </row>
@@ -64373,17 +65410,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第7話</t>
+          <t>第9話(1)</t>
         </is>
       </c>
     </row>
@@ -64393,17 +65430,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第６４話　迷宮の秘密に気付く器用貧乏（１）</t>
+          <t>拷問201</t>
         </is>
       </c>
     </row>
@@ -64413,17 +65450,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>異世界黙示録マイノグーラ ～破滅の文明で始める世界征服～</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>緑華野菜子(著者) 鹿角フェフ(原作) じゅん(キャラクター原案)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第91話その3</t>
+          <t>第33話　乙女覚醒②</t>
         </is>
       </c>
     </row>
@@ -64433,17 +65470,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
+          <t>如意自在(著者)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第5話</t>
+          <t>第6話後半</t>
         </is>
       </c>
     </row>
@@ -64453,17 +65490,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>世界最強の後衛 ～迷宮国の新人探索者～</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>力蔵(著者) とーわ(原作) 風花風花(キャラクター原案)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第72話①　あにめを公開してみた</t>
+          <t>第45話-2</t>
         </is>
       </c>
     </row>
@@ -64473,17 +65510,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>異世界黙示録マイノグーラ ～破滅の文明で始める世界征服～</t>
+          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>緑華野菜子(著者) 鹿角フェフ(原作) じゅん(キャラクター原案)</t>
+          <t>六志麻あさ 業務用餅 kisui</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第33話　乙女覚醒①</t>
+          <t>第９３話</t>
         </is>
       </c>
     </row>
@@ -64493,17 +65530,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>理想のヒモ生活</t>
+          <t>死亡エンドを回避したギャルゲーのヒロインたちが俺の【日記帳】を読んで秘密を知ったらしい</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
+          <t>addict(原作) となりける(作画) へいろー(キャラクター原案)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第110話　その2</t>
+          <t>第1話</t>
         </is>
       </c>
     </row>
@@ -64513,17 +65550,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>アザミヤコを好きになる</t>
+          <t>美容スキルでクラスの女の子を可愛くしたい</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ユニティコング(原作) ツノニガウ(作画)</t>
+          <t>藤白ぺるか(原作) 紺野あずれ(漫画) 水野早桜(キャラクター原案)</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>番外1P漫画②</t>
+          <t>第11話</t>
         </is>
       </c>
     </row>
@@ -64533,17 +65570,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+          <t>異世界でも無難に生きたい症候群</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+          <t>原作：安泰（一二三書房刊） 漫画：笹峰コウ キャラクター原案：ひたきゆう</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第51話　奴は合コンに行く（前編）</t>
+          <t>第38話①</t>
         </is>
       </c>
     </row>
@@ -64553,17 +65590,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>おせっかい女子、恋をする</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>音竹 ひかる(著者)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第160話 よくわからないけれどスニークインするみたいです（２）</t>
+          <t>第33話</t>
         </is>
       </c>
     </row>
@@ -64573,17 +65610,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>女子高生の無駄づかい</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>ビーノ(著者)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第５０話　勇者、神々に封印される・・・いや、マジで！（５）</t>
+          <t>第149話　でんせつ</t>
         </is>
       </c>
     </row>
@@ -64593,17 +65630,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>漫画/すたひろ 原作/Y.A</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>拷問200</t>
+          <t>chapter94【49話①】</t>
         </is>
       </c>
     </row>
@@ -64613,17 +65650,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+          <t>ミタメトウラハラ</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+          <t>ウラベスナヒト</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第13話-1</t>
+          <t>#15世話</t>
         </is>
       </c>
     </row>
@@ -64633,17 +65670,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+          <t>ひとりぼっちの異世界攻略</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>三部べべ(漫画) ねうしとら(原作)</t>
+          <t>びび（漫画） 五示正司（原作）</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>コミックス２巻発売！</t>
+          <t>第288話　至高の甲冑</t>
         </is>
       </c>
     </row>
@@ -64653,17 +65690,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>「お相手は一般の方です」</t>
+          <t>ツンな彼女の太もも事情</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>嵯峨祐介(著者)</t>
+          <t>新島なるい(著者)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第3話後半</t>
+          <t>第4話</t>
         </is>
       </c>
     </row>
@@ -64673,17 +65710,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>バーサス</t>
+          <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+          <t>昼行燈（原作） しいたけ元帥（漫画）</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第36話　巨影（１）</t>
+          <t>第52話(前半）</t>
         </is>
       </c>
     </row>
@@ -64693,17 +65730,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
+          <t>めっちゃ召喚された件 THE COMIC</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>FUNA 東西 モトエ恵介</t>
+          <t>漫画：六甲島カモメ 原作：さいとうさ キャラクター原案：ツグトク</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第134話 攻撃反射作戦［その①］</t>
+          <t>第58話②</t>
         </is>
       </c>
     </row>
@@ -64713,17 +65750,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>異世界転生ダンジョンマスター　温泉ダンジョンを作る</t>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>天原(原作) アルデヒド(作画) じゅん(キャラクター原案)</t>
+          <t>空野進 sorani ファルまろ</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第6話</t>
+          <t>第24話　最弱貴族、エルフの里の長に謁見する(３)</t>
         </is>
       </c>
     </row>
@@ -64733,17 +65770,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
+          <t>Lv２からチートだった元勇者候補のまったり異世界ライフ</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>如意自在(著者)</t>
+          <t>糸町秋音（漫画） 鬼ノ城ミヤ（原作） 片桐（キャラクター原案）</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第6話前半</t>
+          <t>第71話　憂慮（前編）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-09-28
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -73,6 +73,7 @@
     <sheet name="2026-09-07" sheetId="65" state="visible" r:id="rId65"/>
     <sheet name="2026-09-14" sheetId="66" state="visible" r:id="rId66"/>
     <sheet name="2026-09-21" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet name="2026-09-28" sheetId="68" state="visible" r:id="rId68"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -64785,22 +64786,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>ワンパンマン</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>236撃目</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第８１話『炎神停止』③</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第90話その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第８７話　ビーチバレーの戦いが始まった（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第13話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>氷結令嬢さまをフォローしたら、メチャメチャ溺愛されてしまった件@comic</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>漫画：ハレノチアメ 原作：愛坂タカト キャラクター原案：Bcoca</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>アリシア様セクシーショット集2（担当編集厳選）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第140話　エリーナ・ルフォリア（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第156話　戴冠式・前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>まんきつしたい常連さん</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>しんみりん(著者)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第59話後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第104話　番人</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第85話➁</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>ダークサモナーとデキている</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>車王(著者)</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第97話</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>久遠まこと(著者) 石のやっさん(原作)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第40話</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第333話</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第３２食　エリクサー、ゴクゴクですわ！（前編）（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第48話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第7話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第６４話　迷宮の秘密に気付く器用貧乏（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第55話 破壊の魔剣②</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 林たかあき</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第78話 箸使い</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>小林さんちのメイドラゴン</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>クール教信者</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第174話</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第18話-2：すれ違い</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>まったく最近の探偵ときたら</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>五十嵐正邦(著者)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第119話</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>オタくんにだけ優しすぎるアヤメさん</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>藤田丞(原作) 御影夏(作画)</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第2話-2　恋人の実感</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第72話②　あにめを公開してみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第161話 よくわからないけれどマウンティングされたみたいです（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第３話　「暁の剣」を雇って開拓します！（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>聖者無双</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>おまけ　番外編　十五夜その②</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第35話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>俺は星間国家の悪徳領主！</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第51話　懐かしの故郷</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第12話-2：新しい魔法？</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第9話(1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>拷問201</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>異世界黙示録マイノグーラ ～破滅の文明で始める世界征服～</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>緑華野菜子(著者) 鹿角フェフ(原作) じゅん(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第33話　乙女覚醒②</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>如意自在(著者)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第6話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の後衛 ～迷宮国の新人探索者～</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>力蔵(著者) とーわ(原作) 風花風花(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第45話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>六志麻あさ 業務用餅 kisui</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第９３話</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>死亡エンドを回避したギャルゲーのヒロインたちが俺の【日記帳】を読んで秘密を知ったらしい</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>addict(原作) となりける(作画) へいろー(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>美容スキルでクラスの女の子を可愛くしたい</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>藤白ぺるか(原作) 紺野あずれ(漫画) 水野早桜(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第11話</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>異世界でも無難に生きたい症候群</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>原作：安泰（一二三書房刊） 漫画：笹峰コウ キャラクター原案：ひたきゆう</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第38話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>おせっかい女子、恋をする</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>音竹 ひかる(著者)</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第33話</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>女子高生の無駄づかい</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>ビーノ(著者)</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第149話　でんせつ</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>漫画/すたひろ 原作/Y.A</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>chapter94【49話①】</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>ミタメトウラハラ</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>ウラベスナヒト</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>#15世話</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>ひとりぼっちの異世界攻略</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>びび（漫画） 五示正司（原作）</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第288話　至高の甲冑</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>ツンな彼女の太もも事情</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>新島なるい(著者)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第4話</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>昼行燈（原作） しいたけ元帥（漫画）</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第52話(前半）</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>めっちゃ召喚された件 THE COMIC</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>漫画：六甲島カモメ 原作：さいとうさ キャラクター原案：ツグトク</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第58話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>空野進 sorani ファルまろ</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第24話　最弱貴族、エルフの里の長に謁見する(３)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>Lv２からチートだった元勇者候補のまったり異世界ライフ</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>糸町秋音（漫画） 鬼ノ城ミヤ（原作） 片桐（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第71話　憂慮（前編）</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ワンパンマン</t>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>原作/ＯＮＥ 作画/村田雄介</t>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>236撃目</t>
+          <t>第83話 前編</t>
         </is>
       </c>
     </row>
@@ -64810,17 +65847,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>むちまろ</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第８１話『炎神停止』③</t>
+          <t>第161話	有栖しくじる！（前編）</t>
         </is>
       </c>
     </row>
@@ -64830,17 +65867,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第90話その2</t>
+          <t>第27話-1「共闘」</t>
         </is>
       </c>
     </row>
@@ -64850,17 +65887,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第８７話　ビーチバレーの戦いが始まった（１）</t>
+          <t>第８１話『炎神停止』④</t>
         </is>
       </c>
     </row>
@@ -64870,17 +65907,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第13話後半</t>
+          <t>第11話 後編</t>
         </is>
       </c>
     </row>
@@ -64890,17 +65927,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>氷結令嬢さまをフォローしたら、メチャメチャ溺愛されてしまった件@comic</t>
+          <t>魔術師クノンは見えている</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>漫画：ハレノチアメ 原作：愛坂タカト キャラクター原案：Bcoca</t>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>アリシア様セクシーショット集2（担当編集厳選）</t>
+          <t>第51話①</t>
         </is>
       </c>
     </row>
@@ -64910,17 +65947,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第140話　エリーナ・ルフォリア（後編）</t>
+          <t>第10話後編：人間の悪意</t>
         </is>
       </c>
     </row>
@@ -64930,17 +65967,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第156話　戴冠式・前編</t>
+          <t>第８７話　ビーチバレーの戦いが始まった（２）</t>
         </is>
       </c>
     </row>
@@ -64950,17 +65987,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>まんきつしたい常連さん</t>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>しんみりん(著者)</t>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第59話後編</t>
+          <t>第45話①</t>
         </is>
       </c>
     </row>
@@ -64970,17 +66007,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>板垣恵介 猪原賽 陸井栄史</t>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第104話　番人</t>
+          <t>第23話-2</t>
         </is>
       </c>
     </row>
@@ -65000,7 +66037,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第85話➁</t>
+          <t>第85話③</t>
         </is>
       </c>
     </row>
@@ -65010,17 +66047,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ダークサモナーとデキている</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>車王(著者)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第97話</t>
+          <t>第156話　戴冠式・後編</t>
         </is>
       </c>
     </row>
@@ -65030,17 +66067,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>久遠まこと(著者) 石のやっさん(原作)</t>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第40話</t>
+          <t>第13話-1</t>
         </is>
       </c>
     </row>
@@ -65050,17 +66087,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>異世界のんびり農家</t>
+          <t>氷結令嬢さまをフォローしたら、メチャメチャ溺愛されてしまった件@comic</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+          <t>漫画：ハレノチアメ 原作：愛坂タカト キャラクター原案：Bcoca</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第333話</t>
+          <t>第15話</t>
         </is>
       </c>
     </row>
@@ -65070,17 +66107,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+          <t>お前がヤったんだろ！</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>島知宏 音速炒飯 有都あらゆる</t>
+          <t>クシザキ</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第３２食　エリクサー、ゴクゴクですわ！（前編）（２）</t>
+          <t>第20話	絆創膏の正しい使い方</t>
         </is>
       </c>
     </row>
@@ -65090,17 +66127,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
+          <t>隣の席の聖女様は俺にこっそりスカートの中を教えてくれる</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
+          <t>しろみね(漫画) 桜木桜（GA文庫）(原作) ただのゆきこ(原作イラスト)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第48話-2</t>
+          <t>第2話</t>
         </is>
       </c>
     </row>
@@ -65110,17 +66147,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第7話②</t>
+          <t>第13話 おむすび</t>
         </is>
       </c>
     </row>
@@ -65130,17 +66167,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第６４話　迷宮の秘密に気付く器用貧乏（２）</t>
+          <t>第7話③</t>
         </is>
       </c>
     </row>
@@ -65150,17 +66187,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+          <t>物語の黒幕に転生して</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第55話 破壊の魔剣②</t>
+          <t>第44話</t>
         </is>
       </c>
     </row>
@@ -65170,17 +66207,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>板垣恵介 林たかあき</t>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第78話 箸使い</t>
+          <t>第３２食　エリクサー、ゴクゴクですわ！（前編）（３）</t>
         </is>
       </c>
     </row>
@@ -65190,17 +66227,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>小林さんちのメイドラゴン</t>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>クール教信者</t>
+          <t>モリタ Ｕ４ nima</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第174話</t>
+          <t>第18話（１）　メイド大集結でお祝い！結婚披露宴（１）</t>
         </is>
       </c>
     </row>
@@ -65210,17 +66247,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第18話-2：すれ違い</t>
+          <t>第13話後編</t>
         </is>
       </c>
     </row>
@@ -65230,17 +66267,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>まったく最近の探偵ときたら</t>
+          <t>美人女上司滝沢さん</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>五十嵐正邦(著者)</t>
+          <t>やんBARU(著者)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第119話</t>
+          <t>第225話</t>
         </is>
       </c>
     </row>
@@ -65250,17 +66287,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>オタくんにだけ優しすぎるアヤメさん</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>藤田丞(原作) 御影夏(作画)</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第2話-2　恋人の実感</t>
+          <t>第６４話　迷宮の秘密に気付く器用貧乏（３）</t>
         </is>
       </c>
     </row>
@@ -65270,17 +66307,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>幼女戦記</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第72話②　あにめを公開してみた</t>
+          <t>第百二十一章：ドアノッカー作戦Ⅱ</t>
         </is>
       </c>
     </row>
@@ -65290,17 +66327,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第161話 よくわからないけれどマウンティングされたみたいです（１）</t>
+          <t>第92話その1</t>
         </is>
       </c>
     </row>
@@ -65310,17 +66347,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
+          <t>バーサス</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第３話　「暁の剣」を雇って開拓します！（２）</t>
+          <t>第36話　巨影（２）</t>
         </is>
       </c>
     </row>
@@ -65330,17 +66367,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>聖者無双</t>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>漫画：秋風緋色 原作：ブロッコリーライオン キャラクター原案：sime</t>
+          <t>ヨウハ(著者)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>おまけ　番外編　十五夜その②</t>
+          <t>第5話-2</t>
         </is>
       </c>
     </row>
@@ -65350,17 +66387,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>女友達は頼めば意外とヤらせてくれる</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ろくろ(漫画) 鏡遊(原作)</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第35話①</t>
+          <t>第５１話　勇者、完全に封印されて宇宙の彼方へ捨てられてしまう（１）</t>
         </is>
       </c>
     </row>
@@ -65370,17 +66407,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>俺は星間国家の悪徳領主！</t>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>灘島かい（漫画） 三嶋与夢（原作） 高峰ナダレ（キャラクター原案）</t>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第51話　懐かしの故郷</t>
+          <t>第51話　奴は合コンに行く（後編）</t>
         </is>
       </c>
     </row>
@@ -65390,17 +66427,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第12話-2：新しい魔法？</t>
+          <t>第３話　「暁の剣」を雇って開拓します！（３）</t>
         </is>
       </c>
     </row>
@@ -65410,17 +66447,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第9話(1)</t>
+          <t>拷問202</t>
         </is>
       </c>
     </row>
@@ -65430,17 +66467,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>拷問201</t>
+          <t>第161話 よくわからないけれどマウンティングされたみたいです（２）</t>
         </is>
       </c>
     </row>
@@ -65450,17 +66487,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>異世界黙示録マイノグーラ ～破滅の文明で始める世界征服～</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>緑華野菜子(著者) 鹿角フェフ(原作) じゅん(キャラクター原案)</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第33話　乙女覚醒②</t>
+          <t>第73話①　こみけのためにかけ回ってみた</t>
         </is>
       </c>
     </row>
@@ -65470,17 +66507,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>如意自在(著者)</t>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第6話後半</t>
+          <t>第13話-2</t>
         </is>
       </c>
     </row>
@@ -65490,17 +66527,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>世界最強の後衛 ～迷宮国の新人探索者～</t>
+          <t>くらいあの子としたいこと</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>力蔵(著者) とーわ(原作) 風花風花(キャラクター原案)</t>
+          <t>碇マナツ(著者)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第45話-2</t>
+          <t>第104話</t>
         </is>
       </c>
     </row>
@@ -65510,17 +66547,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>六志麻あさ 業務用餅 kisui</t>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第９３話</t>
+          <t>第9話(2)</t>
         </is>
       </c>
     </row>
@@ -65530,17 +66567,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>死亡エンドを回避したギャルゲーのヒロインたちが俺の【日記帳】を読んで秘密を知ったらしい</t>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>addict(原作) となりける(作画) へいろー(キャラクター原案)</t>
+          <t>如意自在(著者)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第1話</t>
+          <t>番外編</t>
         </is>
       </c>
     </row>
@@ -65550,17 +66587,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>美容スキルでクラスの女の子を可愛くしたい</t>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>藤白ぺるか(原作) 紺野あずれ(漫画) 水野早桜(キャラクター原案)</t>
+          <t>KAKERU</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第11話</t>
+          <t>第80話「知らんとこでえらいことなっとる」（後半）</t>
         </is>
       </c>
     </row>
@@ -65570,17 +66607,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>異世界でも無難に生きたい症候群</t>
+          <t>ライブダンジョン！</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>原作：安泰（一二三書房刊） 漫画：笹峰コウ キャラクター原案：ひたきゆう</t>
+          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第38話①</t>
+          <t>第100話前半</t>
         </is>
       </c>
     </row>
@@ -65590,17 +66627,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>おせっかい女子、恋をする</t>
+          <t>異世界「嘘」ガイド</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>音竹 ひかる(著者)</t>
+          <t>辻島もと(著者)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第33話</t>
+          <t>第5話</t>
         </is>
       </c>
     </row>
@@ -65610,17 +66647,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>女子高生の無駄づかい</t>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ビーノ(著者)</t>
+          <t>はぐはぐ(著者)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第149話　でんせつ</t>
+          <t>第103話</t>
         </is>
       </c>
     </row>
@@ -65630,17 +66667,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>婚約者に裏切られた錬金術師は、独立して『ざまぁ』します　コミック版</t>
+          <t>転生剣豪ズバババァーン！！</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>漫画/すたひろ 原作/Y.A</t>
+          <t>富士田けやき(原作) 坂崎ふれでぃ(作画)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>chapter94【49話①】</t>
+          <t>番外編</t>
         </is>
       </c>
     </row>
@@ -65650,17 +66687,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ミタメトウラハラ</t>
+          <t>となりのエルフがだらしない！</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ウラベスナヒト</t>
+          <t>もゆる(著者)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>#15世話</t>
+          <t>第1話</t>
         </is>
       </c>
     </row>
@@ -65670,17 +66707,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ひとりぼっちの異世界攻略</t>
+          <t>塔の管理をしてみよう</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>びび（漫画） 五示正司（原作）</t>
+          <t>盧恩＆雪笠(Friendly Land)(著者) 早秋(原作) 雨神(キャラクター原案)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第288話　至高の甲冑</t>
+          <t>第105話前編</t>
         </is>
       </c>
     </row>
@@ -65690,17 +66727,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ツンな彼女の太もも事情</t>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>新島なるい(著者)</t>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第4話</t>
+          <t>第25話④</t>
         </is>
       </c>
     </row>
@@ -65710,17 +66747,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
+          <t>ギャルの自転車を直したら懐かれた</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>昼行燈（原作） しいたけ元帥（漫画）</t>
+          <t>タケチケイ（漫画） 生姜寧也（原作）</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第52話(前半）</t>
+          <t>第5話　ギャルにだって悩むこともある（後編）</t>
         </is>
       </c>
     </row>
@@ -65730,17 +66767,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>めっちゃ召喚された件 THE COMIC</t>
+          <t>回復術士のやり直し</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>漫画：六甲島カモメ 原作：さいとうさ キャラクター原案：ツグトク</t>
+          <t>月夜涙(原作) 羽賀ソウケン(漫画) しおこんぶ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第58話②</t>
+          <t>第80話-2</t>
         </is>
       </c>
     </row>
@@ -65750,17 +66787,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+          <t>最弱と呼ばれた剣闘士のゲーム知識無双　ー女尊男卑世界のコロシアムで成り上がるー</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>空野進 sorani ファルまろ</t>
+          <t>ワタナベタカシ(著者) ケンノジ(原作)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第24話　最弱貴族、エルフの里の長に謁見する(３)</t>
+          <t>第6話</t>
         </is>
       </c>
     </row>
@@ -65770,17 +66807,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Lv２からチートだった元勇者候補のまったり異世界ライフ</t>
+          <t>追放僧侶の賢者タイム</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>糸町秋音（漫画） 鬼ノ城ミヤ（原作） 片桐（キャラクター原案）</t>
+          <t>原作・野原のはて 作画・鈴木シオン</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第71話　憂慮（前編）</t>
+          <t>第12話　封印空間</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-10-05
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -74,6 +74,7 @@
     <sheet name="2026-09-14" sheetId="66" state="visible" r:id="rId66"/>
     <sheet name="2026-09-21" sheetId="67" state="visible" r:id="rId67"/>
     <sheet name="2026-09-28" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet name="2026-10-05" sheetId="69" state="visible" r:id="rId69"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -65822,22 +65823,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第83話 前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>第161話	有栖しくじる！（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第27話-1「共闘」</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第８１話『炎神停止』④</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第11話 後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>魔術師クノンは見えている</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第51話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第10話後編：人間の悪意</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第８７話　ビーチバレーの戦いが始まった（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第45話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第23話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第85話③</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第156話　戴冠式・後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第13話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>氷結令嬢さまをフォローしたら、メチャメチャ溺愛されてしまった件@comic</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>漫画：ハレノチアメ 原作：愛坂タカト キャラクター原案：Bcoca</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第15話</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>クシザキ</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第20話	絆創膏の正しい使い方</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>隣の席の聖女様は俺にこっそりスカートの中を教えてくれる</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>しろみね(漫画) 桜木桜（GA文庫）(原作) ただのゆきこ(原作イラスト)</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第2話</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第13話 おむすび</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第7話③</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>物語の黒幕に転生して</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第44話</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第３２食　エリクサー、ゴクゴクですわ！（前編）（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>モリタ Ｕ４ nima</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第18話（１）　メイド大集結でお祝い！結婚披露宴（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第13話後編</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>美人女上司滝沢さん</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>やんBARU(著者)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第225話</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第６４話　迷宮の秘密に気付く器用貧乏（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>幼女戦記</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第百二十一章：ドアノッカー作戦Ⅱ</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第92話その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>バーサス</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第36話　巨影（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>ヨウハ(著者)</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第5話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第５１話　勇者、完全に封印されて宇宙の彼方へ捨てられてしまう（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第51話　奴は合コンに行く（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第３話　「暁の剣」を雇って開拓します！（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>拷問202</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第161話 よくわからないけれどマウンティングされたみたいです（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第73話①　こみけのためにかけ回ってみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第13話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第104話</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第9話(2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>如意自在(著者)</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>番外編</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>KAKERU</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第80話「知らんとこでえらいことなっとる」（後半）</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>ライブダンジョン！</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第100話前半</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>異世界「嘘」ガイド</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>辻島もと(著者)</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第5話</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>はぐはぐ(著者)</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第103話</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>転生剣豪ズバババァーン！！</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>富士田けやき(原作) 坂崎ふれでぃ(作画)</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>番外編</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>となりのエルフがだらしない！</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>もゆる(著者)</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第1話</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>塔の管理をしてみよう</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>盧恩＆雪笠(Friendly Land)(著者) 早秋(原作) 雨神(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第105話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第25話④</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>ギャルの自転車を直したら懐かれた</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>タケチケイ（漫画） 生姜寧也（原作）</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第5話　ギャルにだって悩むこともある（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>回復術士のやり直し</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>月夜涙(原作) 羽賀ソウケン(漫画) しおこんぶ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第80話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>最弱と呼ばれた剣闘士のゲーム知識無双　ー女尊男卑世界のコロシアムで成り上がるー</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>ワタナベタカシ(著者) ケンノジ(原作)</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第6話</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>追放僧侶の賢者タイム</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>原作・野原のはて 作画・鈴木シオン</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第12話　封印空間</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+          <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+          <t>丈(著者)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第83話 前編</t>
+          <t>第142話</t>
         </is>
       </c>
     </row>
@@ -65847,17 +66884,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>ワンパンマン</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>むちまろ</t>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>第161話	有栖しくじる！（前編）</t>
+          <t>237撃目</t>
         </is>
       </c>
     </row>
@@ -65867,17 +66904,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+          <t>転生したらスライムだった件</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+          <t>原作：伏瀬 漫画：川上泰樹 キャラクター原案：みっつばー</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第27話-1「共闘」</t>
+          <t>第138話　西方動乱</t>
         </is>
       </c>
     </row>
@@ -65887,17 +66924,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>異世界おじさん</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>殆ど死んでいる(著者)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第８１話『炎神停止』④</t>
+          <t>番外編14</t>
         </is>
       </c>
     </row>
@@ -65907,17 +66944,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
+          <t>異世界居酒屋「のぶ」</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
+          <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第11話 後編</t>
+          <t>第135話</t>
         </is>
       </c>
     </row>
@@ -65927,17 +66964,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>魔術師クノンは見えている</t>
+          <t>蜘蛛ですが、なにか？</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+          <t>かかし朝浩(著者) 馬場翁(原作) 輝竜司(キャラクター原案)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第51話①</t>
+          <t>第80話その2</t>
         </is>
       </c>
     </row>
@@ -65947,17 +66984,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第10話後編：人間の悪意</t>
+          <t>第８８話　身バレの戦いが始まった</t>
         </is>
       </c>
     </row>
@@ -65967,17 +67004,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第８７話　ビーチバレーの戦いが始まった（２）</t>
+          <t>第14話前半</t>
         </is>
       </c>
     </row>
@@ -65987,17 +67024,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+          <t>氷結令嬢さまをフォローしたら、メチャメチャ溺愛されてしまった件@comic</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+          <t>漫画：ハレノチアメ 原作：愛坂タカト キャラクター原案：Bcoca</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第45話①</t>
+          <t>第16話</t>
         </is>
       </c>
     </row>
@@ -66007,17 +67044,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+          <t>食い詰め傭兵の幻想奇譚</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+          <t>原作／まいん キャラクター原案／peroshi 漫画／池宮アレア</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第23話-2</t>
+          <t>第29話 後編</t>
         </is>
       </c>
     </row>
@@ -66027,17 +67064,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>クセ強彼女は床にいざなう</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>須河篤志(著者)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第85話③</t>
+          <t>第26話前半</t>
         </is>
       </c>
     </row>
@@ -66047,17 +67084,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>ギルドの受付嬢リリナさんは俺にだけ冷たい</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>うたしま(漫画) 近藤玲司(原作)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第156話　戴冠式・後編</t>
+          <t>クエスト1</t>
         </is>
       </c>
     </row>
@@ -66067,17 +67104,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+          <t>異世界のんびり農家</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>三部べべ(漫画) ねうしとら(原作)</t>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第13話-1</t>
+          <t>第334話</t>
         </is>
       </c>
     </row>
@@ -66087,17 +67124,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>氷結令嬢さまをフォローしたら、メチャメチャ溺愛されてしまった件@comic</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>漫画：ハレノチアメ 原作：愛坂タカト キャラクター原案：Bcoca</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第15話</t>
+          <t>第85話④</t>
         </is>
       </c>
     </row>
@@ -66107,17 +67144,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>お前がヤったんだろ！</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>クシザキ</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第20話	絆創膏の正しい使い方</t>
+          <t>おまけ77</t>
         </is>
       </c>
     </row>
@@ -66127,17 +67164,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>隣の席の聖女様は俺にこっそりスカートの中を教えてくれる</t>
+          <t>魔のものたちは企てる</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>しろみね(漫画) 桜木桜（GA文庫）(原作) ただのゆきこ(原作イラスト)</t>
+          <t>加藤拓弐(原作) ガしガし(作画)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第2話</t>
+          <t>第40話</t>
         </is>
       </c>
     </row>
@@ -66147,17 +67184,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第13話 おむすび</t>
+          <t>祝！30万部突破記念イラスト</t>
         </is>
       </c>
     </row>
@@ -66167,17 +67204,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>「おかえり、パパ」</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>蝉丸</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第7話③</t>
+          <t>第39話　訪問</t>
         </is>
       </c>
     </row>
@@ -66187,17 +67224,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>物語の黒幕に転生して</t>
+          <t>まんきつしたい常連さん</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>瀬川はじめ(漫画) 結城涼(原作) なかむら(キャラクター原案)</t>
+          <t>しんみりん(著者)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第44話</t>
+          <t>特別イラスト</t>
         </is>
       </c>
     </row>
@@ -66207,17 +67244,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>島知宏 音速炒飯 有都あらゆる</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第３２食　エリクサー、ゴクゴクですわ！（前編）（３）</t>
+          <t>第7話④</t>
         </is>
       </c>
     </row>
@@ -66227,17 +67264,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>モリタ Ｕ４ nima</t>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第18話（１）　メイド大集結でお祝い！結婚披露宴（１）</t>
+          <t>第41話 独身貴族は孤高な馬と駆ける（1）</t>
         </is>
       </c>
     </row>
@@ -66247,17 +67284,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第13話後編</t>
+          <t>番外編　アリシアさんと宿ですわ！</t>
         </is>
       </c>
     </row>
@@ -66267,17 +67304,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>美人女上司滝沢さん</t>
+          <t>ぽんドロイド！ はまさん</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>やんBARU(著者)</t>
+          <t>はれやまはれぞう(著者)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第225話</t>
+          <t>第26話</t>
         </is>
       </c>
     </row>
@@ -66287,17 +67324,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>田舎で恋は難しい!?</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>ねこうめ(著者)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第６４話　迷宮の秘密に気付く器用貧乏（３）</t>
+          <t>第11話</t>
         </is>
       </c>
     </row>
@@ -66307,17 +67344,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>幼女戦記</t>
+          <t>異世界食堂　洋食のねこや</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>東條チカ(漫画) カルロ・ゼン(原作) 篠月しのぶ(キャラクター原案)</t>
+          <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第百二十一章：ドアノッカー作戦Ⅱ</t>
+          <t>第50話➁</t>
         </is>
       </c>
     </row>
@@ -66327,17 +67364,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>姫ヶ崎櫻子は今日も不憫可愛い</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>安田剛助(著者)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第92話その1</t>
+          <t>第60話</t>
         </is>
       </c>
     </row>
@@ -66347,17 +67384,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>バーサス</t>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第36話　巨影（２）</t>
+          <t>第55話 破壊の魔剣③</t>
         </is>
       </c>
     </row>
@@ -66367,17 +67404,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+          <t>まったく最近の探偵ときたら</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ヨウハ(著者)</t>
+          <t>五十嵐正邦(著者)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第5話-2</t>
+          <t>第119話その２</t>
         </is>
       </c>
     </row>
@@ -66387,17 +67424,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>ダークサモナーとデキている</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>車王(著者)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第５１話　勇者、完全に封印されて宇宙の彼方へ捨てられてしまう（１）</t>
+          <t>アニメ放送開始記念イラスト！</t>
         </is>
       </c>
     </row>
@@ -66407,17 +67444,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第51話　奴は合コンに行く（後編）</t>
+          <t>第19話-1：前へ進んで</t>
         </is>
       </c>
     </row>
@@ -66427,17 +67464,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第３話　「暁の剣」を雇って開拓します！（３）</t>
+          <t>第６４話　迷宮の秘密に気付く器用貧乏（４）</t>
         </is>
       </c>
     </row>
@@ -66447,17 +67484,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>拷問202</t>
+          <t>第92話その2</t>
         </is>
       </c>
     </row>
@@ -66467,17 +67504,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>よくわからないけれど異世界に転生していたようです</t>
+          <t>英雄王、武を極めるため転生す ～そして、世界最強の見習い騎士♀～</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>内々けやき あし カオミン</t>
+          <t>漫画‥くろむら基人 原作‥ハヤケン キャラクター原案‥Nagu</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第161話 よくわからないけれどマウンティングされたみたいです（２）</t>
+          <t>第34話 後編</t>
         </is>
       </c>
     </row>
@@ -66487,17 +67524,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>戸賀 環 坂木持丸 riritto</t>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第73話①　こみけのためにかけ回ってみた</t>
+          <t>第35話②</t>
         </is>
       </c>
     </row>
@@ -66507,17 +67544,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第13話-2</t>
+          <t>第５１話　勇者、完全に封印されて宇宙の彼方へ捨てられてしまう（２）</t>
         </is>
       </c>
     </row>
@@ -66527,17 +67564,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>くらいあの子としたいこと</t>
+          <t>わたしで童貞捨てたくせに</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>碇マナツ(著者)</t>
+          <t>雲雀湯(原作) 霧崎秀征(漫画) U35(キャラクター原案)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第104話</t>
+          <t>第1話</t>
         </is>
       </c>
     </row>
@@ -66547,17 +67584,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+          <t>魔術師クノンは見えている</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第9話(2)</t>
+          <t>第51話①</t>
         </is>
       </c>
     </row>
@@ -66567,17 +67604,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>如意自在(著者)</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>番外編</t>
+          <t>拷問203</t>
         </is>
       </c>
     </row>
@@ -66587,17 +67624,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>KAKERU</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第80話「知らんとこでえらいことなっとる」（後半）</t>
+          <t>第73話②　こみけのためにかけ回ってみた</t>
         </is>
       </c>
     </row>
@@ -66607,17 +67644,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ライブダンジョン！</t>
+          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ことりりょう(作画) dy冷凍(原作) Mika Pikazo(キャラクター原案)</t>
+          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第100話前半</t>
+          <t>第４話　ゴーレム任せで開拓します！（１）</t>
         </is>
       </c>
     </row>
@@ -66627,17 +67664,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>異世界「嘘」ガイド</t>
+          <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>辻島もと(著者)</t>
+          <t>内々けやき あし カオミン</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第5話</t>
+          <t>第162話 よくわからないけれど脱出を図るみたいです（１）</t>
         </is>
       </c>
     </row>
@@ -66647,17 +67684,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>サーシャちゃんとクラスメイトオタクくん</t>
+          <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>はぐはぐ(著者)</t>
+          <t>クール教信者</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第103話</t>
+          <t>第175話</t>
         </is>
       </c>
     </row>
@@ -66667,17 +67704,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>転生剣豪ズバババァーン！！</t>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>富士田けやき(原作) 坂崎ふれでぃ(作画)</t>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>番外編</t>
+          <t>第13話-1：王子様です</t>
         </is>
       </c>
     </row>
@@ -66687,17 +67724,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>となりのエルフがだらしない！</t>
+          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>もゆる(著者)</t>
+          <t>六志麻あさ 業務用餅 kisui</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第1話</t>
+          <t>第９４話</t>
         </is>
       </c>
     </row>
@@ -66707,17 +67744,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>塔の管理をしてみよう</t>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>盧恩＆雪笠(Friendly Land)(著者) 早秋(原作) 雨神(キャラクター原案)</t>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第105話前編</t>
+          <t>第9話(2)</t>
         </is>
       </c>
     </row>
@@ -66727,17 +67764,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
+          <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
+          <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第25話④</t>
+          <t>第34話</t>
         </is>
       </c>
     </row>
@@ -66747,17 +67784,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ギャルの自転車を直したら懐かれた</t>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>タケチケイ（漫画） 生姜寧也（原作）</t>
+          <t>如意自在(著者)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第5話　ギャルにだって悩むこともある（後編）</t>
+          <t>第7話前半</t>
         </is>
       </c>
     </row>
@@ -66767,17 +67804,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>回復術士のやり直し</t>
+          <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>月夜涙(原作) 羽賀ソウケン(漫画) しおこんぶ(キャラクター原案)</t>
+          <t>原作:剃り残し 漫画:大窪太一</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第80話-2</t>
+          <t>第12話(後編)</t>
         </is>
       </c>
     </row>
@@ -66787,17 +67824,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>最弱と呼ばれた剣闘士のゲーム知識無双　ー女尊男卑世界のコロシアムで成り上がるー</t>
+          <t>最果てのパラディン</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ワタナベタカシ(著者) ケンノジ(原作)</t>
+          <t>奥橋睦（漫画） 柳野かなた（原作） 輪くすさが（キャラクター原案）</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第6話</t>
+          <t>第73話　無敵の巨人Ⅵ</t>
         </is>
       </c>
     </row>
@@ -66807,17 +67844,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>追放僧侶の賢者タイム</t>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>原作・野原のはて 作画・鈴木シオン</t>
+          <t>セレビィ量産型(著者)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第12話　封印空間</t>
+          <t>第30話前半</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-10-12
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -75,6 +75,7 @@
     <sheet name="2026-09-21" sheetId="67" state="visible" r:id="rId67"/>
     <sheet name="2026-09-28" sheetId="68" state="visible" r:id="rId68"/>
     <sheet name="2026-10-05" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet name="2026-10-12" sheetId="70" state="visible" r:id="rId70"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -66859,1000 +66860,1000 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>宇崎ちゃんは遊びたい！</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="0" t="inlineStr">
         <is>
           <t>丈(著者)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>第142話</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>ワンパンマン</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
         <is>
           <t>237撃目</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>転生したらスライムだった件</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>原作：伏瀬 漫画：川上泰樹 キャラクター原案：みっつばー</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>第138話　西方動乱</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
         <is>
           <t>異世界おじさん</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>殆ど死んでいる(著者)</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>番外編14</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="0" t="inlineStr">
         <is>
           <t>異世界居酒屋「のぶ」</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>蝉川夏哉(原作) ヴァージニア二等兵(漫画) 転(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>第135話</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="0" t="inlineStr">
         <is>
           <t>蜘蛛ですが、なにか？</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>かかし朝浩(著者) 馬場翁(原作) 輝竜司(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>第80話その2</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="0" t="inlineStr">
         <is>
           <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>マツモトケンゴ</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>第８８話　身バレの戦いが始まった</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>貞操逆転世界で頼めばヤれると噂の俺</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
         <is>
           <t>第14話前半</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="0" t="inlineStr">
         <is>
           <t>氷結令嬢さまをフォローしたら、メチャメチャ溺愛されてしまった件@comic</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
         <is>
           <t>漫画：ハレノチアメ 原作：愛坂タカト キャラクター原案：Bcoca</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr">
         <is>
           <t>第16話</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="0" t="inlineStr">
         <is>
           <t>食い詰め傭兵の幻想奇譚</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
         <is>
           <t>原作／まいん キャラクター原案／peroshi 漫画／池宮アレア</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="0" t="inlineStr">
         <is>
           <t>第29話 後編</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="0" t="inlineStr">
         <is>
           <t>クセ強彼女は床にいざなう</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>須河篤志(著者)</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>第26話前半</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="0" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t>ギルドの受付嬢リリナさんは俺にだけ冷たい</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>うたしま(漫画) 近藤玲司(原作)</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>クエスト1</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="0" t="n">
         <v>13</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>異世界のんびり農家</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>第334話</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="0" t="n">
         <v>14</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="0" t="inlineStr">
         <is>
           <t>リビルドワールド</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>第85話④</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="0" t="n">
         <v>15</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
         <is>
           <t>実は俺、最強でした？</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="0" t="inlineStr">
         <is>
           <t>おまけ77</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="0" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="0" t="inlineStr">
         <is>
           <t>魔のものたちは企てる</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>加藤拓弐(原作) ガしガし(作画)</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t>第40話</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" s="0" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="0" t="inlineStr">
         <is>
           <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="0" t="inlineStr">
         <is>
           <t>祝！30万部突破記念イラスト</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" s="0" t="n">
         <v>18</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="0" t="inlineStr">
         <is>
           <t>「おかえり、パパ」</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="0" t="inlineStr">
         <is>
           <t>蝉丸</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="0" t="inlineStr">
         <is>
           <t>第39話　訪問</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" s="0" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="0" t="inlineStr">
         <is>
           <t>まんきつしたい常連さん</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="0" t="inlineStr">
         <is>
           <t>しんみりん(著者)</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="0" t="inlineStr">
         <is>
           <t>特別イラスト</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" s="0" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="0" t="inlineStr">
         <is>
           <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="0" t="inlineStr">
         <is>
           <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="0" t="inlineStr">
         <is>
           <t>第7話④</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="0" t="inlineStr">
         <is>
           <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr">
         <is>
           <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="0" t="inlineStr">
         <is>
           <t>第41話 独身貴族は孤高な馬と駆ける（1）</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="A23" s="0" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="0" t="inlineStr">
         <is>
           <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
         <is>
           <t>島知宏 音速炒飯 有都あらゆる</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="0" t="inlineStr">
         <is>
           <t>番外編　アリシアさんと宿ですわ！</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="n">
+      <c r="A24" s="0" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="0" t="inlineStr">
         <is>
           <t>ぽんドロイド！ はまさん</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>はれやまはれぞう(著者)</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="0" t="inlineStr">
         <is>
           <t>第26話</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
+      <c r="A25" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="0" t="inlineStr">
         <is>
           <t>田舎で恋は難しい!?</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr">
         <is>
           <t>ねこうめ(著者)</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="0" t="inlineStr">
         <is>
           <t>第11話</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="n">
+      <c r="A26" s="0" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="0" t="inlineStr">
         <is>
           <t>異世界食堂　洋食のねこや</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>犬塚惇平(ヒーロー文庫／イマジカインフォス)(原作) ヤミザワ(漫画) モロザワ(漫画) エナミカツミ(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="0" t="inlineStr">
         <is>
           <t>第50話➁</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="n">
+      <c r="A27" s="0" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="0" t="inlineStr">
         <is>
           <t>姫ヶ崎櫻子は今日も不憫可愛い</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="0" t="inlineStr">
         <is>
           <t>安田剛助(著者)</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="0" t="inlineStr">
         <is>
           <t>第60話</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="n">
+      <c r="A28" s="0" t="n">
         <v>27</v>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="0" t="inlineStr">
         <is>
           <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="0" t="inlineStr">
         <is>
           <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="0" t="inlineStr">
         <is>
           <t>第55話 破壊の魔剣③</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="n">
+      <c r="A29" s="0" t="n">
         <v>28</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="0" t="inlineStr">
         <is>
           <t>まったく最近の探偵ときたら</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="0" t="inlineStr">
         <is>
           <t>五十嵐正邦(著者)</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="0" t="inlineStr">
         <is>
           <t>第119話その２</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="n">
+      <c r="A30" s="0" t="n">
         <v>29</v>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="0" t="inlineStr">
         <is>
           <t>ダークサモナーとデキている</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="0" t="inlineStr">
         <is>
           <t>車王(著者)</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="0" t="inlineStr">
         <is>
           <t>アニメ放送開始記念イラスト！</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="n">
+      <c r="A31" s="0" t="n">
         <v>30</v>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="0" t="inlineStr">
         <is>
           <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="0" t="inlineStr">
         <is>
           <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="0" t="inlineStr">
         <is>
           <t>第19話-1：前へ進んで</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="n">
+      <c r="A32" s="0" t="n">
         <v>31</v>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="0" t="inlineStr">
         <is>
           <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr">
         <is>
           <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="0" t="inlineStr">
         <is>
           <t>第６４話　迷宮の秘密に気付く器用貧乏（４）</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="n">
+      <c r="A33" s="0" t="n">
         <v>32</v>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="0" t="inlineStr">
         <is>
           <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="0" t="inlineStr">
         <is>
           <t>第92話その2</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="n">
+      <c r="A34" s="0" t="n">
         <v>33</v>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B34" s="0" t="inlineStr">
         <is>
           <t>英雄王、武を極めるため転生す ～そして、世界最強の見習い騎士♀～</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="0" t="inlineStr">
         <is>
           <t>漫画‥くろむら基人 原作‥ハヤケン キャラクター原案‥Nagu</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="0" t="inlineStr">
         <is>
           <t>第34話 後編</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="n">
+      <c r="A35" s="0" t="n">
         <v>34</v>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B35" s="0" t="inlineStr">
         <is>
           <t>女友達は頼めば意外とヤらせてくれる</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="0" t="inlineStr">
         <is>
           <t>ろくろ(漫画) 鏡遊(原作)</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="0" t="inlineStr">
         <is>
           <t>第35話②</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="n">
+      <c r="A36" s="0" t="n">
         <v>35</v>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="0" t="inlineStr">
         <is>
           <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="0" t="inlineStr">
         <is>
           <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="0" t="inlineStr">
         <is>
           <t>第５１話　勇者、完全に封印されて宇宙の彼方へ捨てられてしまう（２）</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="n">
+      <c r="A37" s="0" t="n">
         <v>36</v>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="0" t="inlineStr">
         <is>
           <t>わたしで童貞捨てたくせに</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="0" t="inlineStr">
         <is>
           <t>雲雀湯(原作) 霧崎秀征(漫画) U35(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="0" t="inlineStr">
         <is>
           <t>第1話</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="n">
+      <c r="A38" s="0" t="n">
         <v>37</v>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B38" s="0" t="inlineStr">
         <is>
           <t>魔術師クノンは見えている</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="0" t="inlineStr">
         <is>
           <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="0" t="inlineStr">
         <is>
           <t>第51話①</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="n">
+      <c r="A39" s="0" t="n">
         <v>38</v>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="0" t="inlineStr">
         <is>
           <t>姫様“拷問”の時間です</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="0" t="inlineStr">
         <is>
           <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="0" t="inlineStr">
         <is>
           <t>拷問203</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="n">
+      <c r="A40" s="0" t="n">
         <v>39</v>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="0" t="inlineStr">
         <is>
           <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="0" t="inlineStr">
         <is>
           <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="0" t="inlineStr">
         <is>
           <t>第73話②　こみけのためにかけ回ってみた</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="n">
+      <c r="A41" s="0" t="n">
         <v>40</v>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="0" t="inlineStr">
         <is>
           <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="0" t="inlineStr">
         <is>
           <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="0" t="inlineStr">
         <is>
           <t>第４話　ゴーレム任せで開拓します！（１）</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="n">
+      <c r="A42" s="0" t="n">
         <v>41</v>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="0" t="inlineStr">
         <is>
           <t>よくわからないけれど異世界に転生していたようです</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="0" t="inlineStr">
         <is>
           <t>内々けやき あし カオミン</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="0" t="inlineStr">
         <is>
           <t>第162話 よくわからないけれど脱出を図るみたいです（１）</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="n">
+      <c r="A43" s="0" t="n">
         <v>42</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="0" t="inlineStr">
         <is>
           <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="0" t="inlineStr">
         <is>
           <t>クール教信者</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="0" t="inlineStr">
         <is>
           <t>第175話</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="n">
+      <c r="A44" s="0" t="n">
         <v>43</v>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="0" t="inlineStr">
         <is>
           <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="0" t="inlineStr">
         <is>
           <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="0" t="inlineStr">
         <is>
           <t>第13話-1：王子様です</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="n">
+      <c r="A45" s="0" t="n">
         <v>44</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="0" t="inlineStr">
         <is>
           <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="0" t="inlineStr">
         <is>
           <t>六志麻あさ 業務用餅 kisui</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="0" t="inlineStr">
         <is>
           <t>第９４話</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="n">
+      <c r="A46" s="0" t="n">
         <v>45</v>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="0" t="inlineStr">
         <is>
           <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="0" t="inlineStr">
         <is>
           <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="0" t="inlineStr">
         <is>
           <t>第9話(2)</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="n">
+      <c r="A47" s="0" t="n">
         <v>46</v>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="0" t="inlineStr">
         <is>
           <t>男嫌いな美人姉妹を名前も告げずに助けたら一体どうなる?</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="0" t="inlineStr">
         <is>
           <t>みょん(原作) 司馬淳子(漫画) ぎうにう(キャラクターデザイン)</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="0" t="inlineStr">
         <is>
           <t>第34話</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="n">
+      <c r="A48" s="0" t="n">
         <v>47</v>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="0" t="inlineStr">
         <is>
           <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="0" t="inlineStr">
         <is>
           <t>如意自在(著者)</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="0" t="inlineStr">
         <is>
           <t>第7話前半</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="n">
+      <c r="A49" s="0" t="n">
         <v>48</v>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="0" t="inlineStr">
         <is>
           <t>立ち飲み居酒屋でクーデレダウナー系女子大生が隣に来る話</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="0" t="inlineStr">
         <is>
           <t>原作:剃り残し 漫画:大窪太一</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="0" t="inlineStr">
         <is>
           <t>第12話(後編)</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="n">
+      <c r="A50" s="0" t="n">
         <v>49</v>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="0" t="inlineStr">
         <is>
           <t>最果てのパラディン</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="0" t="inlineStr">
         <is>
           <t>奥橋睦（漫画） 柳野かなた（原作） 輪くすさが（キャラクター原案）</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="0" t="inlineStr">
         <is>
           <t>第73話　無敵の巨人Ⅵ</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="n">
+      <c r="A51" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="0" t="inlineStr">
         <is>
           <t>三枝さんはメガネ先輩と恋を描く</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="0" t="inlineStr">
         <is>
           <t>セレビィ量産型(著者)</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="0" t="inlineStr">
         <is>
           <t>第30話前半</t>
         </is>
@@ -68899,6 +68900,1042 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>転生したらスライムだった件</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>原作：伏瀬 漫画：川上泰樹 キャラクター原案：みっつばー</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>第140話　西方動乱３</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>【描きおろし公開】人気投票＆キャラへの質問大募集、結果発表！【第13巻発売記念】</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>異種族レビュアーズ</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>天原(原作) masha(作画)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>コミックス12巻発売記念イラスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>第42話：男の覚悟①</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>不徳のギルド</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>河添太一</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>第１１１話：流れた血</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>第162話	有栖しくじる！（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>王子様の友達</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>すけろく(著者)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>第41話</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>コミックス4巻告知</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>第８２話『決壊停止』①</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>魔術師クノンは見えている</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>第51話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>第91話その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ダークサモナーとデキている</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>車王(著者)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>コミックス第8巻情報！</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>このヒーラー、めんどくさい</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>丹念に発酵(著者)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>第102話：忍者</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>第19話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>第141話　決意してみるⅠ（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>第335話</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ダンジョンの幼なじみ</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>久真やすひさ(著者)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>第69話</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>第157話　側近候補</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>第105話　新たな大地(ゆうえんち)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>クシザキ</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>第21話	湯煙の合宿　前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>第86話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>モリタ Ｕ４ nima</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>第18話（２）　メイド大集結でお祝い！結婚披露宴（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>リアデイルの大地にて</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>月見だしお(著者) Ceez(原作) てんまそ(キャラクター原案) 涼風涼(構成)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>第44章</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>第42話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>望まぬ不死の冒険者</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>中曽根ハイジ（漫画） 丘野 優（原作） じゃいあん（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>第67話　討伐依頼</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>第41話 独身貴族は孤高な馬と駆ける（2）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>第7話⑤</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>美人女上司滝沢さん</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>やんBARU(著者)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>第226話</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>番外編　武勇伝の力ですわ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>濁る瞳で何を願う ハイセルク戦記</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>トルトネン 創-taro 斎藤八呑</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>第42話 統率者について②</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>第8話</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>第６４話　迷宮の秘密に気付く器用貧乏（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>第92話その3</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>板垣恵介 林たかあき</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>第79話 魂の咆哮</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>理想のヒモ生活</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>第111話　その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>第５１話　勇者、完全に封印されて宇宙の彼方へ捨てられてしまう（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>第４話　ゴーレム任せで開拓します！（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>おやすみのお知らせ</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>第162話 よくわからないけれど脱出を図るみたいです（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>異世界転生ダンジョンマスター　温泉ダンジョンを作る</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>天原(原作) アルデヒド(作画) じゅん(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>第7話</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>第50話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>久遠まこと(著者) 石のやっさん(原作)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>コミックス８巻発売告知</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>第5話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>第105話</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>豊熟の休載まんが</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>拷問204</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>如意自在(著者)</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>第7話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>バーサス</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>第37話　恐怖の必要性（前編-1）</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>異世界「嘘」ガイド</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>辻島もと(著者)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>第6話</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>氷結令嬢さまをフォローしたら、メチャメチャ溺愛されてしまった件@comic</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>漫画：ハレノチアメ 原作：愛坂タカト キャラクター原案：Bcoca</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>2巻表紙イラスト公開！</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add ranking data for 2026-10-19
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -76,6 +76,7 @@
     <sheet name="2026-09-28" sheetId="68" state="visible" r:id="rId68"/>
     <sheet name="2026-10-05" sheetId="69" state="visible" r:id="rId69"/>
     <sheet name="2026-10-12" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet name="2026-10-19" sheetId="71" state="visible" r:id="rId71"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -68932,22 +68933,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>転生したらスライムだった件</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>原作：伏瀬 漫画：川上泰樹 キャラクター原案：みっつばー</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>第140話　西方動乱３</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>【描きおろし公開】人気投票＆キャラへの質問大募集、結果発表！【第13巻発売記念】</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>異種族レビュアーズ</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>天原(原作) masha(作画)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>コミックス12巻発売記念イラスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第42話：男の覚悟①</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>不徳のギルド</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>河添太一</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第１１１話：流れた血</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>生徒会にも穴はある！</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>むちまろ</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第162話	有栖しくじる！（後編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>王子様の友達</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>すけろく(著者)</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第41話</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>コミックス4巻告知</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第８２話『決壊停止』①</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>魔術師クノンは見えている</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第51話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第91話その1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>ダークサモナーとデキている</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>車王(著者)</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>コミックス第8巻情報！</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>このヒーラー、めんどくさい</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>丹念に発酵(著者)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第102話：忍者</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第19話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第141話　決意してみるⅠ（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>異世界のんびり農家</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第335話</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>ダンジョンの幼なじみ</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>久真やすひさ(著者)</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第69話</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第157話　側近候補</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第105話　新たな大地(ゆうえんち)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>クシザキ</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第21話	湯煙の合宿　前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第86話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>モリタ Ｕ４ nima</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第18話（２）　メイド大集結でお祝い！結婚披露宴（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>リアデイルの大地にて</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>月見だしお(著者) Ceez(原作) てんまそ(キャラクター原案) 涼風涼(構成)</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第44章</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>第42話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>望まぬ不死の冒険者</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>中曽根ハイジ（漫画） 丘野 優（原作） じゃいあん（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第67話　討伐依頼</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第41話 独身貴族は孤高な馬と駆ける（2）</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第7話⑤</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>美人女上司滝沢さん</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>やんBARU(著者)</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>第226話</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>番外編　武勇伝の力ですわ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>濁る瞳で何を願う ハイセルク戦記</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>トルトネン 創-taro 斎藤八呑</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>第42話 統率者について②</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第8話</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第６４話　迷宮の秘密に気付く器用貧乏（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第92話その3</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>板垣恵介 林たかあき</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第79話 魂の咆哮</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>理想のヒモ生活</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第111話　その2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第５１話　勇者、完全に封印されて宇宙の彼方へ捨てられてしまう（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第４話　ゴーレム任せで開拓します！（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>おやすみのお知らせ</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第162話 よくわからないけれど脱出を図るみたいです（２）</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>異世界転生ダンジョンマスター　温泉ダンジョンを作る</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>天原(原作) アルデヒド(作画) じゅん(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>第7話</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第50話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>久遠まこと(著者) 石のやっさん(原作)</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>コミックス８巻発売告知</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第5話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>くらいあの子としたいこと</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>碇マナツ(著者)</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>第105話</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>豊熟の休載まんが</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>拷問204</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>如意自在(著者)</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第7話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>バーサス</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第37話　恐怖の必要性（前編-1）</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>異世界「嘘」ガイド</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>辻島もと(著者)</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>第6話</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>氷結令嬢さまをフォローしたら、メチャメチャ溺愛されてしまった件@comic</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>漫画：ハレノチアメ 原作：愛坂タカト キャラクター原案：Bcoca</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>2巻表紙イラスト公開！</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>転生したらスライムだった件</t>
+          <t>ワンパンマン</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>原作：伏瀬 漫画：川上泰樹 キャラクター原案：みっつばー</t>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>第140話　西方動乱３</t>
+          <t>238撃目</t>
         </is>
       </c>
     </row>
@@ -68957,17 +69994,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+          <t>異世界おじさん</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+          <t>殆ど死んでいる(著者)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>【描きおろし公開】人気投票＆キャラへの質問大募集、結果発表！【第13巻発売記念】</t>
+          <t>コミックス第16巻発売告知</t>
         </is>
       </c>
     </row>
@@ -68977,17 +70014,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>異種族レビュアーズ</t>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>天原(原作) masha(作画)</t>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>コミックス12巻発売記念イラスト</t>
+          <t>第42話：男の覚悟②</t>
         </is>
       </c>
     </row>
@@ -68997,17 +70034,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>zunta(作画) はらわたさいぞう(原作)</t>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第42話：男の覚悟①</t>
+          <t>第27話-2「共闘」</t>
         </is>
       </c>
     </row>
@@ -69017,17 +70054,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>不徳のギルド</t>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>河添太一</t>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第１１１話：流れた血</t>
+          <t>第11話前編：情け無用の討伐戦</t>
         </is>
       </c>
     </row>
@@ -69037,17 +70074,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>生徒会にも穴はある！</t>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>むちまろ</t>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第162話	有栖しくじる！（後編）</t>
+          <t>第27話後半</t>
         </is>
       </c>
     </row>
@@ -69057,17 +70094,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>王子様の友達</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>すけろく(著者)</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第41話</t>
+          <t>第８２話『決壊停止』②</t>
         </is>
       </c>
     </row>
@@ -69077,17 +70114,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>コミックス4巻告知</t>
+          <t>第14話後半</t>
         </is>
       </c>
     </row>
@@ -69097,17 +70134,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第８２話『決壊停止』①</t>
+          <t>第84話 前編</t>
         </is>
       </c>
     </row>
@@ -69117,17 +70154,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>魔術師クノンは見えている</t>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第51話②</t>
+          <t>第45話②</t>
         </is>
       </c>
     </row>
@@ -69137,17 +70174,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第91話その1</t>
+          <t>第８９話　肝試しの戦いが始まった（１）</t>
         </is>
       </c>
     </row>
@@ -69157,17 +70194,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ダークサモナーとデキている</t>
+          <t>クセ強彼女は床にいざなう</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>車王(著者)</t>
+          <t>須河篤志(著者)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>コミックス第8巻情報！</t>
+          <t>第26話後半</t>
         </is>
       </c>
     </row>
@@ -69177,17 +70214,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>このヒーラー、めんどくさい</t>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>丹念に発酵(著者)</t>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第102話：忍者</t>
+          <t>第24話-1</t>
         </is>
       </c>
     </row>
@@ -69197,17 +70234,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>辺境モブ貴族のウチに嫁いできた悪役令嬢が、めちゃくちゃできる良い嫁なんだが？</t>
+          <t>死亡エンドを回避したギャルゲーのヒロインたちが俺の【日記帳】を読んで秘密を知ったらしい</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>tera(原作) 朝倉はやて(作画) 徹田(キャラクター原案)</t>
+          <t>addict(原作) となりける(作画) へいろー(キャラクター原案)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第19話-2</t>
+          <t>第2話</t>
         </is>
       </c>
     </row>
@@ -69227,7 +70264,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第141話　決意してみるⅠ（前編）</t>
+          <t>第141話　決意してみるⅠ（中編）</t>
         </is>
       </c>
     </row>
@@ -69237,17 +70274,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>異世界のんびり農家</t>
+          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
+          <t>六志麻あさ 業務用餅 kisui</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第335話</t>
+          <t>第９６話</t>
         </is>
       </c>
     </row>
@@ -69257,17 +70294,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ダンジョンの幼なじみ</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>久真やすひさ(著者)</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第69話</t>
+          <t>第158話　新王謁見式</t>
         </is>
       </c>
     </row>
@@ -69277,17 +70314,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第157話　側近候補</t>
+          <t>第13話-2</t>
         </is>
       </c>
     </row>
@@ -69297,17 +70334,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>板垣恵介 猪原賽 陸井栄史</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第105話　新たな大地(ゆうえんち)</t>
+          <t>第86話➁</t>
         </is>
       </c>
     </row>
@@ -69317,17 +70354,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>お前がヤったんだろ！</t>
+          <t>ぽんドロイド！ はまさん</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>クシザキ</t>
+          <t>はれやまはれぞう(著者)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第21話	湯煙の合宿　前編</t>
+          <t>第27話</t>
         </is>
       </c>
     </row>
@@ -69337,17 +70374,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第86話①</t>
+          <t>第8話①</t>
         </is>
       </c>
     </row>
@@ -69357,17 +70394,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>モリタ Ｕ４ nima</t>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第18話（２）　メイド大集結でお祝い！結婚披露宴（２）</t>
+          <t>第41話 独身貴族は孤高な馬と駆ける（3）</t>
         </is>
       </c>
     </row>
@@ -69377,17 +70414,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>リアデイルの大地にて</t>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>月見だしお(著者) Ceez(原作) てんまそ(キャラクター原案) 涼風涼(構成)</t>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第44章</t>
+          <t>第14話 灯り（前編）</t>
         </is>
       </c>
     </row>
@@ -69397,17 +70434,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>え、社内システム全てワンオペしている私を解雇ですか？</t>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>漫画：伊於 原作：下城米雪 キャラクター原案：icchi</t>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>第42話後半</t>
+          <t>番外編　お土産ですわ！</t>
         </is>
       </c>
     </row>
@@ -69417,17 +70454,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>望まぬ不死の冒険者</t>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>中曽根ハイジ（漫画） 丘野 優（原作） じゃいあん（キャラクター原案）</t>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第67話　討伐依頼</t>
+          <t>第19話-2：前へ進んで</t>
         </is>
       </c>
     </row>
@@ -69437,17 +70474,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第41話 独身貴族は孤高な馬と駆ける（2）</t>
+          <t>第55話 破壊の魔剣④</t>
         </is>
       </c>
     </row>
@@ -69457,17 +70494,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第7話⑤</t>
+          <t>第14話前編</t>
         </is>
       </c>
     </row>
@@ -69477,17 +70514,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>美人女上司滝沢さん</t>
+          <t>ギルドの受付嬢リリナさんは俺にだけ冷たい</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>やんBARU(著者)</t>
+          <t>うたしま(漫画) 近藤玲司(原作)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>第226話</t>
+          <t>クエスト2 前編</t>
         </is>
       </c>
     </row>
@@ -69497,17 +70534,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+          <t>おとなりのダウナーさんは無理させない</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>島知宏 音速炒飯 有都あらゆる</t>
+          <t>瑠璃いろ(著者)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>番外編　武勇伝の力ですわ！</t>
+          <t>第19話</t>
         </is>
       </c>
     </row>
@@ -69517,17 +70554,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>濁る瞳で何を願う ハイセルク戦記</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>トルトネン 創-taro 斎藤八呑</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>第42話 統率者について②</t>
+          <t>拷問205</t>
         </is>
       </c>
     </row>
@@ -69537,17 +70574,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>バズった?最強種だらけのクリア不可能ダンジョンを配信? 自宅なんだけど?</t>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>原作/相野仁 漫画/今 豊太郎 キャラクター原案/桑島 黎音</t>
+          <t>ヨウハ(著者)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第8話</t>
+          <t>第6話-1</t>
         </is>
       </c>
     </row>
@@ -69557,17 +70594,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>勇者パーティを追い出された器用貧乏　～パーティ事情で付与術士をやっていた剣士、万能へと至る～</t>
+          <t>魔術師クノンは見えている</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>漫画：よねぞう 原作：都神樹 キャラクター原案：きさらぎゆり</t>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第６４話　迷宮の秘密に気付く器用貧乏（４）</t>
+          <t>第51話②</t>
         </is>
       </c>
     </row>
@@ -69577,17 +70614,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>治癒魔法の間違った使い方 ~戦場を駆ける回復要員~</t>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>九我山レキ(漫画) くろかた(原作) ＫｅＧ(キャラクター原案)</t>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第92話その3</t>
+          <t>第13話-2：王子様です</t>
         </is>
       </c>
     </row>
@@ -69597,17 +70634,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>板垣恵介 林たかあき</t>
+          <t>戸賀 環 坂木持丸 riritto</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第79話 魂の咆哮</t>
+          <t>第74話①　こみけを開催してみた</t>
         </is>
       </c>
     </row>
@@ -69617,17 +70654,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>理想のヒモ生活</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>日月ネコ(漫画) 渡辺恒彦（ヒーロー文庫／イマジカインフォス）(原作) 文倉十(キャラクター原案)</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第111話　その2</t>
+          <t>第５１話　勇者、完全に封印されて宇宙の彼方へ捨てられてしまう（４）</t>
         </is>
       </c>
     </row>
@@ -69637,17 +70674,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第５１話　勇者、完全に封印されて宇宙の彼方へ捨てられてしまう（３）</t>
+          <t>第14話-1</t>
         </is>
       </c>
     </row>
@@ -69657,17 +70694,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第４話　ゴーレム任せで開拓します！（２）</t>
+          <t>第10話(1)</t>
         </is>
       </c>
     </row>
@@ -69677,17 +70714,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>小さくて可愛い文芸部の知的な先輩を、膝の上に乗せたら毎日座ってくるようになった</t>
+          <t>小林さんちのメイドラゴン</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>甘露アメ(漫画) ゆめいげつ(原作)</t>
+          <t>クール教信者</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>おやすみのお知らせ</t>
+          <t>第176話</t>
         </is>
       </c>
     </row>
@@ -69707,7 +70744,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第162話 よくわからないけれど脱出を図るみたいです（２）</t>
+          <t>第163話 よくわからないけれど荒波を乗り越えたみたいです（１）</t>
         </is>
       </c>
     </row>
@@ -69717,17 +70754,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>異世界転生ダンジョンマスター　温泉ダンジョンを作る</t>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>天原(原作) アルデヒド(作画) じゅん(キャラクター原案)</t>
+          <t>如意自在(著者)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>第7話</t>
+          <t>番外編2</t>
         </is>
       </c>
     </row>
@@ -69737,17 +70774,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>経験値貯蓄でのんびり傷心旅行 ～勇者と恋人に追放された戦士の無自覚ざまぁ～</t>
+          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>奏ヨシキ(著者) 徳川レモン(原作) riritto(キャラクターデザイン)</t>
+          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第50話-2</t>
+          <t>第４話　ゴーレム任せで開拓します！（３）</t>
         </is>
       </c>
     </row>
@@ -69757,17 +70794,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>勇者に全部奪われた俺は勇者の母親とパーティを組みました！</t>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>久遠まこと(著者) 石のやっさん(原作)</t>
+          <t>はぐはぐ(著者)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>コミックス８巻発売告知</t>
+          <t>第104話</t>
         </is>
       </c>
     </row>
@@ -69777,17 +70814,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
+          <t>雨森潤奈は湿度が高い</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
+          <t>水城水城(原作) 稲鳴四季(作画) 潮崎しの(キャラクター原案)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第5話-1</t>
+          <t>第5話</t>
         </is>
       </c>
     </row>
@@ -69797,17 +70834,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>くらいあの子としたいこと</t>
+          <t>描けないのでヤってみた</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>碇マナツ(著者)</t>
+          <t>逢上おかき(著者)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>第105話</t>
+          <t>連載開始告知</t>
         </is>
       </c>
     </row>
@@ -69817,17 +70854,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
+          <t>おせっかい女子、恋をする</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
+          <t>音竹 ひかる(著者)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>豊熟の休載まんが</t>
+          <t>第37話</t>
         </is>
       </c>
     </row>
@@ -69837,17 +70874,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>女子高生の無駄づかい</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>ビーノ(著者)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>拷問204</t>
+          <t>第150話　じゅんばん</t>
         </is>
       </c>
     </row>
@@ -69857,17 +70894,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
+          <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>如意自在(著者)</t>
+          <t>昼行燈（原作） しいたけ元帥（漫画）</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第7話後半</t>
+          <t>第53話（前半）</t>
         </is>
       </c>
     </row>
@@ -69877,17 +70914,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>バーサス</t>
+          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
+          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第37話　恐怖の必要性（前編-1）</t>
+          <t>第12話②「球技大会！」</t>
         </is>
       </c>
     </row>
@@ -69897,17 +70934,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>異世界「嘘」ガイド</t>
+          <t>異世界でも無難に生きたい症候群</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>辻島もと(著者)</t>
+          <t>原作：安泰（一二三書房刊） 漫画：笹峰コウ キャラクター原案：ひたきゆう</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>第6話</t>
+          <t>特別編</t>
         </is>
       </c>
     </row>
@@ -69917,17 +70954,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>氷結令嬢さまをフォローしたら、メチャメチャ溺愛されてしまった件@comic</t>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>漫画：ハレノチアメ 原作：愛坂タカト キャラクター原案：Bcoca</t>
+          <t>空野進 sorani ファルまろ</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2巻表紙イラスト公開！</t>
+          <t>第25話　最弱貴族、隠蔽を暴く（３）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add ranking data for 2026-10-26
</commit_message>
<xml_diff>
--- a/ranking_weekly.xlsx
+++ b/ranking_weekly.xlsx
@@ -77,6 +77,7 @@
     <sheet name="2026-10-05" sheetId="69" state="visible" r:id="rId69"/>
     <sheet name="2026-10-12" sheetId="70" state="visible" r:id="rId70"/>
     <sheet name="2026-10-19" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="2026-10-26" sheetId="72" state="visible" r:id="rId72"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -69969,22 +69970,1058 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t>ワンパンマン</t>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>原作/ＯＮＥ 作画/村田雄介</t>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t>238撃目</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>異世界おじさん</t>
+        </is>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>殆ど死んでいる(著者)</t>
+        </is>
+      </c>
+      <c r="D3" s="0" t="inlineStr">
+        <is>
+          <t>コミックス第16巻発売告知</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+        </is>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
+        </is>
+      </c>
+      <c r="D4" s="0" t="inlineStr">
+        <is>
+          <t>第42話：男の覚悟②</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+        </is>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D5" s="0" t="inlineStr">
+        <is>
+          <t>第27話-2「共闘」</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+        </is>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D6" s="0" t="inlineStr">
+        <is>
+          <t>第11話前編：情け無用の討伐戦</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+        </is>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D7" s="0" t="inlineStr">
+        <is>
+          <t>第27話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>光永康則</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="inlineStr">
+        <is>
+          <t>第８２話『決壊停止』②</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="inlineStr">
+        <is>
+          <t>第14話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>第84話 前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>第45話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>マツモトケンゴ</t>
+        </is>
+      </c>
+      <c r="D12" s="0" t="inlineStr">
+        <is>
+          <t>第８９話　肝試しの戦いが始まった（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>クセ強彼女は床にいざなう</t>
+        </is>
+      </c>
+      <c r="C13" s="0" t="inlineStr">
+        <is>
+          <t>須河篤志(著者)</t>
+        </is>
+      </c>
+      <c r="D13" s="0" t="inlineStr">
+        <is>
+          <t>第26話後半</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+        </is>
+      </c>
+      <c r="C14" s="0" t="inlineStr">
+        <is>
+          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D14" s="0" t="inlineStr">
+        <is>
+          <t>第24話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>死亡エンドを回避したギャルゲーのヒロインたちが俺の【日記帳】を読んで秘密を知ったらしい</t>
+        </is>
+      </c>
+      <c r="C15" s="0" t="inlineStr">
+        <is>
+          <t>addict(原作) となりける(作画) へいろー(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D15" s="0" t="inlineStr">
+        <is>
+          <t>第2話</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="inlineStr">
+        <is>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
+        </is>
+      </c>
+      <c r="C16" s="0" t="inlineStr">
+        <is>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+        </is>
+      </c>
+      <c r="D16" s="0" t="inlineStr">
+        <is>
+          <t>第141話　決意してみるⅠ（中編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>六志麻あさ 業務用餅 kisui</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="inlineStr">
+        <is>
+          <t>第９６話</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>実は俺、最強でした？</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="inlineStr">
+        <is>
+          <t>第158話　新王謁見式</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>三部べべ(漫画) ねうしとら(原作)</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>第13話-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>リビルドワールド</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>第86話➁</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>ぽんドロイド！ はまさん</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="inlineStr">
+        <is>
+          <t>はれやまはれぞう(著者)</t>
+        </is>
+      </c>
+      <c r="D21" s="0" t="inlineStr">
+        <is>
+          <t>第27話</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="inlineStr">
+        <is>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D22" s="0" t="inlineStr">
+        <is>
+          <t>第8話①</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+        </is>
+      </c>
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+        </is>
+      </c>
+      <c r="D23" s="0" t="inlineStr">
+        <is>
+          <t>第41話 独身貴族は孤高な馬と駆ける（3）</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+        </is>
+      </c>
+      <c r="D24" s="0" t="inlineStr">
+        <is>
+          <t>第14話 灯り（前編）</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
+        </is>
+      </c>
+      <c r="D25" s="0" t="inlineStr">
+        <is>
+          <t>番外編　お土産ですわ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="inlineStr">
+        <is>
+          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+        </is>
+      </c>
+      <c r="C26" s="0" t="inlineStr">
+        <is>
+          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D26" s="0" t="inlineStr">
+        <is>
+          <t>第19話-2：前へ進んで</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+        </is>
+      </c>
+      <c r="C27" s="0" t="inlineStr">
+        <is>
+          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+        </is>
+      </c>
+      <c r="D27" s="0" t="inlineStr">
+        <is>
+          <t>第55話 破壊の魔剣④</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="inlineStr">
+        <is>
+          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+        </is>
+      </c>
+      <c r="C28" s="0" t="inlineStr">
+        <is>
+          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D28" s="0" t="inlineStr">
+        <is>
+          <t>第14話前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="inlineStr">
+        <is>
+          <t>ギルドの受付嬢リリナさんは俺にだけ冷たい</t>
+        </is>
+      </c>
+      <c r="C29" s="0" t="inlineStr">
+        <is>
+          <t>うたしま(漫画) 近藤玲司(原作)</t>
+        </is>
+      </c>
+      <c r="D29" s="0" t="inlineStr">
+        <is>
+          <t>クエスト2 前編</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="inlineStr">
+        <is>
+          <t>おとなりのダウナーさんは無理させない</t>
+        </is>
+      </c>
+      <c r="C30" s="0" t="inlineStr">
+        <is>
+          <t>瑠璃いろ(著者)</t>
+        </is>
+      </c>
+      <c r="D30" s="0" t="inlineStr">
+        <is>
+          <t>第19話</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="inlineStr">
+        <is>
+          <t>姫様“拷問”の時間です</t>
+        </is>
+      </c>
+      <c r="C31" s="0" t="inlineStr">
+        <is>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+        </is>
+      </c>
+      <c r="D31" s="0" t="inlineStr">
+        <is>
+          <t>拷問205</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="inlineStr">
+        <is>
+          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+        </is>
+      </c>
+      <c r="C32" s="0" t="inlineStr">
+        <is>
+          <t>ヨウハ(著者)</t>
+        </is>
+      </c>
+      <c r="D32" s="0" t="inlineStr">
+        <is>
+          <t>第6話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="inlineStr">
+        <is>
+          <t>魔術師クノンは見えている</t>
+        </is>
+      </c>
+      <c r="C33" s="0" t="inlineStr">
+        <is>
+          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D33" s="0" t="inlineStr">
+        <is>
+          <t>第51話②</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="inlineStr">
+        <is>
+          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+        </is>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D34" s="0" t="inlineStr">
+        <is>
+          <t>第13話-2：王子様です</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="inlineStr">
+        <is>
+          <t>世界最強の魔女、始めました 〜私だけ『攻略サイト』を見れる世界で自由に生きます〜</t>
+        </is>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t>戸賀 環 坂木持丸 riritto</t>
+        </is>
+      </c>
+      <c r="D35" s="0" t="inlineStr">
+        <is>
+          <t>第74話①　こみけを開催してみた</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="inlineStr">
+        <is>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+        </is>
+      </c>
+      <c r="C36" s="0" t="inlineStr">
+        <is>
+          <t>村上よしゆき 茨木野 あるてら</t>
+        </is>
+      </c>
+      <c r="D36" s="0" t="inlineStr">
+        <is>
+          <t>第５１話　勇者、完全に封印されて宇宙の彼方へ捨てられてしまう（４）</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="inlineStr">
+        <is>
+          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+        </is>
+      </c>
+      <c r="C37" s="0" t="inlineStr">
+        <is>
+          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+        </is>
+      </c>
+      <c r="D37" s="0" t="inlineStr">
+        <is>
+          <t>第14話-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="inlineStr">
+        <is>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+        </is>
+      </c>
+      <c r="C38" s="0" t="inlineStr">
+        <is>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+        </is>
+      </c>
+      <c r="D38" s="0" t="inlineStr">
+        <is>
+          <t>第10話(1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="inlineStr">
+        <is>
+          <t>小林さんちのメイドラゴン</t>
+        </is>
+      </c>
+      <c r="C39" s="0" t="inlineStr">
+        <is>
+          <t>クール教信者</t>
+        </is>
+      </c>
+      <c r="D39" s="0" t="inlineStr">
+        <is>
+          <t>第176話</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="inlineStr">
+        <is>
+          <t>よくわからないけれど異世界に転生していたようです</t>
+        </is>
+      </c>
+      <c r="C40" s="0" t="inlineStr">
+        <is>
+          <t>内々けやき あし カオミン</t>
+        </is>
+      </c>
+      <c r="D40" s="0" t="inlineStr">
+        <is>
+          <t>第163話 よくわからないけれど荒波を乗り越えたみたいです（１）</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="inlineStr">
+        <is>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
+        </is>
+      </c>
+      <c r="C41" s="0" t="inlineStr">
+        <is>
+          <t>如意自在(著者)</t>
+        </is>
+      </c>
+      <c r="D41" s="0" t="inlineStr">
+        <is>
+          <t>番外編2</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="inlineStr">
+        <is>
+          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
+        </is>
+      </c>
+      <c r="C42" s="0" t="inlineStr">
+        <is>
+          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
+        </is>
+      </c>
+      <c r="D42" s="0" t="inlineStr">
+        <is>
+          <t>第４話　ゴーレム任せで開拓します！（３）</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="inlineStr">
+        <is>
+          <t>サーシャちゃんとクラスメイトオタクくん</t>
+        </is>
+      </c>
+      <c r="C43" s="0" t="inlineStr">
+        <is>
+          <t>はぐはぐ(著者)</t>
+        </is>
+      </c>
+      <c r="D43" s="0" t="inlineStr">
+        <is>
+          <t>第104話</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="inlineStr">
+        <is>
+          <t>雨森潤奈は湿度が高い</t>
+        </is>
+      </c>
+      <c r="C44" s="0" t="inlineStr">
+        <is>
+          <t>水城水城(原作) 稲鳴四季(作画) 潮崎しの(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D44" s="0" t="inlineStr">
+        <is>
+          <t>第5話</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t>描けないのでヤってみた</t>
+        </is>
+      </c>
+      <c r="C45" s="0" t="inlineStr">
+        <is>
+          <t>逢上おかき(著者)</t>
+        </is>
+      </c>
+      <c r="D45" s="0" t="inlineStr">
+        <is>
+          <t>連載開始告知</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="inlineStr">
+        <is>
+          <t>おせっかい女子、恋をする</t>
+        </is>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>音竹 ひかる(著者)</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>第37話</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="inlineStr">
+        <is>
+          <t>女子高生の無駄づかい</t>
+        </is>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>ビーノ(著者)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>第150話　じゅんばん</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="inlineStr">
+        <is>
+          <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
+        </is>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>昼行燈（原作） しいたけ元帥（漫画）</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>第53話（前半）</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="inlineStr">
+        <is>
+          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
+        </is>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>第12話②「球技大会！」</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="0" t="inlineStr">
+        <is>
+          <t>異世界でも無難に生きたい症候群</t>
+        </is>
+      </c>
+      <c r="C50" s="0" t="inlineStr">
+        <is>
+          <t>原作：安泰（一二三書房刊） 漫画：笹峰コウ キャラクター原案：ひたきゆう</t>
+        </is>
+      </c>
+      <c r="D50" s="0" t="inlineStr">
+        <is>
+          <t>特別編</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="0" t="inlineStr">
+        <is>
+          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+        </is>
+      </c>
+      <c r="C51" s="0" t="inlineStr">
+        <is>
+          <t>空野進 sorani ファルまろ</t>
+        </is>
+      </c>
+      <c r="D51" s="0" t="inlineStr">
+        <is>
+          <t>第25話　最弱貴族、隠蔽を暴く（３）</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>author</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>latest_episode</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
       <c r="A2" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ワンパンマン</t>
+          <t>異世界おじさん</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>原作/ＯＮＥ 作画/村田雄介</t>
+          <t>殆ど死んでいる(著者)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>238撃目</t>
+          <t>第81話</t>
         </is>
       </c>
     </row>
@@ -69994,17 +71031,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>異世界おじさん</t>
+          <t>異種族レビュアーズ</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>殆ど死んでいる(著者)</t>
+          <t>天原(原作) masha(作画)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>コミックス第16巻発売告知</t>
+          <t>第95話</t>
         </is>
       </c>
     </row>
@@ -70014,17 +71051,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
+          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>zunta(作画) はらわたさいぞう(原作)</t>
+          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>第42話：男の覚悟②</t>
+          <t>第84話 前編</t>
         </is>
       </c>
     </row>
@@ -70034,17 +71071,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>悪人面したＢ級冒険者 主人公とその幼馴染たちのパパになる</t>
+          <t>転生コロシアム～最弱スキルで最強の女たちを攻略して奴隷ハーレム作ります～</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>こげめ(著者) えんじ(原作) ハラカズヒロ(キャラクター原案)</t>
+          <t>zunta(作画) はらわたさいぞう(原作)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>第27話-2「共闘」</t>
+          <t>第42話：男の覚悟③</t>
         </is>
       </c>
     </row>
@@ -70054,17 +71091,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>全滅エンドを死に物狂いで回避した。パーティが病んだ。</t>
+          <t>生徒会にも穴はある！</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>縞(漫画) 雨糸雀(原作) kodamazon(キャラクター原案)</t>
+          <t>むちまろ</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>第11話前編：情け無用の討伐戦</t>
+          <t>第163話	おしくら★ウィンター♪</t>
         </is>
       </c>
     </row>
@@ -70074,17 +71111,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>怠惰な悪辱貴族に転生した俺、シナリオをぶっ壊したら規格外の魔力で最凶になった</t>
+          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>菊池快晴(原作) 小田童馬(作画) 桑島黎音(キャラクター原案)</t>
+          <t>光永康則</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>第27話後半</t>
+          <t>第８２話『決壊停止』③</t>
         </is>
       </c>
     </row>
@@ -70094,17 +71131,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>時間停止勇者―余命３日の設定じゃ世界を救うには短すぎる―</t>
+          <t>勇者パーティーをクビになったので故郷に帰ったら、メンバー全員がついてきたんだが</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>光永康則</t>
+          <t>絶叫あいす。(漫画) 木の芽(原作) 希(キャラクター原案)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>第８２話『決壊停止』②</t>
+          <t>第12話 前編</t>
         </is>
       </c>
     </row>
@@ -70114,17 +71151,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>貞操逆転世界で頼めばヤれると噂の俺</t>
+          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>澄田佑貴(漫画) aaa168（スリーエー）(原作)</t>
+          <t>マツモトケンゴ</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>第14話後半</t>
+          <t>第８９話　肝試しの戦いが始まった（２）</t>
         </is>
       </c>
     </row>
@@ -70134,17 +71171,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>新米オッサン冒険者、最強パーティに死ぬほど鍛えられて無敵になる</t>
+          <t>元・世界１位のサブキャラ育成日記 ～廃プレイヤー、異世界を攻略中！～</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>漫画：荻野ケン 原作：岸馬きらく キャラクター原案：Tea</t>
+          <t>沢村治太郎(原作) 前田理想(漫画) まろ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>第84話 前編</t>
+          <t>第91話その2</t>
         </is>
       </c>
     </row>
@@ -70154,17 +71191,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>クラスで２番目に可愛い女の子と友だちになった</t>
+          <t>お前がヤったんだろ！</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>尾野凛(漫画) たかた(原作) 日向あずり(キャラクター原案)</t>
+          <t>クシザキ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>第45話②</t>
+          <t>第22話	湯煙の合宿　後編</t>
         </is>
       </c>
     </row>
@@ -70174,17 +71211,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>地元のいじめっ子達に仕返ししようとしたら、別の戦いが始まった。</t>
+          <t>異世界のんびり農家</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>マツモトケンゴ</t>
+          <t>剣康之(作画) 内藤騎之介(原作) やすも(キャラクター原案)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>第８９話　肝試しの戦いが始まった（１）</t>
+          <t>第336話</t>
         </is>
       </c>
     </row>
@@ -70194,17 +71231,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>クセ強彼女は床にいざなう</t>
+          <t>異世界魔王と召喚少女の奴隷魔術</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>須河篤志(著者)</t>
+          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>第26話後半</t>
+          <t>第141話　決意してみるⅠ（後編）</t>
         </is>
       </c>
     </row>
@@ -70214,17 +71251,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>男女比1：5の世界でも普通に生きられると思った？　～激重感情な彼女たちが無自覚男子に翻弄されたら～</t>
+          <t>バキ外伝 烈海王は異世界転生しても一向にかまわんッッ</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>三藤 孝太郎(原作) 桃季憂(漫画) jimmy(キャラクター原案)</t>
+          <t>板垣恵介 猪原賽 陸井栄史</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>第24話-1</t>
+          <t>第106話　再会</t>
         </is>
       </c>
     </row>
@@ -70234,17 +71271,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>死亡エンドを回避したギャルゲーのヒロインたちが俺の【日記帳】を読んで秘密を知ったらしい</t>
+          <t>ダークサモナーとデキている</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>addict(原作) となりける(作画) へいろー(キャラクター原案)</t>
+          <t>車王(著者)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>第2話</t>
+          <t>第99話</t>
         </is>
       </c>
     </row>
@@ -70254,17 +71291,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>異世界魔王と召喚少女の奴隷魔術</t>
+          <t>リビルドワールド</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>原作：むらさきゆきや 漫画：福田直叶 キャラクター原案：鶴崎貴大</t>
+          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>第141話　決意してみるⅠ（中編）</t>
+          <t>第86話③</t>
         </is>
       </c>
     </row>
@@ -70274,17 +71311,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>追放されたチート付与魔術師は気ままなセカンドライフを謳歌する。</t>
+          <t>実は俺、最強でした？</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>六志麻あさ 業務用餅 kisui</t>
+          <t>原作：澄守 彩 漫画：高橋 愛</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>第９６話</t>
+          <t>第159話　魔物討伐の依頼・前編</t>
         </is>
       </c>
     </row>
@@ -70294,17 +71331,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>実は俺、最強でした？</t>
+          <t>お姉さん派の俺がなぜちっちゃい君を好きになったのか？</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>原作：澄守 彩 漫画：高橋 愛</t>
+          <t>三ツ谷亮(漫画) うらのりつ(構成) 鏡遊(原作) 富士やま(キャラクター原案)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>第158話　新王謁見式</t>
+          <t>第2話②</t>
         </is>
       </c>
     </row>
@@ -70314,17 +71351,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ゲーム世界で魔物に転生してしまった俺、前世で推しだったヒロインを拾ってしまう</t>
+          <t>異世界メイドの三ツ星グルメ ～現代ごはん作ったら王宮で大バズリしました～</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>三部べべ(漫画) ねうしとら(原作)</t>
+          <t>モリタ Ｕ４ nima</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>第13話-2</t>
+          <t>第18話（３）　メイド大集結でお祝い！結婚披露宴（３）</t>
         </is>
       </c>
     </row>
@@ -70334,17 +71371,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>リビルドワールド</t>
+          <t>せっかく農家に転生したので勇者は目指しません</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>綾村切人(漫画) ナフセ(原作) 吟(キャラクターデザイン) わいっしゅ(世界観デザイン) cell(メカニックデザイン)</t>
+          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>第86話➁</t>
+          <t>第8話②</t>
         </is>
       </c>
     </row>
@@ -70354,17 +71391,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ぽんドロイド！ はまさん</t>
+          <t>転生貴族の異世界冒険録 ～自重を知らない神々の使徒～</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>はれやまはれぞう(著者)</t>
+          <t>夜州 nini 藻</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>第27話</t>
+          <t>第77話（前編）</t>
         </is>
       </c>
     </row>
@@ -70374,17 +71411,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>せっかく農家に転生したので勇者は目指しません</t>
+          <t>Ｓ級ギルドを追放されたけど、実は俺だけドラゴンの言葉がわかるので、気付いたときには竜騎士の頂点を極めてました。</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>マツオカヨシノリ(漫画) 月見里嘉助(原作) ゆーにっと(キャラクター原案)</t>
+          <t>ひそな(漫画) 三木なずな(原作) 白狼(キャラクター原案)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>第8話①</t>
+          <t>第49話-2</t>
         </is>
       </c>
     </row>
@@ -70394,17 +71431,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
+          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
+          <t>島知宏 音速炒飯 有都あらゆる</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>第41話 独身貴族は孤高な馬と駆ける（3）</t>
+          <t>番外編　お土産ですわ！</t>
         </is>
       </c>
     </row>
@@ -70414,17 +71451,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>仲間を守って死んだら二十年後の同じ世界に生まれ変わった件……でも俺、転生二回目なんだけど？</t>
+          <t>美人女上司滝沢さん</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>みょん（原作） 樋野友行（漫画） ひやしみらの（キャラクター原案）</t>
+          <t>やんBARU(著者)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>第14話 灯り（前編）</t>
+          <t>第227話</t>
         </is>
       </c>
     </row>
@@ -70434,17 +71471,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>【パクパクですわ】追放されたお嬢様の『モンスターを食べるほど強くなる』スキルは、１食で１レベルアップする前代未聞の最強スキルでした。３日で人類最強になりましたわ～！</t>
+          <t>独身貴族は異世界を謳歌する ～結婚しない男の優雅なおひとりさまライフ～</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>島知宏 音速炒飯 有都あらゆる</t>
+          <t>漫画：駒鳥 ひわ 原作：錬金王 キャラクター原案：三登 いつき</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>番外編　お土産ですわ！</t>
+          <t>第41話 独身貴族は孤高な馬と駆ける（4）</t>
         </is>
       </c>
     </row>
@@ -70454,17 +71491,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>願ってもない追放後からのスローライフ？ 〜引退したはずが成り行きで美少女ギャルの師匠になったらなぜかめちゃくちゃ懐かれた〜</t>
+          <t>バキ外伝　ガイアとシコルスキー　～ときどきノムラ 二人だけど三人暮らし～</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ヤミーゴ(漫画) シュガースプーン。（GA文庫/SBクリエイティブ）(原作) なたーしゃ(キャラクター原案)</t>
+          <t>板垣恵介 林たかあき</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>第19話-2：前へ進んで</t>
+          <t>第80話 退屈しのぎ</t>
         </is>
       </c>
     </row>
@@ -70474,17 +71511,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>魔導具師ダリヤはうつむかない ～Dahliya Wilts No More～</t>
+          <t>「ククク……。奴は四天王の中でも最弱」と解雇された俺、なぜか勇者と聖女の師匠になる</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>漫画：住川惠 原作：甘岸久弥(｢魔導具師ダリヤはうつむかない ～今日から自由な職人ライフ～｣MFブックス刊) キャラクター原案：景、駒田ハチ</t>
+          <t>漫画：芳橋アツシ 原作：延野正行 キャラクター原案：坂野杏梨</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>第55話 破壊の魔剣④</t>
+          <t>第52話　奴はキレる（前編）</t>
         </is>
       </c>
     </row>
@@ -70494,17 +71531,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>配信に致命的に向いていない女の子が迷宮で黙々と人助けする配信</t>
+          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>下田将也(漫画) 佐藤悪糖(原作) 福きつね(キャラクター原案)</t>
+          <t>村上よしゆき 茨木野 あるてら</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>第14話前編</t>
+          <t>第５１話　勇者、完全に封印されて宇宙の彼方へ捨てられてしまう（５）</t>
         </is>
       </c>
     </row>
@@ -70514,17 +71551,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ギルドの受付嬢リリナさんは俺にだけ冷たい</t>
+          <t>インフィニット・デンドログラム</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>うたしま(漫画) 近藤玲司(原作)</t>
+          <t>今井神 原作：海道左近 キャラクター原案：タイキ</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>クエスト2 前編</t>
+          <t>第82話</t>
         </is>
       </c>
     </row>
@@ -70534,17 +71571,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>おとなりのダウナーさんは無理させない</t>
+          <t>何の取り柄もない平凡な俺が美人双子姉妹を命懸けで助けた結果、実はヤンデレだった二人をガチ惚れさせてしまった件</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>瑠璃いろ(著者)</t>
+          <t>原作：水島紗鳥 漫画：megumi キャラクター原案：にわ田</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>第19話</t>
+          <t>第4話</t>
         </is>
       </c>
     </row>
@@ -70554,17 +71591,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>姫様“拷問”の時間です</t>
+          <t>女友達は頼めば意外とヤらせてくれる</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>原作:春原ロビンソン　漫画:ひらけい</t>
+          <t>ろくろ(漫画) 鏡遊(原作)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>拷問205</t>
+          <t>第36話①</t>
         </is>
       </c>
     </row>
@@ -70574,17 +71611,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>イケメンお姉さんはそーゆー目で見られたい</t>
+          <t>骸骨騎士様、只今異世界へお出掛け中</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ヨウハ(著者)</t>
+          <t>サワノアキラ（漫画） 秤猿鬼（原作） KeG（キャラクター原案）</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>第6話-1</t>
+          <t>第70章　開戦Ⅰ</t>
         </is>
       </c>
     </row>
@@ -70594,17 +71631,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>魔術師クノンは見えている</t>
+          <t>衛宮さんちの今日のごはん</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>La-na(作画) 南野海風(原作) Ｌａｒｕｈａ(キャラクター原案)</t>
+          <t>TAa(漫画) 只野まこと(料理監修) ＴＹＰＥ－ＭＯＯＮ(原作)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>第51話②</t>
+          <t>第81話</t>
         </is>
       </c>
     </row>
@@ -70614,17 +71651,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>モブ司祭だけど、この世界が乙女ゲームだと気づいたのでヒロインを育成します</t>
+          <t>回復術士のやり直し</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>井冬良(漫画) レオナールＤ(原作) りいちゅ(キャラクター原案)</t>
+          <t>月夜涙(原作) 羽賀ソウケン(漫画) しおこんぶ(キャラクター原案)</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>第13話-2：王子様です</t>
+          <t>第81話-2</t>
         </is>
       </c>
     </row>
@@ -70644,7 +71681,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>第74話①　こみけを開催してみた</t>
+          <t>第74話②　こみけを開催してみた</t>
         </is>
       </c>
     </row>
@@ -70654,17 +71691,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>落ちこぼれだった兄が実は最強 ～史上最強の勇者は転生し、学園で無自覚に無双する～</t>
+          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>村上よしゆき 茨木野 あるてら</t>
+          <t>如意自在(著者)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>第５１話　勇者、完全に封印されて宇宙の彼方へ捨てられてしまう（４）</t>
+          <t>第8話前半</t>
         </is>
       </c>
     </row>
@@ -70674,17 +71711,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>乙女ゲー世界はモブに厳しい世界です【共和国編】</t>
+          <t>くらいあの子としたいこと</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>三嶋与夢(原作) 行々狸(作画) 孟達(キャラクター原案) マツリセイシロウ(構成) FTops(制作)</t>
+          <t>碇マナツ(著者)</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>第14話-1</t>
+          <t>第106話</t>
         </is>
       </c>
     </row>
@@ -70694,17 +71731,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
+          <t>三枝さんはメガネ先輩と恋を描く</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
+          <t>セレビィ量産型(著者)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>第10話(1)</t>
+          <t>第30話後半</t>
         </is>
       </c>
     </row>
@@ -70714,17 +71751,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>小林さんちのメイドラゴン</t>
+          <t>姫様“拷問”の時間です</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>クール教信者</t>
+          <t>原作:春原ロビンソン　漫画:ひらけい</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>第176話</t>
+          <t>拷問206</t>
         </is>
       </c>
     </row>
@@ -70744,7 +71781,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>第163話 よくわからないけれど荒波を乗り越えたみたいです（１）</t>
+          <t>第163話 よくわからないけれど荒波を乗り越えたみたいです（２）</t>
         </is>
       </c>
     </row>
@@ -70754,17 +71791,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>新婚だけどキャプテンの彼女とはまだヤれない</t>
+          <t>俺の幼馴染がデッッッッかくなりすぎた</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>如意自在(著者)</t>
+          <t>ヨシカ(漫画) 折口良乃(原作) ろうか(キャラクター原案)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>番外編2</t>
+          <t>第5話-2</t>
         </is>
       </c>
     </row>
@@ -70774,17 +71811,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
+          <t>回復魔法を極めたらぶっ壊れ性能になった。妾の子と迫害されるので実家に頼らず生きていく！（コミック）</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
+          <t>漫画／にゃ藻 原作／年中麦茶太郎 キャラクター原案／YeoNwa</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>第４話　ゴーレム任せで開拓します！（３）</t>
+          <t>第10話(2)</t>
         </is>
       </c>
     </row>
@@ -70794,17 +71831,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>サーシャちゃんとクラスメイトオタクくん</t>
+          <t>異世界のすみっこで快適ものづくり生活 ～女神さまのくれた工房はちょっとやりすぎ性能だった～</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>はぐはぐ(著者)</t>
+          <t>西山アラタ(漫画) 長田信織(原作) 東上文(キャラクター原案)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>第104話</t>
+          <t>EP.30①</t>
         </is>
       </c>
     </row>
@@ -70814,17 +71851,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>雨森潤奈は湿度が高い</t>
+          <t>異世界「嘘」ガイド</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>水城水城(原作) 稲鳴四季(作画) 潮崎しの(キャラクター原案)</t>
+          <t>辻島もと(著者)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>第5話</t>
+          <t>第7話</t>
         </is>
       </c>
     </row>
@@ -70844,7 +71881,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>連載開始告知</t>
+          <t>第5話前半</t>
         </is>
       </c>
     </row>
@@ -70854,17 +71891,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>おせっかい女子、恋をする</t>
+          <t>十年目、帰還を諦めた転移者はいまさら主人公になる</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>音竹 ひかる(著者)</t>
+          <t>原作：氷純（「十年目、帰還を諦めた転移者はいまさら主人公になる」MFブックス刊） 漫画：しゅーかま キャラクター原案：あんべよしろう</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>第37話</t>
+          <t>第26話②</t>
         </is>
       </c>
     </row>
@@ -70874,17 +71911,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>女子高生の無駄づかい</t>
+          <t>ふかふかダンジョン攻略記～俺の異世界転生冒険譚～</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ビーノ(著者)</t>
+          <t>KAKERU</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>第150話　じゅんばん</t>
+          <t>第81話「チャリオット（危）」（後半）</t>
         </is>
       </c>
     </row>
@@ -70894,17 +71931,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ゲーム悪役貴族に転生した俺は、チート筋肉で無双する</t>
+          <t>領地のすべてをゴーレムで自動化した俺、サボっていると言われて追放されたので魔境をチート技術で開拓します！</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>昼行燈（原作） しいたけ元帥（漫画）</t>
+          <t>kimimaro シシキすず 吉田屋敷 詰め木</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>第53話（前半）</t>
+          <t>第５話　お風呂入って開拓します！（１）</t>
         </is>
       </c>
     </row>
@@ -70914,17 +71951,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>彼女にしたい女子一位、の隣で見つけたあまりちゃん</t>
+          <t>バーサス</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>寝巻ネルゾ(漫画) 裕時悠示(原作) たん旦(キャラクター原案)</t>
+          <t>原作：ONE 漫画：あずま京太郎 構成：bose</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>第12話②「球技大会！」</t>
+          <t>第37話　恐怖の必要性（前編-2）</t>
         </is>
       </c>
     </row>
@@ -70934,17 +71971,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>異世界でも無難に生きたい症候群</t>
+          <t>北斗の拳 世紀末ドラマ撮影伝</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>原作：安泰（一二三書房刊） 漫画：笹峰コウ キャラクター原案：ひたきゆう</t>
+          <t>原案/武論尊・原哲夫 漫画/倉尾宏</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>特別編</t>
+          <t>第91話 雨月リュウガ、飛び立つ!!</t>
         </is>
       </c>
     </row>
@@ -70954,17 +71991,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>最弱貴族に転生したので悪役たちを集めてみた</t>
+          <t>老後に備えて異世界で８万枚の金貨を貯めます</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>空野進 sorani ファルまろ</t>
+          <t>FUNA 東西 モトエ恵介</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>第25話　最弱貴族、隠蔽を暴く（３）</t>
+          <t>第135話 攻撃反射作戦［その②］</t>
         </is>
       </c>
     </row>

</xml_diff>